<commit_message>
Update dashboard/data (2026-07-14 11:14)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89825AA-5E33-4460-8FBE-7FC2C745075D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB89A13-8B60-478F-BAD3-06683222C7A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -1882,7 +1882,7 @@
       <c r="E23" s="41"/>
       <c r="F23" s="41"/>
       <c r="G23" s="42">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H23" s="40" t="s">
         <v>22</v>
@@ -1907,7 +1907,7 @@
       <c r="E24" s="38"/>
       <c r="F24" s="38"/>
       <c r="G24" s="39">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="H24" s="37" t="s">
         <v>22</v>
@@ -3013,7 +3013,7 @@
         <v>70</v>
       </c>
       <c r="D14" s="22">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E14" s="17">
         <v>1707089</v>
@@ -5395,6 +5395,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5647,29 +5669,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5686,23 +5705,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-17 15:20)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB89A13-8B60-478F-BAD3-06683222C7A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FAE77B-CAFF-4E48-B1AA-92AECADB3EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -236,21 +236,12 @@
     <t>วริษฐ์ ยุวโชติพันธุ์</t>
   </si>
   <si>
-    <t>รอลูกค้าคอนเฟิมวันส่งงาน Frist fix</t>
-  </si>
-  <si>
-    <t>ส่งงาน Frist fix 07/13/2026</t>
-  </si>
-  <si>
     <t>1 กันยา เริ่มเข้าไซต์</t>
   </si>
   <si>
     <t>โครงการล่าช้า เดือน 9 ส่งมอบงาน</t>
   </si>
   <si>
-    <t>โครงการล่าช้า/ติดกริลวันที่ 17/07/2026 กำหนดส่งงานได้ กันยา-ตุลา</t>
-  </si>
-  <si>
     <t>Project Type</t>
   </si>
   <si>
@@ -356,9 +347,6 @@
     <t>The Grand Pinkao</t>
   </si>
   <si>
-    <t>บริษัท NAME 7 AIR</t>
-  </si>
-  <si>
     <t>รอสรุปแผนงานหลังจากสำรวจหน้างาน</t>
   </si>
   <si>
@@ -432,6 +420,18 @@
   </si>
   <si>
     <t>Site Meenting</t>
+  </si>
+  <si>
+    <t>รอลูกค้าแจ้งการแก้ไขเรื่องไฟฟ้าไม่สามารถ ออนไฟได้ งวดสุดท้าย</t>
+  </si>
+  <si>
+    <t>โครงการล่าช้า/ติดกริลวันที่ 24-27 /07 Pretest 30/07/2026 ส่งงานงวดสุดท้าย เดือนตุลา</t>
+  </si>
+  <si>
+    <t>ส่งงาน Frist Fix เสร็จแล้ว รอเดือนตุลาเข้าดำเนินงาน Second Fix</t>
+  </si>
+  <si>
+    <t>รองานโครงสร้าง เข้าได้ ปลายเดือน 8</t>
   </si>
 </sst>
 </file>
@@ -922,29 +922,29 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1355,31 +1355,31 @@
       <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1395,10 +1395,10 @@
         <v>5</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>6</v>
@@ -1410,14 +1410,14 @@
         <v>8</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="67" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1437,14 +1437,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="66">
+      <c r="I5" s="61">
         <v>46213</v>
       </c>
-      <c r="J5" s="66"/>
+      <c r="J5" s="61"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="61"/>
+      <c r="A6" s="64"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1462,12 +1462,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="61"/>
-      <c r="J6" s="67"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="60"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="60" t="s">
+      <c r="A7" s="63" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1487,14 +1487,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="62" t="s">
+      <c r="I7" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="62"/>
+      <c r="J7" s="59"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="61"/>
+      <c r="A8" s="64"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1512,12 +1512,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="61"/>
-      <c r="J8" s="67"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="60"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="60" t="s">
+      <c r="A9" s="63" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1537,14 +1537,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="59">
         <v>46218</v>
       </c>
-      <c r="J9" s="62"/>
+      <c r="J9" s="59"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="61"/>
+      <c r="A10" s="64"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1562,12 +1562,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="61"/>
-      <c r="J10" s="67"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="60"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="60" t="s">
+      <c r="A11" s="63" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1587,14 +1587,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="62">
+      <c r="I11" s="59">
         <v>46171</v>
       </c>
-      <c r="J11" s="62"/>
+      <c r="J11" s="59"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="61"/>
+      <c r="A12" s="64"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1612,12 +1612,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="61"/>
-      <c r="J12" s="67"/>
+      <c r="I12" s="64"/>
+      <c r="J12" s="60"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="60" t="s">
+      <c r="A13" s="63" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1637,14 +1637,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="62" t="s">
+      <c r="I13" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="62"/>
+      <c r="J13" s="59"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="61"/>
+      <c r="A14" s="64"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1662,12 +1662,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="61"/>
-      <c r="J14" s="67"/>
+      <c r="I14" s="64"/>
+      <c r="J14" s="60"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="60" t="s">
+      <c r="A15" s="63" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1687,14 +1687,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="62">
+      <c r="I15" s="59">
         <v>46199</v>
       </c>
-      <c r="J15" s="62"/>
+      <c r="J15" s="59"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="61"/>
+      <c r="A16" s="64"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1712,12 +1712,12 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="61"/>
-      <c r="J16" s="67"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="60"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="64" t="s">
+      <c r="A17" s="65" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="34" t="s">
@@ -1737,14 +1737,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="63">
+      <c r="I17" s="62">
         <v>46305</v>
       </c>
-      <c r="J17" s="63"/>
+      <c r="J17" s="62"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="61"/>
+      <c r="A18" s="64"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1762,12 +1762,12 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="61"/>
-      <c r="J18" s="67"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="60"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="64" t="s">
+      <c r="A19" s="65" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="34" t="s">
@@ -1787,14 +1787,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="63">
+      <c r="I19" s="62">
         <v>46336</v>
       </c>
-      <c r="J19" s="63"/>
+      <c r="J19" s="62"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="61"/>
+      <c r="A20" s="64"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1812,12 +1812,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="61"/>
-      <c r="J20" s="67"/>
+      <c r="I20" s="64"/>
+      <c r="J20" s="60"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="60" t="s">
+      <c r="A21" s="63" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1837,14 +1837,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="62">
+      <c r="I21" s="59">
         <v>46336</v>
       </c>
-      <c r="J21" s="62"/>
+      <c r="J21" s="59"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="61"/>
+      <c r="A22" s="64"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1862,62 +1862,62 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="61"/>
-      <c r="J22" s="67"/>
+      <c r="I22" s="64"/>
+      <c r="J22" s="60"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="60" t="s">
+      <c r="A23" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="41">
+      <c r="C23" s="44">
         <v>46190</v>
       </c>
-      <c r="D23" s="41">
+      <c r="D23" s="44">
         <v>46206</v>
       </c>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="42">
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="45">
         <v>1</v>
       </c>
-      <c r="H23" s="40" t="s">
+      <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="62">
-        <v>46218</v>
-      </c>
-      <c r="J23" s="62"/>
+      <c r="I23" s="59">
+        <v>46220</v>
+      </c>
+      <c r="J23" s="59"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="61"/>
-      <c r="B24" s="37" t="s">
+      <c r="A24" s="64"/>
+      <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="38">
-        <v>46209</v>
-      </c>
-      <c r="D24" s="38">
-        <v>46211</v>
-      </c>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="39">
-        <v>0.2</v>
-      </c>
-      <c r="H24" s="37" t="s">
+      <c r="C24" s="47">
+        <v>46216</v>
+      </c>
+      <c r="D24" s="47">
+        <v>46220</v>
+      </c>
+      <c r="E24" s="47"/>
+      <c r="F24" s="47"/>
+      <c r="G24" s="48">
+        <v>1</v>
+      </c>
+      <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="61"/>
-      <c r="J24" s="67"/>
+      <c r="I24" s="64"/>
+      <c r="J24" s="60"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="60" t="s">
+      <c r="A25" s="63" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1937,14 +1937,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="62">
+      <c r="I25" s="59">
         <v>46188</v>
       </c>
-      <c r="J25" s="62"/>
+      <c r="J25" s="59"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="61"/>
+      <c r="A26" s="64"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1962,12 +1962,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="61"/>
-      <c r="J26" s="67"/>
+      <c r="I26" s="64"/>
+      <c r="J26" s="60"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="60" t="s">
+      <c r="A27" s="63" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -1987,14 +1987,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="62">
+      <c r="I27" s="59">
         <v>46321</v>
       </c>
-      <c r="J27" s="62"/>
+      <c r="J27" s="59"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="61"/>
+      <c r="A28" s="64"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2012,12 +2012,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="61"/>
-      <c r="J28" s="67"/>
+      <c r="I28" s="64"/>
+      <c r="J28" s="60"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="60" t="s">
+      <c r="A29" s="63" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2037,14 +2037,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="62">
+      <c r="I29" s="59">
         <v>46139</v>
       </c>
-      <c r="J29" s="62"/>
+      <c r="J29" s="59"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="61"/>
+      <c r="A30" s="64"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2062,12 +2062,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="61"/>
-      <c r="J30" s="67"/>
+      <c r="I30" s="64"/>
+      <c r="J30" s="60"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="60" t="s">
+      <c r="A31" s="63" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2087,14 +2087,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="62">
+      <c r="I31" s="59">
         <v>46133</v>
       </c>
-      <c r="J31" s="62"/>
+      <c r="J31" s="59"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="61"/>
+      <c r="A32" s="64"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2112,12 +2112,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="61"/>
-      <c r="J32" s="67"/>
+      <c r="I32" s="64"/>
+      <c r="J32" s="60"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="60" t="s">
+      <c r="A33" s="63" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2137,14 +2137,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="62">
+      <c r="I33" s="59">
         <v>46295</v>
       </c>
-      <c r="J33" s="62"/>
+      <c r="J33" s="59"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="61"/>
+      <c r="A34" s="64"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2162,12 +2162,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="61"/>
-      <c r="J34" s="67"/>
+      <c r="I34" s="64"/>
+      <c r="J34" s="60"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="60" t="s">
+      <c r="A35" s="63" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2187,14 +2187,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="62">
+      <c r="I35" s="59">
         <v>45737</v>
       </c>
-      <c r="J35" s="62"/>
+      <c r="J35" s="59"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="61"/>
+      <c r="A36" s="64"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2212,12 +2212,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="61"/>
-      <c r="J36" s="67"/>
+      <c r="I36" s="64"/>
+      <c r="J36" s="60"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="60" t="s">
+      <c r="A37" s="63" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2237,14 +2237,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="62">
+      <c r="I37" s="59">
         <v>45737</v>
       </c>
-      <c r="J37" s="62"/>
+      <c r="J37" s="59"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="61"/>
+      <c r="A38" s="64"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2262,26 +2262,35 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="61"/>
-      <c r="J38" s="67"/>
+      <c r="I38" s="64"/>
+      <c r="J38" s="60"/>
       <c r="K38" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2298,29 +2307,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2382,30 +2382,30 @@
       <c r="V1" s="57"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="59"/>
-      <c r="R2" s="59"/>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="U2" s="59"/>
-      <c r="V2" s="59"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+      <c r="Q2" s="58"/>
+      <c r="R2" s="58"/>
+      <c r="S2" s="58"/>
+      <c r="T2" s="58"/>
+      <c r="U2" s="58"/>
+      <c r="V2" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -2415,7 +2415,7 @@
         <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>35</v>
@@ -2469,10 +2469,10 @@
         <v>9</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:22" s="10" customFormat="1" ht="18.600000000000001">
@@ -2483,7 +2483,7 @@
         <v>22</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D5" s="16">
         <v>0.9</v>
@@ -2497,8 +2497,8 @@
       </c>
       <c r="G5" s="17"/>
       <c r="H5" s="17">
-        <f>E5*0.8</f>
-        <v>261429.08799999999</v>
+        <f>E5*0.9</f>
+        <v>294107.72399999999</v>
       </c>
       <c r="I5" s="18">
         <v>12</v>
@@ -2530,7 +2530,7 @@
         <v>50</v>
       </c>
       <c r="U5" s="30" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="V5" s="20"/>
     </row>
@@ -2542,7 +2542,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D6" s="16">
         <v>0</v>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="S6" s="15"/>
       <c r="T6" s="27" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="U6" s="27"/>
       <c r="V6" s="20"/>
@@ -2596,13 +2596,13 @@
         <v>17</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D7" s="16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E7" s="17">
         <v>576317.9</v>
@@ -2615,8 +2615,8 @@
         <v>603</v>
       </c>
       <c r="H7" s="17">
-        <f>E7*0.9</f>
-        <v>518686.11000000004</v>
+        <f>E7*1</f>
+        <v>576317.9</v>
       </c>
       <c r="I7" s="18">
         <v>20</v>
@@ -2648,7 +2648,7 @@
         <v>52</v>
       </c>
       <c r="U7" s="30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="V7" s="20"/>
     </row>
@@ -2660,7 +2660,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D8" s="16">
         <v>1</v>
@@ -2707,7 +2707,7 @@
       <c r="S8" s="15"/>
       <c r="T8" s="27"/>
       <c r="U8" s="32" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="V8" s="20">
         <v>46134</v>
@@ -2721,7 +2721,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D9" s="16">
         <v>0</v>
@@ -2771,7 +2771,7 @@
         <v>12</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D10" s="16">
         <v>1</v>
@@ -2818,7 +2818,7 @@
       <c r="S10" s="15"/>
       <c r="T10" s="28"/>
       <c r="U10" s="32" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="V10" s="20">
         <v>46141</v>
@@ -2832,7 +2832,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D11" s="16">
         <v>0.7</v>
@@ -2841,15 +2841,15 @@
         <v>1156111.18</v>
       </c>
       <c r="F11" s="17">
-        <f>P11*0.3</f>
-        <v>84000</v>
+        <f>P11*0.5</f>
+        <v>140000</v>
       </c>
       <c r="G11" s="17">
         <v>840</v>
       </c>
       <c r="H11" s="17">
-        <f t="shared" si="0"/>
-        <v>462444.47200000001</v>
+        <f>E11*0.7</f>
+        <v>809277.82599999988</v>
       </c>
       <c r="I11" s="18">
         <v>10</v>
@@ -2877,10 +2877,10 @@
       </c>
       <c r="S11" s="15"/>
       <c r="T11" s="28" t="s">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="U11" s="32" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="V11" s="20">
         <v>46147</v>
@@ -2894,7 +2894,7 @@
         <v>15</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D12" s="16">
         <v>0</v>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="S12" s="15"/>
       <c r="T12" s="28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="U12" s="27"/>
       <c r="V12" s="20">
@@ -2953,7 +2953,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D13" s="16">
         <v>0</v>
@@ -2993,10 +2993,10 @@
         <v>46336</v>
       </c>
       <c r="T13" s="27" t="s">
-        <v>51</v>
+        <v>129</v>
       </c>
       <c r="U13" s="32" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="V13" s="20">
         <v>46147</v>
@@ -3010,10 +3010,10 @@
         <v>22</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D14" s="22">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E14" s="17">
         <v>1707089</v>
@@ -3050,13 +3050,13 @@
         <v>46042</v>
       </c>
       <c r="R14" s="12">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="T14" s="28" t="s">
-        <v>65</v>
+        <v>126</v>
       </c>
       <c r="U14" s="30" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="V14" s="20">
         <v>46169</v>
@@ -3070,7 +3070,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D15" s="16">
         <v>1</v>
@@ -3126,7 +3126,7 @@
         <v>22</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D16" s="16">
         <v>0</v>
@@ -3169,7 +3169,7 @@
         <v>51</v>
       </c>
       <c r="U16" s="30" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="V16" s="20">
         <v>46182</v>
@@ -3183,7 +3183,7 @@
         <v>12</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D17" s="16">
         <v>1</v>
@@ -3239,7 +3239,7 @@
         <v>12</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D18" s="16">
         <v>1</v>
@@ -3291,7 +3291,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D19" s="16">
         <v>0</v>
@@ -3334,10 +3334,10 @@
         <v>46295</v>
       </c>
       <c r="T19" s="28" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="U19" s="33" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="V19" s="20">
         <v>46203</v>
@@ -3351,7 +3351,7 @@
         <v>22</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D20" s="16">
         <v>0.9</v>
@@ -3379,7 +3379,7 @@
         <v>45737</v>
       </c>
       <c r="T20" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U20" s="27"/>
       <c r="V20" s="20"/>
@@ -3392,7 +3392,7 @@
         <v>22</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D21" s="16">
         <v>0.9</v>
@@ -3415,19 +3415,19 @@
         <v>45737</v>
       </c>
       <c r="T21" s="28" t="s">
-        <v>68</v>
+        <v>127</v>
       </c>
       <c r="V21" s="20"/>
     </row>
     <row r="22" spans="1:22" s="10" customFormat="1" ht="18.600000000000001">
       <c r="A22" s="10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B22" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D22" s="16"/>
       <c r="F22" s="26"/>
@@ -3441,19 +3441,19 @@
       <c r="Q22" s="20"/>
       <c r="R22" s="20"/>
       <c r="T22" s="28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="V22" s="20"/>
     </row>
     <row r="23" spans="1:22" s="10" customFormat="1" ht="18.600000000000001">
       <c r="A23" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D23" s="16">
         <v>0</v>
@@ -3488,13 +3488,13 @@
     </row>
     <row r="24" spans="1:22" s="10" customFormat="1" ht="18.600000000000001">
       <c r="A24" s="10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D24" s="16">
         <v>0</v>
@@ -3505,31 +3505,39 @@
       <c r="F24" s="17">
         <v>0</v>
       </c>
-      <c r="G24" s="17"/>
+      <c r="G24" s="17">
+        <f>400+140</f>
+        <v>540</v>
+      </c>
       <c r="H24" s="17">
         <f>E24*0.4</f>
         <v>81552</v>
       </c>
-      <c r="I24" s="23"/>
+      <c r="I24" s="23">
+        <v>6</v>
+      </c>
       <c r="K24" s="15"/>
       <c r="L24" s="17">
         <f>36480/2</f>
         <v>18240</v>
       </c>
       <c r="N24" s="56">
-        <f>82500-P24</f>
-        <v>17500</v>
+        <v>497</v>
       </c>
       <c r="O24" s="10" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="P24" s="11">
-        <v>65000</v>
-      </c>
-      <c r="Q24" s="20"/>
-      <c r="R24" s="12"/>
+        <v>58000</v>
+      </c>
+      <c r="Q24" s="20">
+        <v>46225</v>
+      </c>
+      <c r="R24" s="12">
+        <v>46227</v>
+      </c>
       <c r="T24" s="28" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="U24" s="33"/>
       <c r="V24" s="20">
@@ -4079,20 +4087,20 @@
         <v>57</v>
       </c>
       <c r="B1" s="57"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
@@ -4104,7 +4112,7 @@
         <v>60</v>
       </c>
       <c r="E4" s="55" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -4124,7 +4132,7 @@
         <v>46185</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>61</v>
@@ -4133,7 +4141,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4141,7 +4149,7 @@
         <v>46189</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>61</v>
@@ -4150,7 +4158,7 @@
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4158,7 +4166,7 @@
         <v>46183</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>62</v>
@@ -4167,7 +4175,7 @@
         <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4175,7 +4183,7 @@
         <v>46185</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>63</v>
@@ -4184,7 +4192,7 @@
         <v>2.5</v>
       </c>
       <c r="E10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -4192,7 +4200,7 @@
         <v>46190</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>61</v>
@@ -4201,7 +4209,7 @@
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -4209,7 +4217,7 @@
         <v>46190</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>63</v>
@@ -4218,7 +4226,7 @@
         <v>3</v>
       </c>
       <c r="E12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -4226,7 +4234,7 @@
         <v>46192</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>61</v>
@@ -4235,7 +4243,7 @@
         <v>3</v>
       </c>
       <c r="E13" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -4243,7 +4251,7 @@
         <v>46197</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>63</v>
@@ -4252,7 +4260,7 @@
         <v>3</v>
       </c>
       <c r="E14" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -4260,7 +4268,7 @@
         <v>46198</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>61</v>
@@ -4269,7 +4277,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -4277,7 +4285,7 @@
         <v>46202</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>61</v>
@@ -4286,7 +4294,7 @@
         <v>6</v>
       </c>
       <c r="E16" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -4294,7 +4302,7 @@
         <v>46205</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>61</v>
@@ -4303,7 +4311,7 @@
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -4311,7 +4319,7 @@
         <v>46209</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>61</v>
@@ -4320,7 +4328,7 @@
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -4328,7 +4336,7 @@
         <v>46211</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>62</v>
@@ -4337,7 +4345,7 @@
         <v>3</v>
       </c>
       <c r="E19" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -4345,16 +4353,16 @@
         <v>46216</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D20" s="4">
         <v>2.6999999999999993</v>
       </c>
       <c r="E20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -4362,7 +4370,7 @@
         <v>46216</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>61</v>
@@ -4371,7 +4379,7 @@
         <v>6</v>
       </c>
       <c r="E21" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -4379,7 +4387,7 @@
         <v>46218</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>61</v>
@@ -4388,7 +4396,7 @@
         <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -4396,7 +4404,7 @@
         <v>46218</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>61</v>
@@ -4405,7 +4413,7 @@
         <v>3</v>
       </c>
       <c r="E23" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -4413,16 +4421,16 @@
         <v>46218</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D24" s="4">
         <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -4430,16 +4438,16 @@
         <v>46218</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D25" s="4">
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -4482,7 +4490,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
       <c r="A1" s="57" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B1" s="57"/>
       <c r="C1" s="57"/>
@@ -4490,20 +4498,20 @@
       <c r="E1" s="57"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="59" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
+      <c r="A2" s="58" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
@@ -4517,10 +4525,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C5" s="6">
         <v>46204</v>
@@ -4529,15 +4537,15 @@
         <v>46224</v>
       </c>
       <c r="E5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C6" s="6">
         <v>46204</v>
@@ -4546,15 +4554,15 @@
         <v>46224</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C7" s="6">
         <v>46204</v>
@@ -4563,11 +4571,11 @@
         <v>46224</v>
       </c>
       <c r="E7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="6"/>
+      <c r="A8" s="3"/>
       <c r="B8" s="5"/>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
@@ -5395,15 +5403,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5414,6 +5413,15 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5670,20 +5678,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-17 15:25)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FAE77B-CAFF-4E48-B1AA-92AECADB3EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CE05AD-A82A-48BF-B807-F10904D9BD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -923,28 +923,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1355,31 +1355,31 @@
       <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1417,7 +1417,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="65" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1437,14 +1437,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="61">
+      <c r="I5" s="66">
         <v>46213</v>
       </c>
-      <c r="J5" s="61"/>
+      <c r="J5" s="66"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="64"/>
+      <c r="A6" s="60"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1462,12 +1462,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="64"/>
-      <c r="J6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="67"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="59" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1487,14 +1487,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="59" t="s">
+      <c r="I7" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="59"/>
+      <c r="J7" s="61"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="64"/>
+      <c r="A8" s="60"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1512,12 +1512,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="64"/>
-      <c r="J8" s="60"/>
+      <c r="I8" s="60"/>
+      <c r="J8" s="67"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="63" t="s">
+      <c r="A9" s="59" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1537,14 +1537,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="59">
+      <c r="I9" s="61">
         <v>46218</v>
       </c>
-      <c r="J9" s="59"/>
+      <c r="J9" s="61"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="64"/>
+      <c r="A10" s="60"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1562,12 +1562,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="64"/>
-      <c r="J10" s="60"/>
+      <c r="I10" s="60"/>
+      <c r="J10" s="67"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="59" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1587,14 +1587,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="59">
+      <c r="I11" s="61">
         <v>46171</v>
       </c>
-      <c r="J11" s="59"/>
+      <c r="J11" s="61"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="64"/>
+      <c r="A12" s="60"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1612,12 +1612,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="64"/>
-      <c r="J12" s="60"/>
+      <c r="I12" s="60"/>
+      <c r="J12" s="67"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="59" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1637,14 +1637,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="59" t="s">
+      <c r="I13" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="59"/>
+      <c r="J13" s="61"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="64"/>
+      <c r="A14" s="60"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1662,12 +1662,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="64"/>
-      <c r="J14" s="60"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="67"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="59" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1687,14 +1687,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="59">
+      <c r="I15" s="61">
         <v>46199</v>
       </c>
-      <c r="J15" s="59"/>
+      <c r="J15" s="61"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="64"/>
+      <c r="A16" s="60"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1712,12 +1712,12 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="64"/>
-      <c r="J16" s="60"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="67"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="64" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="34" t="s">
@@ -1737,14 +1737,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="62">
+      <c r="I17" s="63">
         <v>46305</v>
       </c>
-      <c r="J17" s="62"/>
+      <c r="J17" s="63"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="64"/>
+      <c r="A18" s="60"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1762,12 +1762,12 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="64"/>
-      <c r="J18" s="60"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="67"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="65" t="s">
+      <c r="A19" s="64" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="34" t="s">
@@ -1787,14 +1787,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="62">
+      <c r="I19" s="63">
         <v>46336</v>
       </c>
-      <c r="J19" s="62"/>
+      <c r="J19" s="63"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="64"/>
+      <c r="A20" s="60"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1812,12 +1812,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="64"/>
-      <c r="J20" s="60"/>
+      <c r="I20" s="60"/>
+      <c r="J20" s="67"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="63" t="s">
+      <c r="A21" s="59" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1837,14 +1837,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="59">
+      <c r="I21" s="61">
         <v>46336</v>
       </c>
-      <c r="J21" s="59"/>
+      <c r="J21" s="61"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="64"/>
+      <c r="A22" s="60"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1862,12 +1862,12 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="64"/>
-      <c r="J22" s="60"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="67"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="63" t="s">
+      <c r="A23" s="59" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="43" t="s">
@@ -1887,14 +1887,14 @@
       <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="59">
+      <c r="I23" s="61">
         <v>46220</v>
       </c>
-      <c r="J23" s="59"/>
+      <c r="J23" s="61"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="64"/>
+      <c r="A24" s="60"/>
       <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
@@ -1912,12 +1912,12 @@
       <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="64"/>
-      <c r="J24" s="60"/>
+      <c r="I24" s="60"/>
+      <c r="J24" s="67"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="63" t="s">
+      <c r="A25" s="59" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1937,14 +1937,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="59">
+      <c r="I25" s="61">
         <v>46188</v>
       </c>
-      <c r="J25" s="59"/>
+      <c r="J25" s="61"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="64"/>
+      <c r="A26" s="60"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1962,12 +1962,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="64"/>
-      <c r="J26" s="60"/>
+      <c r="I26" s="60"/>
+      <c r="J26" s="67"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="63" t="s">
+      <c r="A27" s="59" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -1987,14 +1987,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="59">
+      <c r="I27" s="61">
         <v>46321</v>
       </c>
-      <c r="J27" s="59"/>
+      <c r="J27" s="61"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="64"/>
+      <c r="A28" s="60"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2012,12 +2012,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="64"/>
-      <c r="J28" s="60"/>
+      <c r="I28" s="60"/>
+      <c r="J28" s="67"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="63" t="s">
+      <c r="A29" s="59" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2037,14 +2037,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="59">
+      <c r="I29" s="61">
         <v>46139</v>
       </c>
-      <c r="J29" s="59"/>
+      <c r="J29" s="61"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="64"/>
+      <c r="A30" s="60"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2062,12 +2062,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="64"/>
-      <c r="J30" s="60"/>
+      <c r="I30" s="60"/>
+      <c r="J30" s="67"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="59" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2087,14 +2087,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="59">
+      <c r="I31" s="61">
         <v>46133</v>
       </c>
-      <c r="J31" s="59"/>
+      <c r="J31" s="61"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="64"/>
+      <c r="A32" s="60"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2112,12 +2112,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="64"/>
-      <c r="J32" s="60"/>
+      <c r="I32" s="60"/>
+      <c r="J32" s="67"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="63" t="s">
+      <c r="A33" s="59" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2137,14 +2137,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="59">
+      <c r="I33" s="61">
         <v>46295</v>
       </c>
-      <c r="J33" s="59"/>
+      <c r="J33" s="61"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="64"/>
+      <c r="A34" s="60"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2162,12 +2162,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="64"/>
-      <c r="J34" s="60"/>
+      <c r="I34" s="60"/>
+      <c r="J34" s="67"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="59" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2187,14 +2187,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="59">
+      <c r="I35" s="61">
         <v>45737</v>
       </c>
-      <c r="J35" s="59"/>
+      <c r="J35" s="61"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="64"/>
+      <c r="A36" s="60"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2212,12 +2212,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="64"/>
-      <c r="J36" s="60"/>
+      <c r="I36" s="60"/>
+      <c r="J36" s="67"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="63" t="s">
+      <c r="A37" s="59" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2237,14 +2237,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="59">
+      <c r="I37" s="61">
         <v>45737</v>
       </c>
-      <c r="J37" s="59"/>
+      <c r="J37" s="61"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="64"/>
+      <c r="A38" s="60"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2262,12 +2262,49 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="64"/>
-      <c r="J38" s="60"/>
+      <c r="I38" s="60"/>
+      <c r="J38" s="67"/>
       <c r="K38" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="53">
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2284,43 +2321,6 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -3450,7 +3450,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>67</v>
@@ -4087,16 +4087,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="57"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="58" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="58"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5416,15 +5416,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5677,6 +5668,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
@@ -5689,14 +5689,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5713,4 +5705,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-20 09:33)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CE05AD-A82A-48BF-B807-F10904D9BD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A76920B-F05A-4B55-A076-41831A8D29FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -923,28 +923,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1355,31 +1355,31 @@
       <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1417,7 +1417,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="67" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1437,14 +1437,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="66">
+      <c r="I5" s="61">
         <v>46213</v>
       </c>
-      <c r="J5" s="66"/>
+      <c r="J5" s="61"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="60"/>
+      <c r="A6" s="64"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1462,12 +1462,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="60"/>
-      <c r="J6" s="67"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="60"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="63" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1487,14 +1487,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="61" t="s">
+      <c r="I7" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="61"/>
+      <c r="J7" s="59"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="60"/>
+      <c r="A8" s="64"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1512,12 +1512,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="60"/>
-      <c r="J8" s="67"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="60"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="59" t="s">
+      <c r="A9" s="63" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1537,14 +1537,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="61">
+      <c r="I9" s="59">
         <v>46218</v>
       </c>
-      <c r="J9" s="61"/>
+      <c r="J9" s="59"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="60"/>
+      <c r="A10" s="64"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1562,12 +1562,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="60"/>
-      <c r="J10" s="67"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="60"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="59" t="s">
+      <c r="A11" s="63" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1587,14 +1587,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="61">
+      <c r="I11" s="59">
         <v>46171</v>
       </c>
-      <c r="J11" s="61"/>
+      <c r="J11" s="59"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="60"/>
+      <c r="A12" s="64"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1612,12 +1612,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="60"/>
-      <c r="J12" s="67"/>
+      <c r="I12" s="64"/>
+      <c r="J12" s="60"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="59" t="s">
+      <c r="A13" s="63" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1637,14 +1637,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="61" t="s">
+      <c r="I13" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="59"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="60"/>
+      <c r="A14" s="64"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1662,12 +1662,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="60"/>
-      <c r="J14" s="67"/>
+      <c r="I14" s="64"/>
+      <c r="J14" s="60"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="59" t="s">
+      <c r="A15" s="63" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1687,14 +1687,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="61">
+      <c r="I15" s="59">
         <v>46199</v>
       </c>
-      <c r="J15" s="61"/>
+      <c r="J15" s="59"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="60"/>
+      <c r="A16" s="64"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1712,12 +1712,12 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="60"/>
-      <c r="J16" s="67"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="60"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="64" t="s">
+      <c r="A17" s="65" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="34" t="s">
@@ -1737,14 +1737,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="63">
+      <c r="I17" s="62">
         <v>46305</v>
       </c>
-      <c r="J17" s="63"/>
+      <c r="J17" s="62"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="60"/>
+      <c r="A18" s="64"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1762,12 +1762,12 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="60"/>
-      <c r="J18" s="67"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="60"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="64" t="s">
+      <c r="A19" s="65" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="34" t="s">
@@ -1787,14 +1787,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="63">
+      <c r="I19" s="62">
         <v>46336</v>
       </c>
-      <c r="J19" s="63"/>
+      <c r="J19" s="62"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="60"/>
+      <c r="A20" s="64"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1812,12 +1812,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="60"/>
-      <c r="J20" s="67"/>
+      <c r="I20" s="64"/>
+      <c r="J20" s="60"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="59" t="s">
+      <c r="A21" s="63" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1837,14 +1837,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="61">
+      <c r="I21" s="59">
         <v>46336</v>
       </c>
-      <c r="J21" s="61"/>
+      <c r="J21" s="59"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="60"/>
+      <c r="A22" s="64"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1862,12 +1862,12 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="60"/>
-      <c r="J22" s="67"/>
+      <c r="I22" s="64"/>
+      <c r="J22" s="60"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="59" t="s">
+      <c r="A23" s="63" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="43" t="s">
@@ -1887,14 +1887,14 @@
       <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="61">
+      <c r="I23" s="59">
         <v>46220</v>
       </c>
-      <c r="J23" s="61"/>
+      <c r="J23" s="59"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="60"/>
+      <c r="A24" s="64"/>
       <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
@@ -1912,12 +1912,12 @@
       <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="60"/>
-      <c r="J24" s="67"/>
+      <c r="I24" s="64"/>
+      <c r="J24" s="60"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="59" t="s">
+      <c r="A25" s="63" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1937,14 +1937,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="61">
+      <c r="I25" s="59">
         <v>46188</v>
       </c>
-      <c r="J25" s="61"/>
+      <c r="J25" s="59"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="60"/>
+      <c r="A26" s="64"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1962,12 +1962,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="60"/>
-      <c r="J26" s="67"/>
+      <c r="I26" s="64"/>
+      <c r="J26" s="60"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="59" t="s">
+      <c r="A27" s="63" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -1987,14 +1987,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="61">
+      <c r="I27" s="59">
         <v>46321</v>
       </c>
-      <c r="J27" s="61"/>
+      <c r="J27" s="59"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="60"/>
+      <c r="A28" s="64"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2012,12 +2012,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="60"/>
-      <c r="J28" s="67"/>
+      <c r="I28" s="64"/>
+      <c r="J28" s="60"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="63" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2037,14 +2037,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="61">
+      <c r="I29" s="59">
         <v>46139</v>
       </c>
-      <c r="J29" s="61"/>
+      <c r="J29" s="59"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="60"/>
+      <c r="A30" s="64"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2062,12 +2062,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="60"/>
-      <c r="J30" s="67"/>
+      <c r="I30" s="64"/>
+      <c r="J30" s="60"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="59" t="s">
+      <c r="A31" s="63" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2087,14 +2087,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="61">
+      <c r="I31" s="59">
         <v>46133</v>
       </c>
-      <c r="J31" s="61"/>
+      <c r="J31" s="59"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="60"/>
+      <c r="A32" s="64"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2112,12 +2112,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="60"/>
-      <c r="J32" s="67"/>
+      <c r="I32" s="64"/>
+      <c r="J32" s="60"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="63" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2137,14 +2137,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="61">
+      <c r="I33" s="59">
         <v>46295</v>
       </c>
-      <c r="J33" s="61"/>
+      <c r="J33" s="59"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="60"/>
+      <c r="A34" s="64"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2162,12 +2162,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="60"/>
-      <c r="J34" s="67"/>
+      <c r="I34" s="64"/>
+      <c r="J34" s="60"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="59" t="s">
+      <c r="A35" s="63" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2187,14 +2187,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="61">
+      <c r="I35" s="59">
         <v>45737</v>
       </c>
-      <c r="J35" s="61"/>
+      <c r="J35" s="59"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="60"/>
+      <c r="A36" s="64"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2212,12 +2212,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="60"/>
-      <c r="J36" s="67"/>
+      <c r="I36" s="64"/>
+      <c r="J36" s="60"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="59" t="s">
+      <c r="A37" s="63" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2237,14 +2237,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="61">
+      <c r="I37" s="59">
         <v>45737</v>
       </c>
-      <c r="J37" s="61"/>
+      <c r="J37" s="59"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="60"/>
+      <c r="A38" s="64"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2262,26 +2262,35 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="60"/>
-      <c r="J38" s="67"/>
+      <c r="I38" s="64"/>
+      <c r="J38" s="60"/>
       <c r="K38" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2298,29 +2307,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -3013,7 +3013,7 @@
         <v>67</v>
       </c>
       <c r="D14" s="22">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E14" s="17">
         <v>1707089</v>
@@ -4087,16 +4087,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="57"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="58" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="58"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5403,19 +5403,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5668,6 +5655,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5678,17 +5678,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5707,6 +5696,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-20 09:36)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A76920B-F05A-4B55-A076-41831A8D29FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A37062-5A93-4A6E-972C-45BB4D2D5887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="131">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -347,9 +347,6 @@
     <t>The Grand Pinkao</t>
   </si>
   <si>
-    <t>รอสรุปแผนงานหลังจากสำรวจหน้างาน</t>
-  </si>
-  <si>
     <t>Phanasorn</t>
   </si>
   <si>
@@ -432,6 +429,12 @@
   </si>
   <si>
     <t>รองานโครงสร้าง เข้าได้ ปลายเดือน 8</t>
+  </si>
+  <si>
+    <t>https://corallife806.sharepoint.com/:b:/s/CoralLife2/IQB85P7JtoSZT6532Il6VakbAcqfI6xy5EwPf0pgbRJpT3Y?e=Qwe5V0</t>
+  </si>
+  <si>
+    <t>ส่งงาน 100% วันที่ 07/24/2026</t>
   </si>
 </sst>
 </file>
@@ -923,28 +926,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1355,31 +1358,31 @@
       <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1417,7 +1420,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="65" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1437,14 +1440,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="61">
+      <c r="I5" s="66">
         <v>46213</v>
       </c>
-      <c r="J5" s="61"/>
+      <c r="J5" s="66"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="64"/>
+      <c r="A6" s="60"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1462,12 +1465,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="64"/>
-      <c r="J6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="67"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="59" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1487,14 +1490,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="59" t="s">
+      <c r="I7" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="59"/>
+      <c r="J7" s="61"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="64"/>
+      <c r="A8" s="60"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1512,12 +1515,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="64"/>
-      <c r="J8" s="60"/>
+      <c r="I8" s="60"/>
+      <c r="J8" s="67"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="63" t="s">
+      <c r="A9" s="59" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1537,14 +1540,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="59">
+      <c r="I9" s="61">
         <v>46218</v>
       </c>
-      <c r="J9" s="59"/>
+      <c r="J9" s="61"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="64"/>
+      <c r="A10" s="60"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1562,12 +1565,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="64"/>
-      <c r="J10" s="60"/>
+      <c r="I10" s="60"/>
+      <c r="J10" s="67"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="59" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1587,14 +1590,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="59">
+      <c r="I11" s="61">
         <v>46171</v>
       </c>
-      <c r="J11" s="59"/>
+      <c r="J11" s="61"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="64"/>
+      <c r="A12" s="60"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1612,12 +1615,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="64"/>
-      <c r="J12" s="60"/>
+      <c r="I12" s="60"/>
+      <c r="J12" s="67"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="59" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1637,14 +1640,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="59" t="s">
+      <c r="I13" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="59"/>
+      <c r="J13" s="61"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="64"/>
+      <c r="A14" s="60"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1662,12 +1665,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="64"/>
-      <c r="J14" s="60"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="67"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="59" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1687,14 +1690,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="59">
+      <c r="I15" s="61">
         <v>46199</v>
       </c>
-      <c r="J15" s="59"/>
+      <c r="J15" s="61"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="64"/>
+      <c r="A16" s="60"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1712,12 +1715,12 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="64"/>
-      <c r="J16" s="60"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="67"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="64" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="34" t="s">
@@ -1737,14 +1740,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="62">
+      <c r="I17" s="63">
         <v>46305</v>
       </c>
-      <c r="J17" s="62"/>
+      <c r="J17" s="63"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="64"/>
+      <c r="A18" s="60"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1762,12 +1765,12 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="64"/>
-      <c r="J18" s="60"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="67"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="65" t="s">
+      <c r="A19" s="64" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="34" t="s">
@@ -1787,14 +1790,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="62">
+      <c r="I19" s="63">
         <v>46336</v>
       </c>
-      <c r="J19" s="62"/>
+      <c r="J19" s="63"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="64"/>
+      <c r="A20" s="60"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1812,12 +1815,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="64"/>
-      <c r="J20" s="60"/>
+      <c r="I20" s="60"/>
+      <c r="J20" s="67"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="63" t="s">
+      <c r="A21" s="59" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1837,14 +1840,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="59">
+      <c r="I21" s="61">
         <v>46336</v>
       </c>
-      <c r="J21" s="59"/>
+      <c r="J21" s="61"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="64"/>
+      <c r="A22" s="60"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1862,12 +1865,12 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="64"/>
-      <c r="J22" s="60"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="67"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="63" t="s">
+      <c r="A23" s="59" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="43" t="s">
@@ -1887,14 +1890,14 @@
       <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="59">
+      <c r="I23" s="61">
         <v>46220</v>
       </c>
-      <c r="J23" s="59"/>
+      <c r="J23" s="61"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="64"/>
+      <c r="A24" s="60"/>
       <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
@@ -1912,12 +1915,12 @@
       <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="64"/>
-      <c r="J24" s="60"/>
+      <c r="I24" s="60"/>
+      <c r="J24" s="67"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="63" t="s">
+      <c r="A25" s="59" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1937,14 +1940,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="59">
+      <c r="I25" s="61">
         <v>46188</v>
       </c>
-      <c r="J25" s="59"/>
+      <c r="J25" s="61"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="64"/>
+      <c r="A26" s="60"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1962,12 +1965,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="64"/>
-      <c r="J26" s="60"/>
+      <c r="I26" s="60"/>
+      <c r="J26" s="67"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="63" t="s">
+      <c r="A27" s="59" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -1987,14 +1990,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="59">
+      <c r="I27" s="61">
         <v>46321</v>
       </c>
-      <c r="J27" s="59"/>
+      <c r="J27" s="61"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="64"/>
+      <c r="A28" s="60"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2012,12 +2015,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="64"/>
-      <c r="J28" s="60"/>
+      <c r="I28" s="60"/>
+      <c r="J28" s="67"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="63" t="s">
+      <c r="A29" s="59" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2037,14 +2040,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="59">
+      <c r="I29" s="61">
         <v>46139</v>
       </c>
-      <c r="J29" s="59"/>
+      <c r="J29" s="61"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="64"/>
+      <c r="A30" s="60"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2062,12 +2065,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="64"/>
-      <c r="J30" s="60"/>
+      <c r="I30" s="60"/>
+      <c r="J30" s="67"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="59" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2087,14 +2090,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="59">
+      <c r="I31" s="61">
         <v>46133</v>
       </c>
-      <c r="J31" s="59"/>
+      <c r="J31" s="61"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="64"/>
+      <c r="A32" s="60"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2112,12 +2115,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="64"/>
-      <c r="J32" s="60"/>
+      <c r="I32" s="60"/>
+      <c r="J32" s="67"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="63" t="s">
+      <c r="A33" s="59" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2137,14 +2140,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="59">
+      <c r="I33" s="61">
         <v>46295</v>
       </c>
-      <c r="J33" s="59"/>
+      <c r="J33" s="61"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="64"/>
+      <c r="A34" s="60"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2162,12 +2165,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="64"/>
-      <c r="J34" s="60"/>
+      <c r="I34" s="60"/>
+      <c r="J34" s="67"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="59" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2187,14 +2190,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="59">
+      <c r="I35" s="61">
         <v>45737</v>
       </c>
-      <c r="J35" s="59"/>
+      <c r="J35" s="61"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="64"/>
+      <c r="A36" s="60"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2212,12 +2215,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="64"/>
-      <c r="J36" s="60"/>
+      <c r="I36" s="60"/>
+      <c r="J36" s="67"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="63" t="s">
+      <c r="A37" s="59" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2237,14 +2240,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="59">
+      <c r="I37" s="61">
         <v>45737</v>
       </c>
-      <c r="J37" s="59"/>
+      <c r="J37" s="61"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="64"/>
+      <c r="A38" s="60"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2262,12 +2265,49 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="64"/>
-      <c r="J38" s="60"/>
+      <c r="I38" s="60"/>
+      <c r="J38" s="67"/>
       <c r="K38" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="53">
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2284,43 +2324,6 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2877,7 +2880,7 @@
       </c>
       <c r="S11" s="15"/>
       <c r="T11" s="28" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="U11" s="32" t="s">
         <v>83</v>
@@ -2993,7 +2996,7 @@
         <v>46336</v>
       </c>
       <c r="T13" s="27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="U13" s="32" t="s">
         <v>84</v>
@@ -3053,7 +3056,7 @@
         <v>46220</v>
       </c>
       <c r="T14" s="28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="U14" s="30" t="s">
         <v>70</v>
@@ -3415,7 +3418,7 @@
         <v>45737</v>
       </c>
       <c r="T21" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="V21" s="20"/>
     </row>
@@ -3537,9 +3540,11 @@
         <v>46227</v>
       </c>
       <c r="T24" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="U24" s="33"/>
+        <v>130</v>
+      </c>
+      <c r="U24" s="33" t="s">
+        <v>129</v>
+      </c>
       <c r="V24" s="20">
         <v>46213</v>
       </c>
@@ -4065,6 +4070,7 @@
     <hyperlink ref="U13" r:id="rId7" display="https://corallife806.sharepoint.com/:b:/s/CoralLife2/IQBSB6_w6g72TLKUHWGlGBMFARs9IGLaqRfLn5C5zWJMU04?e=8SAokd" xr:uid="{60CE460F-1314-44B6-832C-5ABF13522EB6}"/>
     <hyperlink ref="U16" r:id="rId8" xr:uid="{02895EAD-8F6D-4728-91D1-12231471B411}"/>
     <hyperlink ref="U19" r:id="rId9" xr:uid="{64B77621-4464-4729-B1C8-C74F3BC4DC5C}"/>
+    <hyperlink ref="U24" r:id="rId10" xr:uid="{DFFF659B-3A50-4FD0-AA9F-289AE4EB0963}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4087,16 +4093,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="57"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="58" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="58"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4132,7 +4138,7 @@
         <v>46185</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>61</v>
@@ -4141,7 +4147,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4149,7 +4155,7 @@
         <v>46189</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>61</v>
@@ -4158,7 +4164,7 @@
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4166,7 +4172,7 @@
         <v>46183</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>62</v>
@@ -4175,7 +4181,7 @@
         <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4183,7 +4189,7 @@
         <v>46185</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>63</v>
@@ -4192,7 +4198,7 @@
         <v>2.5</v>
       </c>
       <c r="E10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -4200,7 +4206,7 @@
         <v>46190</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>61</v>
@@ -4209,7 +4215,7 @@
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -4217,7 +4223,7 @@
         <v>46190</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>63</v>
@@ -4226,7 +4232,7 @@
         <v>3</v>
       </c>
       <c r="E12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -4234,7 +4240,7 @@
         <v>46192</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>61</v>
@@ -4243,7 +4249,7 @@
         <v>3</v>
       </c>
       <c r="E13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -4251,7 +4257,7 @@
         <v>46197</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>63</v>
@@ -4260,7 +4266,7 @@
         <v>3</v>
       </c>
       <c r="E14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -4268,7 +4274,7 @@
         <v>46198</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>61</v>
@@ -4277,7 +4283,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -4285,7 +4291,7 @@
         <v>46202</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>61</v>
@@ -4294,7 +4300,7 @@
         <v>6</v>
       </c>
       <c r="E16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -4302,7 +4308,7 @@
         <v>46205</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>61</v>
@@ -4311,7 +4317,7 @@
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -4319,7 +4325,7 @@
         <v>46209</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>61</v>
@@ -4328,7 +4334,7 @@
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -4336,7 +4342,7 @@
         <v>46211</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>62</v>
@@ -4345,7 +4351,7 @@
         <v>3</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -4353,16 +4359,16 @@
         <v>46216</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D20" s="4">
         <v>2.6999999999999993</v>
       </c>
       <c r="E20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -4370,7 +4376,7 @@
         <v>46216</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>61</v>
@@ -4379,7 +4385,7 @@
         <v>6</v>
       </c>
       <c r="E21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -4387,7 +4393,7 @@
         <v>46218</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>61</v>
@@ -4396,7 +4402,7 @@
         <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -4404,7 +4410,7 @@
         <v>46218</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>61</v>
@@ -4413,7 +4419,7 @@
         <v>3</v>
       </c>
       <c r="E23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -4424,13 +4430,13 @@
         <v>100</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D24" s="4">
         <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -4441,13 +4447,13 @@
         <v>100</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D25" s="4">
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -5403,6 +5409,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5655,19 +5674,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5678,6 +5684,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5696,17 +5713,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-20 10:01)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A37062-5A93-4A6E-972C-45BB4D2D5887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FC008C-45B0-4002-96F0-2DCEC69E496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -926,28 +926,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1358,31 +1358,31 @@
       <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1420,7 +1420,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="67" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1440,14 +1440,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="66">
+      <c r="I5" s="61">
         <v>46213</v>
       </c>
-      <c r="J5" s="66"/>
+      <c r="J5" s="61"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="60"/>
+      <c r="A6" s="64"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1465,12 +1465,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="60"/>
-      <c r="J6" s="67"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="60"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="63" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1490,14 +1490,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="61" t="s">
+      <c r="I7" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="61"/>
+      <c r="J7" s="59"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="60"/>
+      <c r="A8" s="64"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1515,12 +1515,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="60"/>
-      <c r="J8" s="67"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="60"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="59" t="s">
+      <c r="A9" s="63" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1540,14 +1540,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="61">
+      <c r="I9" s="59">
         <v>46218</v>
       </c>
-      <c r="J9" s="61"/>
+      <c r="J9" s="59"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="60"/>
+      <c r="A10" s="64"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1565,12 +1565,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="60"/>
-      <c r="J10" s="67"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="60"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="59" t="s">
+      <c r="A11" s="63" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1590,14 +1590,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="61">
+      <c r="I11" s="59">
         <v>46171</v>
       </c>
-      <c r="J11" s="61"/>
+      <c r="J11" s="59"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="60"/>
+      <c r="A12" s="64"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1615,12 +1615,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="60"/>
-      <c r="J12" s="67"/>
+      <c r="I12" s="64"/>
+      <c r="J12" s="60"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="59" t="s">
+      <c r="A13" s="63" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1640,14 +1640,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="61" t="s">
+      <c r="I13" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="59"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="60"/>
+      <c r="A14" s="64"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1665,12 +1665,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="60"/>
-      <c r="J14" s="67"/>
+      <c r="I14" s="64"/>
+      <c r="J14" s="60"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="59" t="s">
+      <c r="A15" s="63" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1690,14 +1690,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="61">
+      <c r="I15" s="59">
         <v>46199</v>
       </c>
-      <c r="J15" s="61"/>
+      <c r="J15" s="59"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="60"/>
+      <c r="A16" s="64"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1715,12 +1715,12 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="60"/>
-      <c r="J16" s="67"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="60"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="64" t="s">
+      <c r="A17" s="65" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="34" t="s">
@@ -1740,14 +1740,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="63">
+      <c r="I17" s="62">
         <v>46305</v>
       </c>
-      <c r="J17" s="63"/>
+      <c r="J17" s="62"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="60"/>
+      <c r="A18" s="64"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1765,12 +1765,12 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="60"/>
-      <c r="J18" s="67"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="60"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="64" t="s">
+      <c r="A19" s="65" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="34" t="s">
@@ -1790,14 +1790,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="63">
+      <c r="I19" s="62">
         <v>46336</v>
       </c>
-      <c r="J19" s="63"/>
+      <c r="J19" s="62"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="60"/>
+      <c r="A20" s="64"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1815,12 +1815,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="60"/>
-      <c r="J20" s="67"/>
+      <c r="I20" s="64"/>
+      <c r="J20" s="60"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="59" t="s">
+      <c r="A21" s="63" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1840,14 +1840,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="61">
+      <c r="I21" s="59">
         <v>46336</v>
       </c>
-      <c r="J21" s="61"/>
+      <c r="J21" s="59"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="60"/>
+      <c r="A22" s="64"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1865,12 +1865,12 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="60"/>
-      <c r="J22" s="67"/>
+      <c r="I22" s="64"/>
+      <c r="J22" s="60"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="59" t="s">
+      <c r="A23" s="63" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="43" t="s">
@@ -1890,14 +1890,14 @@
       <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="61">
+      <c r="I23" s="59">
         <v>46220</v>
       </c>
-      <c r="J23" s="61"/>
+      <c r="J23" s="59"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="60"/>
+      <c r="A24" s="64"/>
       <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
@@ -1915,12 +1915,12 @@
       <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="60"/>
-      <c r="J24" s="67"/>
+      <c r="I24" s="64"/>
+      <c r="J24" s="60"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="59" t="s">
+      <c r="A25" s="63" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1940,14 +1940,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="61">
+      <c r="I25" s="59">
         <v>46188</v>
       </c>
-      <c r="J25" s="61"/>
+      <c r="J25" s="59"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="60"/>
+      <c r="A26" s="64"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1965,12 +1965,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="60"/>
-      <c r="J26" s="67"/>
+      <c r="I26" s="64"/>
+      <c r="J26" s="60"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="59" t="s">
+      <c r="A27" s="63" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -1990,14 +1990,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="61">
+      <c r="I27" s="59">
         <v>46321</v>
       </c>
-      <c r="J27" s="61"/>
+      <c r="J27" s="59"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="60"/>
+      <c r="A28" s="64"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2015,12 +2015,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="60"/>
-      <c r="J28" s="67"/>
+      <c r="I28" s="64"/>
+      <c r="J28" s="60"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="63" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2040,14 +2040,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="61">
+      <c r="I29" s="59">
         <v>46139</v>
       </c>
-      <c r="J29" s="61"/>
+      <c r="J29" s="59"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="60"/>
+      <c r="A30" s="64"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2065,12 +2065,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="60"/>
-      <c r="J30" s="67"/>
+      <c r="I30" s="64"/>
+      <c r="J30" s="60"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="59" t="s">
+      <c r="A31" s="63" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2090,14 +2090,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="61">
+      <c r="I31" s="59">
         <v>46133</v>
       </c>
-      <c r="J31" s="61"/>
+      <c r="J31" s="59"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="60"/>
+      <c r="A32" s="64"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2115,12 +2115,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="60"/>
-      <c r="J32" s="67"/>
+      <c r="I32" s="64"/>
+      <c r="J32" s="60"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="63" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2140,14 +2140,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="61">
+      <c r="I33" s="59">
         <v>46295</v>
       </c>
-      <c r="J33" s="61"/>
+      <c r="J33" s="59"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="60"/>
+      <c r="A34" s="64"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2165,12 +2165,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="60"/>
-      <c r="J34" s="67"/>
+      <c r="I34" s="64"/>
+      <c r="J34" s="60"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="59" t="s">
+      <c r="A35" s="63" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2190,14 +2190,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="61">
+      <c r="I35" s="59">
         <v>45737</v>
       </c>
-      <c r="J35" s="61"/>
+      <c r="J35" s="59"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="60"/>
+      <c r="A36" s="64"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2215,12 +2215,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="60"/>
-      <c r="J36" s="67"/>
+      <c r="I36" s="64"/>
+      <c r="J36" s="60"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="59" t="s">
+      <c r="A37" s="63" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2240,14 +2240,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="61">
+      <c r="I37" s="59">
         <v>45737</v>
       </c>
-      <c r="J37" s="61"/>
+      <c r="J37" s="59"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="60"/>
+      <c r="A38" s="64"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2265,26 +2265,35 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="60"/>
-      <c r="J38" s="67"/>
+      <c r="I38" s="64"/>
+      <c r="J38" s="60"/>
       <c r="K38" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2301,29 +2310,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -4093,16 +4093,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="57"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="58" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="58"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5409,19 +5409,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5674,6 +5661,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5684,17 +5684,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5713,6 +5702,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-20 17:47)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\Desktop\Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FC008C-45B0-4002-96F0-2DCEC69E496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{A99066B1-997E-44F2-9F7D-DC0E9654FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C6943DA-79D2-448E-9995-3F7348B8A102}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="132">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -435,6 +435,9 @@
   </si>
   <si>
     <t>ส่งงาน 100% วันที่ 07/24/2026</t>
+  </si>
+  <si>
+    <t>บ้านคุณทวีชัย สมุทปราการ</t>
   </si>
 </sst>
 </file>
@@ -766,7 +769,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -948,6 +951,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1340,7 +1361,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="41.33203125" bestFit="1" customWidth="1"/>
@@ -2269,8 +2290,88 @@
       <c r="J38" s="60"/>
       <c r="K38" s="54"/>
     </row>
+    <row r="39" spans="1:11">
+      <c r="A39" s="63" t="s">
+        <v>131</v>
+      </c>
+      <c r="B39" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="C39" s="69"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="69"/>
+      <c r="F39" s="69"/>
+      <c r="G39" s="70"/>
+      <c r="H39" s="68"/>
+      <c r="I39" s="59"/>
+      <c r="J39" s="59"/>
+      <c r="K39" s="53"/>
+    </row>
+    <row r="40" spans="1:11" ht="15" thickBot="1">
+      <c r="A40" s="64"/>
+      <c r="B40" s="71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="72"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="72"/>
+      <c r="G40" s="73"/>
+      <c r="H40" s="71"/>
+      <c r="I40" s="64"/>
+      <c r="J40" s="60"/>
+      <c r="K40" s="54"/>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" s="63" t="s">
+        <v>100</v>
+      </c>
+      <c r="B41" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="69">
+        <v>46225</v>
+      </c>
+      <c r="D41" s="69">
+        <v>46227</v>
+      </c>
+      <c r="E41" s="69"/>
+      <c r="F41" s="69"/>
+      <c r="G41" s="70">
+        <v>0</v>
+      </c>
+      <c r="H41" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="I41" s="59">
+        <v>46227</v>
+      </c>
+      <c r="J41" s="59"/>
+      <c r="K41" s="53"/>
+    </row>
+    <row r="42" spans="1:11" ht="15" thickBot="1">
+      <c r="A42" s="64"/>
+      <c r="B42" s="71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="72"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
+      <c r="G42" s="73"/>
+      <c r="H42" s="71"/>
+      <c r="I42" s="64"/>
+      <c r="J42" s="60"/>
+      <c r="K42" s="54"/>
+    </row>
   </sheetData>
-  <mergeCells count="53">
+  <mergeCells count="59">
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -4049,7 +4150,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-21 15:59)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{A99066B1-997E-44F2-9F7D-DC0E9654FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C6943DA-79D2-448E-9995-3F7348B8A102}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{A99066B1-997E-44F2-9F7D-DC0E9654FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC8067FE-3EFF-493D-9D70-ACAA281592D9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="132">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -769,7 +769,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -927,6 +927,15 @@
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -951,24 +960,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1376,34 +1367,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1441,7 +1432,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="70" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1461,14 +1452,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="61">
+      <c r="I5" s="64">
         <v>46213</v>
       </c>
-      <c r="J5" s="61"/>
+      <c r="J5" s="64"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="64"/>
+      <c r="A6" s="67"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1486,12 +1477,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="64"/>
-      <c r="J6" s="60"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="63"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="66" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1511,14 +1502,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="59" t="s">
+      <c r="I7" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="59"/>
+      <c r="J7" s="62"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="64"/>
+      <c r="A8" s="67"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1536,12 +1527,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="64"/>
-      <c r="J8" s="60"/>
+      <c r="I8" s="67"/>
+      <c r="J8" s="63"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="63" t="s">
+      <c r="A9" s="66" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1561,14 +1552,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="59">
+      <c r="I9" s="62">
         <v>46218</v>
       </c>
-      <c r="J9" s="59"/>
+      <c r="J9" s="62"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="64"/>
+      <c r="A10" s="67"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1586,12 +1577,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="64"/>
-      <c r="J10" s="60"/>
+      <c r="I10" s="67"/>
+      <c r="J10" s="63"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="66" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1611,14 +1602,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="59">
+      <c r="I11" s="62">
         <v>46171</v>
       </c>
-      <c r="J11" s="59"/>
+      <c r="J11" s="62"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="64"/>
+      <c r="A12" s="67"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1636,12 +1627,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="64"/>
-      <c r="J12" s="60"/>
+      <c r="I12" s="67"/>
+      <c r="J12" s="63"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="66" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1661,14 +1652,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="59" t="s">
+      <c r="I13" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="59"/>
+      <c r="J13" s="62"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="64"/>
+      <c r="A14" s="67"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1686,12 +1677,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="64"/>
-      <c r="J14" s="60"/>
+      <c r="I14" s="67"/>
+      <c r="J14" s="63"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="66" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1711,14 +1702,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="59">
+      <c r="I15" s="62">
         <v>46199</v>
       </c>
-      <c r="J15" s="59"/>
+      <c r="J15" s="62"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="64"/>
+      <c r="A16" s="67"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1736,12 +1727,12 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="64"/>
-      <c r="J16" s="60"/>
+      <c r="I16" s="67"/>
+      <c r="J16" s="63"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="68" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="34" t="s">
@@ -1761,14 +1752,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="62">
+      <c r="I17" s="65">
         <v>46305</v>
       </c>
-      <c r="J17" s="62"/>
+      <c r="J17" s="65"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="64"/>
+      <c r="A18" s="67"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1786,12 +1777,12 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="64"/>
-      <c r="J18" s="60"/>
+      <c r="I18" s="67"/>
+      <c r="J18" s="63"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="65" t="s">
+      <c r="A19" s="68" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="34" t="s">
@@ -1811,14 +1802,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="62">
+      <c r="I19" s="65">
         <v>46336</v>
       </c>
-      <c r="J19" s="62"/>
+      <c r="J19" s="65"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="64"/>
+      <c r="A20" s="67"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1836,12 +1827,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="64"/>
-      <c r="J20" s="60"/>
+      <c r="I20" s="67"/>
+      <c r="J20" s="63"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="63" t="s">
+      <c r="A21" s="66" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1861,14 +1852,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="59">
+      <c r="I21" s="62">
         <v>46336</v>
       </c>
-      <c r="J21" s="59"/>
+      <c r="J21" s="62"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="64"/>
+      <c r="A22" s="67"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1886,12 +1877,12 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="64"/>
-      <c r="J22" s="60"/>
+      <c r="I22" s="67"/>
+      <c r="J22" s="63"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="63" t="s">
+      <c r="A23" s="66" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="43" t="s">
@@ -1911,14 +1902,14 @@
       <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="59">
+      <c r="I23" s="62">
         <v>46220</v>
       </c>
-      <c r="J23" s="59"/>
+      <c r="J23" s="62"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="64"/>
+      <c r="A24" s="67"/>
       <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
@@ -1936,12 +1927,12 @@
       <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="64"/>
-      <c r="J24" s="60"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="63"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="63" t="s">
+      <c r="A25" s="66" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1961,14 +1952,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="59">
+      <c r="I25" s="62">
         <v>46188</v>
       </c>
-      <c r="J25" s="59"/>
+      <c r="J25" s="62"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="64"/>
+      <c r="A26" s="67"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1986,12 +1977,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="64"/>
-      <c r="J26" s="60"/>
+      <c r="I26" s="67"/>
+      <c r="J26" s="63"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="63" t="s">
+      <c r="A27" s="66" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -2011,14 +2002,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="59">
+      <c r="I27" s="62">
         <v>46321</v>
       </c>
-      <c r="J27" s="59"/>
+      <c r="J27" s="62"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="64"/>
+      <c r="A28" s="67"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2036,12 +2027,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="64"/>
-      <c r="J28" s="60"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="63"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="63" t="s">
+      <c r="A29" s="66" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2061,14 +2052,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="59">
+      <c r="I29" s="62">
         <v>46139</v>
       </c>
-      <c r="J29" s="59"/>
+      <c r="J29" s="62"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="64"/>
+      <c r="A30" s="67"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2086,12 +2077,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="64"/>
-      <c r="J30" s="60"/>
+      <c r="I30" s="67"/>
+      <c r="J30" s="63"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="66" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2111,14 +2102,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="59">
+      <c r="I31" s="62">
         <v>46133</v>
       </c>
-      <c r="J31" s="59"/>
+      <c r="J31" s="62"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="64"/>
+      <c r="A32" s="67"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2136,12 +2127,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="64"/>
-      <c r="J32" s="60"/>
+      <c r="I32" s="67"/>
+      <c r="J32" s="63"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="63" t="s">
+      <c r="A33" s="66" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2161,14 +2152,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="59">
+      <c r="I33" s="62">
         <v>46295</v>
       </c>
-      <c r="J33" s="59"/>
+      <c r="J33" s="62"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="64"/>
+      <c r="A34" s="67"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2186,12 +2177,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="64"/>
-      <c r="J34" s="60"/>
+      <c r="I34" s="67"/>
+      <c r="J34" s="63"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="66" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2211,14 +2202,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="59">
+      <c r="I35" s="62">
         <v>45737</v>
       </c>
-      <c r="J35" s="59"/>
+      <c r="J35" s="62"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="64"/>
+      <c r="A36" s="67"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2236,12 +2227,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="64"/>
-      <c r="J36" s="60"/>
+      <c r="I36" s="67"/>
+      <c r="J36" s="63"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="63" t="s">
+      <c r="A37" s="66" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2261,14 +2252,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="59">
+      <c r="I37" s="62">
         <v>45737</v>
       </c>
-      <c r="J37" s="59"/>
+      <c r="J37" s="62"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="64"/>
+      <c r="A38" s="67"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2286,82 +2277,90 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="64"/>
-      <c r="J38" s="60"/>
+      <c r="I38" s="67"/>
+      <c r="J38" s="63"/>
       <c r="K38" s="54"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="63" t="s">
+      <c r="A39" s="66" t="s">
         <v>131</v>
       </c>
-      <c r="B39" s="68" t="s">
+      <c r="B39" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="69"/>
-      <c r="D39" s="69"/>
-      <c r="E39" s="69"/>
-      <c r="F39" s="69"/>
-      <c r="G39" s="70"/>
-      <c r="H39" s="68"/>
-      <c r="I39" s="59"/>
-      <c r="J39" s="59"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="42">
+        <v>0</v>
+      </c>
+      <c r="H39" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="I39" s="62"/>
+      <c r="J39" s="62"/>
       <c r="K39" s="53"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="64"/>
-      <c r="B40" s="71" t="s">
+      <c r="A40" s="67"/>
+      <c r="B40" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C40" s="72"/>
-      <c r="D40" s="72"/>
-      <c r="E40" s="72"/>
-      <c r="F40" s="72"/>
-      <c r="G40" s="73"/>
-      <c r="H40" s="71"/>
-      <c r="I40" s="64"/>
-      <c r="J40" s="60"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="59">
+        <v>0</v>
+      </c>
+      <c r="H40" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="I40" s="67"/>
+      <c r="J40" s="63"/>
       <c r="K40" s="54"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="63" t="s">
+      <c r="A41" s="66" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="68" t="s">
+      <c r="B41" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="69">
+      <c r="C41" s="41">
         <v>46225</v>
       </c>
-      <c r="D41" s="69">
+      <c r="D41" s="41">
         <v>46227</v>
       </c>
-      <c r="E41" s="69"/>
-      <c r="F41" s="69"/>
-      <c r="G41" s="70">
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="42">
         <v>0</v>
       </c>
-      <c r="H41" s="68" t="s">
+      <c r="H41" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="59">
+      <c r="I41" s="62">
         <v>46227</v>
       </c>
-      <c r="J41" s="59"/>
+      <c r="J41" s="62"/>
       <c r="K41" s="53"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="64"/>
-      <c r="B42" s="71" t="s">
+      <c r="A42" s="67"/>
+      <c r="B42" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C42" s="72"/>
-      <c r="D42" s="72"/>
-      <c r="E42" s="72"/>
-      <c r="F42" s="72"/>
-      <c r="G42" s="73"/>
-      <c r="H42" s="71"/>
-      <c r="I42" s="64"/>
-      <c r="J42" s="60"/>
+      <c r="C42" s="58"/>
+      <c r="D42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="58"/>
+      <c r="G42" s="59"/>
+      <c r="H42" s="57"/>
+      <c r="I42" s="67"/>
+      <c r="J42" s="63"/>
       <c r="K42" s="54"/>
     </row>
   </sheetData>
@@ -2460,56 +2459,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="57"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="Q2" s="58"/>
-      <c r="R2" s="58"/>
-      <c r="S2" s="58"/>
-      <c r="T2" s="58"/>
-      <c r="U2" s="58"/>
-      <c r="V2" s="58"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
+      <c r="N2" s="61"/>
+      <c r="O2" s="61"/>
+      <c r="P2" s="61"/>
+      <c r="Q2" s="61"/>
+      <c r="R2" s="61"/>
+      <c r="S2" s="61"/>
+      <c r="T2" s="61"/>
+      <c r="U2" s="61"/>
+      <c r="V2" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -3575,7 +3574,9 @@
       </c>
       <c r="I23" s="23"/>
       <c r="K23" s="15"/>
-      <c r="L23" s="17"/>
+      <c r="L23" s="17">
+        <v>15000</v>
+      </c>
       <c r="O23" s="10" t="s">
         <v>54</v>
       </c>
@@ -3622,8 +3623,7 @@
       </c>
       <c r="K24" s="15"/>
       <c r="L24" s="17">
-        <f>36480/2</f>
-        <v>18240</v>
+        <v>13500</v>
       </c>
       <c r="N24" s="56">
         <v>497</v>
@@ -4150,7 +4150,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4190,20 +4190,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4596,22 +4596,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5510,6 +5510,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5762,7 +5771,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5775,16 +5784,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5803,7 +5811,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5812,12 +5820,4 @@
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-21 16:04)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{A99066B1-997E-44F2-9F7D-DC0E9654FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC8067FE-3EFF-493D-9D70-ACAA281592D9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BD7622-B184-4FD8-9186-EA2DC3959814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -938,28 +938,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1370,31 +1370,31 @@
       <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1432,7 +1432,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="69" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1452,14 +1452,14 @@
       <c r="H5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="64">
+      <c r="I5" s="70">
         <v>46213</v>
       </c>
-      <c r="J5" s="64"/>
+      <c r="J5" s="70"/>
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="67"/>
+      <c r="A6" s="63"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
@@ -1477,12 +1477,12 @@
       <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="67"/>
-      <c r="J6" s="63"/>
+      <c r="I6" s="63"/>
+      <c r="J6" s="65"/>
       <c r="K6" s="50"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="66" t="s">
+      <c r="A7" s="62" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="40" t="s">
@@ -1502,14 +1502,14 @@
       <c r="H7" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="62" t="s">
+      <c r="I7" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="62"/>
+      <c r="J7" s="64"/>
       <c r="K7" s="51"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="67"/>
+      <c r="A8" s="63"/>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
@@ -1527,12 +1527,12 @@
       <c r="H8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="67"/>
-      <c r="J8" s="63"/>
+      <c r="I8" s="63"/>
+      <c r="J8" s="65"/>
       <c r="K8" s="50"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="66" t="s">
+      <c r="A9" s="62" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="40" t="s">
@@ -1552,14 +1552,14 @@
       <c r="H9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="64">
         <v>46218</v>
       </c>
-      <c r="J9" s="62"/>
+      <c r="J9" s="64"/>
       <c r="K9" s="51"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="67"/>
+      <c r="A10" s="63"/>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
@@ -1577,12 +1577,12 @@
       <c r="H10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="67"/>
-      <c r="J10" s="63"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="65"/>
       <c r="K10" s="50"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="62" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -1602,14 +1602,14 @@
       <c r="H11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="62">
+      <c r="I11" s="64">
         <v>46171</v>
       </c>
-      <c r="J11" s="62"/>
+      <c r="J11" s="64"/>
       <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="67"/>
+      <c r="A12" s="63"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
@@ -1627,12 +1627,12 @@
       <c r="H12" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="67"/>
-      <c r="J12" s="63"/>
+      <c r="I12" s="63"/>
+      <c r="J12" s="65"/>
       <c r="K12" s="50"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="66" t="s">
+      <c r="A13" s="62" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="40" t="s">
@@ -1652,14 +1652,14 @@
       <c r="H13" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="62" t="s">
+      <c r="I13" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="62"/>
+      <c r="J13" s="64"/>
       <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="67"/>
+      <c r="A14" s="63"/>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
@@ -1677,12 +1677,12 @@
       <c r="H14" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="67"/>
-      <c r="J14" s="63"/>
+      <c r="I14" s="63"/>
+      <c r="J14" s="65"/>
       <c r="K14" s="50"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="66" t="s">
+      <c r="A15" s="62" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="43" t="s">
@@ -1702,14 +1702,14 @@
       <c r="H15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="62">
+      <c r="I15" s="64">
         <v>46199</v>
       </c>
-      <c r="J15" s="62"/>
+      <c r="J15" s="64"/>
       <c r="K15" s="51"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="67"/>
+      <c r="A16" s="63"/>
       <c r="B16" s="46" t="s">
         <v>13</v>
       </c>
@@ -1727,8 +1727,8 @@
       <c r="H16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="67"/>
-      <c r="J16" s="63"/>
+      <c r="I16" s="63"/>
+      <c r="J16" s="65"/>
       <c r="K16" s="50"/>
     </row>
     <row r="17" spans="1:11">
@@ -1752,14 +1752,14 @@
       <c r="H17" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="65">
+      <c r="I17" s="67">
         <v>46305</v>
       </c>
-      <c r="J17" s="65"/>
+      <c r="J17" s="67"/>
       <c r="K17" s="52"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="67"/>
+      <c r="A18" s="63"/>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
@@ -1777,8 +1777,8 @@
       <c r="H18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="67"/>
-      <c r="J18" s="63"/>
+      <c r="I18" s="63"/>
+      <c r="J18" s="65"/>
       <c r="K18" s="50"/>
     </row>
     <row r="19" spans="1:11">
@@ -1802,14 +1802,14 @@
       <c r="H19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="65">
+      <c r="I19" s="67">
         <v>46336</v>
       </c>
-      <c r="J19" s="65"/>
+      <c r="J19" s="67"/>
       <c r="K19" s="52"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="67"/>
+      <c r="A20" s="63"/>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
@@ -1827,12 +1827,12 @@
       <c r="H20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="67"/>
-      <c r="J20" s="63"/>
+      <c r="I20" s="63"/>
+      <c r="J20" s="65"/>
       <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="62" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="40" t="s">
@@ -1852,14 +1852,14 @@
       <c r="H21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="62">
+      <c r="I21" s="64">
         <v>46336</v>
       </c>
-      <c r="J21" s="62"/>
+      <c r="J21" s="64"/>
       <c r="K21" s="53"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="67"/>
+      <c r="A22" s="63"/>
       <c r="B22" s="37" t="s">
         <v>13</v>
       </c>
@@ -1877,12 +1877,12 @@
       <c r="H22" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="67"/>
-      <c r="J22" s="63"/>
+      <c r="I22" s="63"/>
+      <c r="J22" s="65"/>
       <c r="K22" s="54"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="62" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="43" t="s">
@@ -1902,14 +1902,14 @@
       <c r="H23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="62">
+      <c r="I23" s="64">
         <v>46220</v>
       </c>
-      <c r="J23" s="62"/>
+      <c r="J23" s="64"/>
       <c r="K23" s="53"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="67"/>
+      <c r="A24" s="63"/>
       <c r="B24" s="46" t="s">
         <v>13</v>
       </c>
@@ -1927,12 +1927,12 @@
       <c r="H24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="67"/>
-      <c r="J24" s="63"/>
+      <c r="I24" s="63"/>
+      <c r="J24" s="65"/>
       <c r="K24" s="54"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="66" t="s">
+      <c r="A25" s="62" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="43" t="s">
@@ -1952,14 +1952,14 @@
       <c r="H25" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="62">
+      <c r="I25" s="64">
         <v>46188</v>
       </c>
-      <c r="J25" s="62"/>
+      <c r="J25" s="64"/>
       <c r="K25" s="53"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="67"/>
+      <c r="A26" s="63"/>
       <c r="B26" s="46" t="s">
         <v>13</v>
       </c>
@@ -1977,12 +1977,12 @@
       <c r="H26" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="67"/>
-      <c r="J26" s="63"/>
+      <c r="I26" s="63"/>
+      <c r="J26" s="65"/>
       <c r="K26" s="54"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="62" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="40" t="s">
@@ -2002,14 +2002,14 @@
       <c r="H27" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="62">
+      <c r="I27" s="64">
         <v>46321</v>
       </c>
-      <c r="J27" s="62"/>
+      <c r="J27" s="64"/>
       <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="67"/>
+      <c r="A28" s="63"/>
       <c r="B28" s="37" t="s">
         <v>13</v>
       </c>
@@ -2027,12 +2027,12 @@
       <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="67"/>
-      <c r="J28" s="63"/>
+      <c r="I28" s="63"/>
+      <c r="J28" s="65"/>
       <c r="K28" s="54"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="66" t="s">
+      <c r="A29" s="62" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="43" t="s">
@@ -2052,14 +2052,14 @@
       <c r="H29" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="62">
+      <c r="I29" s="64">
         <v>46139</v>
       </c>
-      <c r="J29" s="62"/>
+      <c r="J29" s="64"/>
       <c r="K29" s="53"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="67"/>
+      <c r="A30" s="63"/>
       <c r="B30" s="46" t="s">
         <v>13</v>
       </c>
@@ -2077,12 +2077,12 @@
       <c r="H30" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="67"/>
-      <c r="J30" s="63"/>
+      <c r="I30" s="63"/>
+      <c r="J30" s="65"/>
       <c r="K30" s="54"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="66" t="s">
+      <c r="A31" s="62" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="43" t="s">
@@ -2102,14 +2102,14 @@
       <c r="H31" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="62">
+      <c r="I31" s="64">
         <v>46133</v>
       </c>
-      <c r="J31" s="62"/>
+      <c r="J31" s="64"/>
       <c r="K31" s="53"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="67"/>
+      <c r="A32" s="63"/>
       <c r="B32" s="46" t="s">
         <v>13</v>
       </c>
@@ -2127,12 +2127,12 @@
       <c r="H32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="67"/>
-      <c r="J32" s="63"/>
+      <c r="I32" s="63"/>
+      <c r="J32" s="65"/>
       <c r="K32" s="54"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="66" t="s">
+      <c r="A33" s="62" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="40" t="s">
@@ -2152,14 +2152,14 @@
       <c r="H33" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="62">
+      <c r="I33" s="64">
         <v>46295</v>
       </c>
-      <c r="J33" s="62"/>
+      <c r="J33" s="64"/>
       <c r="K33" s="53"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="67"/>
+      <c r="A34" s="63"/>
       <c r="B34" s="37" t="s">
         <v>13</v>
       </c>
@@ -2177,12 +2177,12 @@
       <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="67"/>
-      <c r="J34" s="63"/>
+      <c r="I34" s="63"/>
+      <c r="J34" s="65"/>
       <c r="K34" s="54"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="66" t="s">
+      <c r="A35" s="62" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -2202,14 +2202,14 @@
       <c r="H35" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="62">
+      <c r="I35" s="64">
         <v>45737</v>
       </c>
-      <c r="J35" s="62"/>
+      <c r="J35" s="64"/>
       <c r="K35" s="53"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="67"/>
+      <c r="A36" s="63"/>
       <c r="B36" s="37" t="s">
         <v>13</v>
       </c>
@@ -2227,12 +2227,12 @@
       <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="67"/>
-      <c r="J36" s="63"/>
+      <c r="I36" s="63"/>
+      <c r="J36" s="65"/>
       <c r="K36" s="54"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="66" t="s">
+      <c r="A37" s="62" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="40" t="s">
@@ -2252,14 +2252,14 @@
       <c r="H37" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="62">
+      <c r="I37" s="64">
         <v>45737</v>
       </c>
-      <c r="J37" s="62"/>
+      <c r="J37" s="64"/>
       <c r="K37" s="53"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="67"/>
+      <c r="A38" s="63"/>
       <c r="B38" s="37" t="s">
         <v>13</v>
       </c>
@@ -2277,12 +2277,12 @@
       <c r="H38" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="67"/>
-      <c r="J38" s="63"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="65"/>
       <c r="K38" s="54"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="66" t="s">
+      <c r="A39" s="62" t="s">
         <v>131</v>
       </c>
       <c r="B39" s="40" t="s">
@@ -2298,12 +2298,12 @@
       <c r="H39" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I39" s="62"/>
-      <c r="J39" s="62"/>
+      <c r="I39" s="64"/>
+      <c r="J39" s="64"/>
       <c r="K39" s="53"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="67"/>
+      <c r="A40" s="63"/>
       <c r="B40" s="57" t="s">
         <v>13</v>
       </c>
@@ -2317,12 +2317,12 @@
       <c r="H40" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="67"/>
-      <c r="J40" s="63"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="65"/>
       <c r="K40" s="54"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="66" t="s">
+      <c r="A41" s="62" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="40" t="s">
@@ -2342,14 +2342,14 @@
       <c r="H41" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="62">
+      <c r="I41" s="64">
         <v>46227</v>
       </c>
-      <c r="J41" s="62"/>
+      <c r="J41" s="64"/>
       <c r="K41" s="53"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="67"/>
+      <c r="A42" s="63"/>
       <c r="B42" s="57" t="s">
         <v>13</v>
       </c>
@@ -2359,18 +2359,49 @@
       <c r="F42" s="58"/>
       <c r="G42" s="59"/>
       <c r="H42" s="57"/>
-      <c r="I42" s="67"/>
-      <c r="J42" s="63"/>
+      <c r="I42" s="63"/>
+      <c r="J42" s="65"/>
       <c r="K42" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2387,43 +2418,12 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2444,8 +2444,8 @@
     <col min="4" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="10" max="10" width="13" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="16" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="18" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
@@ -2883,8 +2883,8 @@
         <v>338450.2</v>
       </c>
       <c r="F10" s="17">
-        <f>P10*0.8</f>
-        <v>110400</v>
+        <f>P10*1</f>
+        <v>138000</v>
       </c>
       <c r="G10" s="17">
         <v>370</v>
@@ -2944,8 +2944,8 @@
         <v>1156111.18</v>
       </c>
       <c r="F11" s="17">
-        <f>P11*0.5</f>
-        <v>140000</v>
+        <f>P11*0.8</f>
+        <v>224000</v>
       </c>
       <c r="G11" s="17">
         <v>840</v>
@@ -4194,16 +4194,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="60"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="61" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="61"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5510,15 +5510,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5771,6 +5762,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5785,14 +5785,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5811,6 +5803,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 10:26)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BD7622-B184-4FD8-9186-EA2DC3959814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EAC909E-603B-4776-A9D2-B09EBA2A8D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3553,7 +3553,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 13:14)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -939,39 +939,39 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1369,34 +1369,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1434,34 +1434,34 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="71">
+      <c r="C5" s="60">
         <v>46084</v>
       </c>
-      <c r="D5" s="71">
+      <c r="D5" s="60">
         <v>46127</v>
       </c>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="72">
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="61">
         <v>1</v>
       </c>
-      <c r="H5" s="70" t="s">
+      <c r="H5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="69">
+      <c r="I5" s="64">
         <v>46213</v>
       </c>
-      <c r="J5" s="69"/>
+      <c r="J5" s="64"/>
       <c r="K5" s="48"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="62"/>
+      <c r="A6" s="67"/>
       <c r="B6" s="45" t="s">
         <v>13</v>
       </c>
@@ -1479,12 +1479,12 @@
       <c r="H6" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="62"/>
-      <c r="J6" s="64"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="63"/>
       <c r="K6" s="49"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="66" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="39" t="s">
@@ -1504,14 +1504,14 @@
       <c r="H7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="63" t="s">
+      <c r="I7" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="63"/>
+      <c r="J7" s="62"/>
       <c r="K7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="62"/>
+      <c r="A8" s="67"/>
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1529,12 +1529,12 @@
       <c r="H8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="62"/>
-      <c r="J8" s="64"/>
+      <c r="I8" s="67"/>
+      <c r="J8" s="63"/>
       <c r="K8" s="49"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="66" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="39" t="s">
@@ -1554,14 +1554,14 @@
       <c r="H9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="63">
+      <c r="I9" s="62">
         <v>46218</v>
       </c>
-      <c r="J9" s="63"/>
+      <c r="J9" s="62"/>
       <c r="K9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="62"/>
+      <c r="A10" s="67"/>
       <c r="B10" s="36" t="s">
         <v>13</v>
       </c>
@@ -1579,12 +1579,12 @@
       <c r="H10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="62"/>
-      <c r="J10" s="64"/>
+      <c r="I10" s="67"/>
+      <c r="J10" s="63"/>
       <c r="K10" s="49"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="66" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="42" t="s">
@@ -1604,14 +1604,14 @@
       <c r="H11" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="63">
+      <c r="I11" s="62">
         <v>46171</v>
       </c>
-      <c r="J11" s="63"/>
+      <c r="J11" s="62"/>
       <c r="K11" s="50"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="62"/>
+      <c r="A12" s="67"/>
       <c r="B12" s="45" t="s">
         <v>13</v>
       </c>
@@ -1629,12 +1629,12 @@
       <c r="H12" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="62"/>
-      <c r="J12" s="64"/>
+      <c r="I12" s="67"/>
+      <c r="J12" s="63"/>
       <c r="K12" s="49"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="61" t="s">
+      <c r="A13" s="66" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="39" t="s">
@@ -1654,14 +1654,14 @@
       <c r="H13" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="63" t="s">
+      <c r="I13" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="63"/>
+      <c r="J13" s="62"/>
       <c r="K13" s="50"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="62"/>
+      <c r="A14" s="67"/>
       <c r="B14" s="36" t="s">
         <v>13</v>
       </c>
@@ -1679,12 +1679,12 @@
       <c r="H14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="62"/>
-      <c r="J14" s="64"/>
+      <c r="I14" s="67"/>
+      <c r="J14" s="63"/>
       <c r="K14" s="49"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="61" t="s">
+      <c r="A15" s="66" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="42" t="s">
@@ -1704,14 +1704,14 @@
       <c r="H15" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="63">
+      <c r="I15" s="62">
         <v>46199</v>
       </c>
-      <c r="J15" s="63"/>
+      <c r="J15" s="62"/>
       <c r="K15" s="50"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="62"/>
+      <c r="A16" s="67"/>
       <c r="B16" s="45" t="s">
         <v>13</v>
       </c>
@@ -1729,12 +1729,12 @@
       <c r="H16" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="62"/>
-      <c r="J16" s="64"/>
+      <c r="I16" s="67"/>
+      <c r="J16" s="63"/>
       <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="67" t="s">
+      <c r="A17" s="68" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="33" t="s">
@@ -1754,14 +1754,14 @@
       <c r="H17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="66">
+      <c r="I17" s="65">
         <v>46305</v>
       </c>
-      <c r="J17" s="66"/>
+      <c r="J17" s="65"/>
       <c r="K17" s="51"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="62"/>
+      <c r="A18" s="67"/>
       <c r="B18" s="36" t="s">
         <v>13</v>
       </c>
@@ -1779,12 +1779,12 @@
       <c r="H18" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="62"/>
-      <c r="J18" s="64"/>
+      <c r="I18" s="67"/>
+      <c r="J18" s="63"/>
       <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="67" t="s">
+      <c r="A19" s="68" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="33" t="s">
@@ -1804,14 +1804,14 @@
       <c r="H19" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="66">
+      <c r="I19" s="65">
         <v>46336</v>
       </c>
-      <c r="J19" s="66"/>
+      <c r="J19" s="65"/>
       <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="62"/>
+      <c r="A20" s="67"/>
       <c r="B20" s="36" t="s">
         <v>13</v>
       </c>
@@ -1829,12 +1829,12 @@
       <c r="H20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="62"/>
-      <c r="J20" s="64"/>
+      <c r="I20" s="67"/>
+      <c r="J20" s="63"/>
       <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="61" t="s">
+      <c r="A21" s="66" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="39" t="s">
@@ -1854,14 +1854,14 @@
       <c r="H21" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="63">
+      <c r="I21" s="62">
         <v>46336</v>
       </c>
-      <c r="J21" s="63"/>
+      <c r="J21" s="62"/>
       <c r="K21" s="52"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="62"/>
+      <c r="A22" s="67"/>
       <c r="B22" s="36" t="s">
         <v>13</v>
       </c>
@@ -1879,12 +1879,12 @@
       <c r="H22" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="62"/>
-      <c r="J22" s="64"/>
+      <c r="I22" s="67"/>
+      <c r="J22" s="63"/>
       <c r="K22" s="53"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="61" t="s">
+      <c r="A23" s="66" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="42" t="s">
@@ -1904,14 +1904,14 @@
       <c r="H23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="63">
+      <c r="I23" s="62">
         <v>46237</v>
       </c>
-      <c r="J23" s="63"/>
+      <c r="J23" s="62"/>
       <c r="K23" s="52"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="62"/>
+      <c r="A24" s="67"/>
       <c r="B24" s="45" t="s">
         <v>13</v>
       </c>
@@ -1929,12 +1929,12 @@
       <c r="H24" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="62"/>
-      <c r="J24" s="64"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="63"/>
       <c r="K24" s="53"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="61" t="s">
+      <c r="A25" s="66" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="42" t="s">
@@ -1954,14 +1954,14 @@
       <c r="H25" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="63">
+      <c r="I25" s="62">
         <v>46188</v>
       </c>
-      <c r="J25" s="63"/>
+      <c r="J25" s="62"/>
       <c r="K25" s="52"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="62"/>
+      <c r="A26" s="67"/>
       <c r="B26" s="45" t="s">
         <v>13</v>
       </c>
@@ -1979,12 +1979,12 @@
       <c r="H26" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="62"/>
-      <c r="J26" s="64"/>
+      <c r="I26" s="67"/>
+      <c r="J26" s="63"/>
       <c r="K26" s="53"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="61" t="s">
+      <c r="A27" s="66" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="39" t="s">
@@ -2004,14 +2004,14 @@
       <c r="H27" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="63">
+      <c r="I27" s="62">
         <v>46321</v>
       </c>
-      <c r="J27" s="63"/>
+      <c r="J27" s="62"/>
       <c r="K27" s="52"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="62"/>
+      <c r="A28" s="67"/>
       <c r="B28" s="36" t="s">
         <v>13</v>
       </c>
@@ -2029,12 +2029,12 @@
       <c r="H28" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="62"/>
-      <c r="J28" s="64"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="63"/>
       <c r="K28" s="53"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="61" t="s">
+      <c r="A29" s="66" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="42" t="s">
@@ -2054,14 +2054,14 @@
       <c r="H29" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="63">
+      <c r="I29" s="62">
         <v>46139</v>
       </c>
-      <c r="J29" s="63"/>
+      <c r="J29" s="62"/>
       <c r="K29" s="52"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="62"/>
+      <c r="A30" s="67"/>
       <c r="B30" s="45" t="s">
         <v>13</v>
       </c>
@@ -2079,12 +2079,12 @@
       <c r="H30" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="62"/>
-      <c r="J30" s="64"/>
+      <c r="I30" s="67"/>
+      <c r="J30" s="63"/>
       <c r="K30" s="53"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="66" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="42" t="s">
@@ -2104,14 +2104,14 @@
       <c r="H31" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="63">
+      <c r="I31" s="62">
         <v>46133</v>
       </c>
-      <c r="J31" s="63"/>
+      <c r="J31" s="62"/>
       <c r="K31" s="52"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="62"/>
+      <c r="A32" s="67"/>
       <c r="B32" s="45" t="s">
         <v>13</v>
       </c>
@@ -2129,12 +2129,12 @@
       <c r="H32" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="62"/>
-      <c r="J32" s="64"/>
+      <c r="I32" s="67"/>
+      <c r="J32" s="63"/>
       <c r="K32" s="53"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="61" t="s">
+      <c r="A33" s="66" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="39" t="s">
@@ -2154,14 +2154,14 @@
       <c r="H33" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="63">
+      <c r="I33" s="62">
         <v>46295</v>
       </c>
-      <c r="J33" s="63"/>
+      <c r="J33" s="62"/>
       <c r="K33" s="52"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="62"/>
+      <c r="A34" s="67"/>
       <c r="B34" s="36" t="s">
         <v>13</v>
       </c>
@@ -2179,12 +2179,12 @@
       <c r="H34" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="62"/>
-      <c r="J34" s="64"/>
+      <c r="I34" s="67"/>
+      <c r="J34" s="63"/>
       <c r="K34" s="53"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="61" t="s">
+      <c r="A35" s="66" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="39" t="s">
@@ -2204,14 +2204,14 @@
       <c r="H35" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="63">
+      <c r="I35" s="62">
         <v>45884</v>
       </c>
-      <c r="J35" s="63"/>
+      <c r="J35" s="62"/>
       <c r="K35" s="52"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="62"/>
+      <c r="A36" s="67"/>
       <c r="B36" s="36" t="s">
         <v>13</v>
       </c>
@@ -2229,12 +2229,12 @@
       <c r="H36" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="62"/>
-      <c r="J36" s="64"/>
+      <c r="I36" s="67"/>
+      <c r="J36" s="63"/>
       <c r="K36" s="53"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="61" t="s">
+      <c r="A37" s="66" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="39" t="s">
@@ -2254,14 +2254,14 @@
       <c r="H37" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="63">
+      <c r="I37" s="62">
         <v>45915</v>
       </c>
-      <c r="J37" s="63"/>
+      <c r="J37" s="62"/>
       <c r="K37" s="52"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="62"/>
+      <c r="A38" s="67"/>
       <c r="B38" s="36" t="s">
         <v>13</v>
       </c>
@@ -2279,12 +2279,12 @@
       <c r="H38" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="62"/>
-      <c r="J38" s="64"/>
+      <c r="I38" s="67"/>
+      <c r="J38" s="63"/>
       <c r="K38" s="53"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="61" t="s">
+      <c r="A39" s="66" t="s">
         <v>131</v>
       </c>
       <c r="B39" s="39" t="s">
@@ -2300,12 +2300,12 @@
       <c r="H39" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I39" s="63"/>
-      <c r="J39" s="63"/>
+      <c r="I39" s="62"/>
+      <c r="J39" s="62"/>
       <c r="K39" s="52"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="62"/>
+      <c r="A40" s="67"/>
       <c r="B40" s="56" t="s">
         <v>13</v>
       </c>
@@ -2319,12 +2319,12 @@
       <c r="H40" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="62"/>
-      <c r="J40" s="64"/>
+      <c r="I40" s="67"/>
+      <c r="J40" s="63"/>
       <c r="K40" s="53"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="61" t="s">
+      <c r="A41" s="66" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="39" t="s">
@@ -2344,14 +2344,14 @@
       <c r="H41" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="63">
+      <c r="I41" s="62">
         <v>46230</v>
       </c>
-      <c r="J41" s="63"/>
+      <c r="J41" s="62"/>
       <c r="K41" s="52"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="62"/>
+      <c r="A42" s="67"/>
       <c r="B42" s="56" t="s">
         <v>13</v>
       </c>
@@ -2361,26 +2361,41 @@
       <c r="F42" s="57"/>
       <c r="G42" s="58"/>
       <c r="H42" s="56"/>
-      <c r="I42" s="62"/>
-      <c r="J42" s="64"/>
+      <c r="I42" s="67"/>
+      <c r="J42" s="63"/>
       <c r="K42" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2397,35 +2412,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2461,56 +2461,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
-      <c r="P1" s="59"/>
-      <c r="Q1" s="59"/>
-      <c r="R1" s="59"/>
-      <c r="S1" s="59"/>
-      <c r="T1" s="59"/>
-      <c r="U1" s="59"/>
-      <c r="V1" s="59"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="60"/>
-      <c r="P2" s="60"/>
-      <c r="Q2" s="60"/>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60"/>
-      <c r="U2" s="60"/>
-      <c r="V2" s="60"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="71"/>
+      <c r="Q2" s="71"/>
+      <c r="R2" s="71"/>
+      <c r="S2" s="71"/>
+      <c r="T2" s="71"/>
+      <c r="U2" s="71"/>
+      <c r="V2" s="71"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -4190,20 +4190,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="69" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="71" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4596,22 +4596,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="71" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5774,15 +5774,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5793,6 +5784,15 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5815,14 +5815,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5831,4 +5823,12 @@
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 13:28)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFD760CD-EEE6-4E9E-ACC2-376EC4F5F17F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="135">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -444,6 +444,9 @@
   </si>
   <si>
     <t>ทำราคาขั้นต่ำ ในกรณีงานเล็กเป็นงานเหมา</t>
+  </si>
+  <si>
+    <t>Data Actual  Plan</t>
   </si>
 </sst>
 </file>
@@ -456,7 +459,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,6 +559,12 @@
       <family val="2"/>
       <charset val="222"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -775,7 +784,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -972,6 +981,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2140,10 +2155,10 @@
       <c r="B33" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="40">
+      <c r="C33" s="73">
         <v>46091</v>
       </c>
-      <c r="D33" s="40">
+      <c r="D33" s="73">
         <v>46094</v>
       </c>
       <c r="E33" s="40"/>
@@ -2165,10 +2180,10 @@
       <c r="B34" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="37">
+      <c r="C34" s="74">
         <v>46091</v>
       </c>
-      <c r="D34" s="37">
+      <c r="D34" s="74">
         <v>46094</v>
       </c>
       <c r="E34" s="37"/>
@@ -2269,7 +2284,7 @@
         <v>45729</v>
       </c>
       <c r="D38" s="37">
-        <v>45732</v>
+        <v>45862</v>
       </c>
       <c r="E38" s="37"/>
       <c r="F38" s="37"/>
@@ -2433,6 +2448,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4699,10 +4715,19 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="6"/>
+      <c r="A9" s="3" t="s">
+        <v>134</v>
+      </c>
       <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="C9" s="6">
+        <v>46217</v>
+      </c>
+      <c r="D9" s="6">
+        <v>46224</v>
+      </c>
+      <c r="E9" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="6"/>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 13:41)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFD760CD-EEE6-4E9E-ACC2-376EC4F5F17F}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA7C2CBC-69B9-4AA1-9D0F-52034DD4022A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -459,7 +459,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -559,12 +559,6 @@
       <family val="2"/>
       <charset val="222"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10.5"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -957,36 +951,36 @@
     <xf numFmtId="9" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1384,34 +1378,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1449,7 +1443,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="73" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="59" t="s">
@@ -1469,14 +1463,14 @@
       <c r="H5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="64">
+      <c r="I5" s="74">
         <v>46213</v>
       </c>
-      <c r="J5" s="64"/>
+      <c r="J5" s="74"/>
       <c r="K5" s="48"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="67"/>
+      <c r="A6" s="65"/>
       <c r="B6" s="45" t="s">
         <v>13</v>
       </c>
@@ -1494,12 +1488,12 @@
       <c r="H6" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="67"/>
-      <c r="J6" s="63"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="67"/>
       <c r="K6" s="49"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="66" t="s">
+      <c r="A7" s="64" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="39" t="s">
@@ -1519,14 +1513,14 @@
       <c r="H7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="62" t="s">
+      <c r="I7" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="62"/>
+      <c r="J7" s="66"/>
       <c r="K7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="67"/>
+      <c r="A8" s="65"/>
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1544,12 +1538,12 @@
       <c r="H8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="67"/>
-      <c r="J8" s="63"/>
+      <c r="I8" s="65"/>
+      <c r="J8" s="67"/>
       <c r="K8" s="49"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="66" t="s">
+      <c r="A9" s="64" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="39" t="s">
@@ -1569,14 +1563,14 @@
       <c r="H9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="66">
         <v>46218</v>
       </c>
-      <c r="J9" s="62"/>
+      <c r="J9" s="66"/>
       <c r="K9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="67"/>
+      <c r="A10" s="65"/>
       <c r="B10" s="36" t="s">
         <v>13</v>
       </c>
@@ -1594,12 +1588,12 @@
       <c r="H10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="67"/>
-      <c r="J10" s="63"/>
+      <c r="I10" s="65"/>
+      <c r="J10" s="67"/>
       <c r="K10" s="49"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="64" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="42" t="s">
@@ -1619,14 +1613,14 @@
       <c r="H11" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="62">
+      <c r="I11" s="66">
         <v>46171</v>
       </c>
-      <c r="J11" s="62"/>
+      <c r="J11" s="66"/>
       <c r="K11" s="50"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="67"/>
+      <c r="A12" s="65"/>
       <c r="B12" s="45" t="s">
         <v>13</v>
       </c>
@@ -1644,12 +1638,12 @@
       <c r="H12" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="67"/>
-      <c r="J12" s="63"/>
+      <c r="I12" s="65"/>
+      <c r="J12" s="67"/>
       <c r="K12" s="49"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="66" t="s">
+      <c r="A13" s="64" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="39" t="s">
@@ -1669,14 +1663,14 @@
       <c r="H13" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="62" t="s">
+      <c r="I13" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="62"/>
+      <c r="J13" s="66"/>
       <c r="K13" s="50"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="67"/>
+      <c r="A14" s="65"/>
       <c r="B14" s="36" t="s">
         <v>13</v>
       </c>
@@ -1694,12 +1688,12 @@
       <c r="H14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="67"/>
-      <c r="J14" s="63"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="67"/>
       <c r="K14" s="49"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="66" t="s">
+      <c r="A15" s="64" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="42" t="s">
@@ -1719,14 +1713,14 @@
       <c r="H15" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="62">
+      <c r="I15" s="66">
         <v>46199</v>
       </c>
-      <c r="J15" s="62"/>
+      <c r="J15" s="66"/>
       <c r="K15" s="50"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="67"/>
+      <c r="A16" s="65"/>
       <c r="B16" s="45" t="s">
         <v>13</v>
       </c>
@@ -1744,12 +1738,12 @@
       <c r="H16" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="67"/>
-      <c r="J16" s="63"/>
+      <c r="I16" s="65"/>
+      <c r="J16" s="67"/>
       <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="68" t="s">
+      <c r="A17" s="71" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="33" t="s">
@@ -1769,14 +1763,14 @@
       <c r="H17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="65">
+      <c r="I17" s="70">
         <v>46305</v>
       </c>
-      <c r="J17" s="65"/>
+      <c r="J17" s="70"/>
       <c r="K17" s="51"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="67"/>
+      <c r="A18" s="65"/>
       <c r="B18" s="36" t="s">
         <v>13</v>
       </c>
@@ -1794,12 +1788,12 @@
       <c r="H18" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="67"/>
-      <c r="J18" s="63"/>
+      <c r="I18" s="65"/>
+      <c r="J18" s="67"/>
       <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="71" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="33" t="s">
@@ -1819,14 +1813,14 @@
       <c r="H19" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="65">
+      <c r="I19" s="70">
         <v>46336</v>
       </c>
-      <c r="J19" s="65"/>
+      <c r="J19" s="70"/>
       <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="67"/>
+      <c r="A20" s="65"/>
       <c r="B20" s="36" t="s">
         <v>13</v>
       </c>
@@ -1844,12 +1838,12 @@
       <c r="H20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="67"/>
-      <c r="J20" s="63"/>
+      <c r="I20" s="65"/>
+      <c r="J20" s="67"/>
       <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="64" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="39" t="s">
@@ -1869,14 +1863,14 @@
       <c r="H21" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="62">
+      <c r="I21" s="66">
         <v>46336</v>
       </c>
-      <c r="J21" s="62"/>
+      <c r="J21" s="66"/>
       <c r="K21" s="52"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="67"/>
+      <c r="A22" s="65"/>
       <c r="B22" s="36" t="s">
         <v>13</v>
       </c>
@@ -1894,12 +1888,12 @@
       <c r="H22" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="67"/>
-      <c r="J22" s="63"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="67"/>
       <c r="K22" s="53"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="64" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="42" t="s">
@@ -1919,14 +1913,14 @@
       <c r="H23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="62">
+      <c r="I23" s="66">
         <v>46237</v>
       </c>
-      <c r="J23" s="62"/>
+      <c r="J23" s="66"/>
       <c r="K23" s="52"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="67"/>
+      <c r="A24" s="65"/>
       <c r="B24" s="45" t="s">
         <v>13</v>
       </c>
@@ -1944,12 +1938,12 @@
       <c r="H24" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="67"/>
-      <c r="J24" s="63"/>
+      <c r="I24" s="65"/>
+      <c r="J24" s="67"/>
       <c r="K24" s="53"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="66" t="s">
+      <c r="A25" s="64" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="42" t="s">
@@ -1969,14 +1963,14 @@
       <c r="H25" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="62">
+      <c r="I25" s="66">
         <v>46188</v>
       </c>
-      <c r="J25" s="62"/>
+      <c r="J25" s="66"/>
       <c r="K25" s="52"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="67"/>
+      <c r="A26" s="65"/>
       <c r="B26" s="45" t="s">
         <v>13</v>
       </c>
@@ -1994,12 +1988,12 @@
       <c r="H26" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="67"/>
-      <c r="J26" s="63"/>
+      <c r="I26" s="65"/>
+      <c r="J26" s="67"/>
       <c r="K26" s="53"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="64" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="39" t="s">
@@ -2019,14 +2013,14 @@
       <c r="H27" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="62">
+      <c r="I27" s="66">
         <v>46321</v>
       </c>
-      <c r="J27" s="62"/>
+      <c r="J27" s="66"/>
       <c r="K27" s="52"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="67"/>
+      <c r="A28" s="65"/>
       <c r="B28" s="36" t="s">
         <v>13</v>
       </c>
@@ -2044,12 +2038,12 @@
       <c r="H28" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="67"/>
-      <c r="J28" s="63"/>
+      <c r="I28" s="65"/>
+      <c r="J28" s="67"/>
       <c r="K28" s="53"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="66" t="s">
+      <c r="A29" s="64" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="42" t="s">
@@ -2069,14 +2063,14 @@
       <c r="H29" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="62">
+      <c r="I29" s="66">
         <v>46139</v>
       </c>
-      <c r="J29" s="62"/>
+      <c r="J29" s="66"/>
       <c r="K29" s="52"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="67"/>
+      <c r="A30" s="65"/>
       <c r="B30" s="45" t="s">
         <v>13</v>
       </c>
@@ -2094,12 +2088,12 @@
       <c r="H30" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="67"/>
-      <c r="J30" s="63"/>
+      <c r="I30" s="65"/>
+      <c r="J30" s="67"/>
       <c r="K30" s="53"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="66" t="s">
+      <c r="A31" s="64" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="42" t="s">
@@ -2119,14 +2113,14 @@
       <c r="H31" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="62">
+      <c r="I31" s="66">
         <v>46133</v>
       </c>
-      <c r="J31" s="62"/>
+      <c r="J31" s="66"/>
       <c r="K31" s="52"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="67"/>
+      <c r="A32" s="65"/>
       <c r="B32" s="45" t="s">
         <v>13</v>
       </c>
@@ -2144,22 +2138,22 @@
       <c r="H32" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="67"/>
-      <c r="J32" s="63"/>
+      <c r="I32" s="65"/>
+      <c r="J32" s="67"/>
       <c r="K32" s="53"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="66" t="s">
+      <c r="A33" s="64" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="73">
-        <v>46091</v>
-      </c>
-      <c r="D33" s="73">
-        <v>46094</v>
+      <c r="C33" s="62">
+        <v>46237</v>
+      </c>
+      <c r="D33" s="62">
+        <v>46248</v>
       </c>
       <c r="E33" s="40"/>
       <c r="F33" s="40"/>
@@ -2169,22 +2163,22 @@
       <c r="H33" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="62">
+      <c r="I33" s="66">
         <v>46295</v>
       </c>
-      <c r="J33" s="62"/>
+      <c r="J33" s="66"/>
       <c r="K33" s="52"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="67"/>
+      <c r="A34" s="65"/>
       <c r="B34" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="74">
-        <v>46091</v>
-      </c>
-      <c r="D34" s="74">
-        <v>46094</v>
+      <c r="C34" s="63">
+        <v>46296</v>
+      </c>
+      <c r="D34" s="63">
+        <v>46303</v>
       </c>
       <c r="E34" s="37"/>
       <c r="F34" s="37"/>
@@ -2194,12 +2188,12 @@
       <c r="H34" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="67"/>
-      <c r="J34" s="63"/>
+      <c r="I34" s="65"/>
+      <c r="J34" s="67"/>
       <c r="K34" s="53"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="66" t="s">
+      <c r="A35" s="64" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="39" t="s">
@@ -2219,14 +2213,14 @@
       <c r="H35" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="62">
+      <c r="I35" s="66">
         <v>45884</v>
       </c>
-      <c r="J35" s="62"/>
+      <c r="J35" s="66"/>
       <c r="K35" s="52"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="67"/>
+      <c r="A36" s="65"/>
       <c r="B36" s="36" t="s">
         <v>13</v>
       </c>
@@ -2244,12 +2238,12 @@
       <c r="H36" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="67"/>
-      <c r="J36" s="63"/>
+      <c r="I36" s="65"/>
+      <c r="J36" s="67"/>
       <c r="K36" s="53"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="66" t="s">
+      <c r="A37" s="64" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="39" t="s">
@@ -2269,14 +2263,14 @@
       <c r="H37" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="62">
+      <c r="I37" s="66">
         <v>45915</v>
       </c>
-      <c r="J37" s="62"/>
+      <c r="J37" s="66"/>
       <c r="K37" s="52"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="67"/>
+      <c r="A38" s="65"/>
       <c r="B38" s="36" t="s">
         <v>13</v>
       </c>
@@ -2294,12 +2288,12 @@
       <c r="H38" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="67"/>
-      <c r="J38" s="63"/>
+      <c r="I38" s="65"/>
+      <c r="J38" s="67"/>
       <c r="K38" s="53"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="66" t="s">
+      <c r="A39" s="64" t="s">
         <v>131</v>
       </c>
       <c r="B39" s="39" t="s">
@@ -2315,12 +2309,12 @@
       <c r="H39" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I39" s="62"/>
-      <c r="J39" s="62"/>
+      <c r="I39" s="66"/>
+      <c r="J39" s="66"/>
       <c r="K39" s="52"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="67"/>
+      <c r="A40" s="65"/>
       <c r="B40" s="56" t="s">
         <v>13</v>
       </c>
@@ -2334,12 +2328,12 @@
       <c r="H40" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="67"/>
-      <c r="J40" s="63"/>
+      <c r="I40" s="65"/>
+      <c r="J40" s="67"/>
       <c r="K40" s="53"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="66" t="s">
+      <c r="A41" s="64" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="39" t="s">
@@ -2359,14 +2353,14 @@
       <c r="H41" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="62">
+      <c r="I41" s="66">
         <v>46230</v>
       </c>
-      <c r="J41" s="62"/>
+      <c r="J41" s="66"/>
       <c r="K41" s="52"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="67"/>
+      <c r="A42" s="65"/>
       <c r="B42" s="56" t="s">
         <v>13</v>
       </c>
@@ -2376,18 +2370,49 @@
       <c r="F42" s="57"/>
       <c r="G42" s="58"/>
       <c r="H42" s="56"/>
-      <c r="I42" s="67"/>
-      <c r="J42" s="63"/>
+      <c r="I42" s="65"/>
+      <c r="J42" s="67"/>
       <c r="K42" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2404,43 +2429,12 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2477,56 +2471,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69"/>
-      <c r="U1" s="69"/>
-      <c r="V1" s="69"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="68"/>
+      <c r="U1" s="68"/>
+      <c r="V1" s="68"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="71"/>
-      <c r="R2" s="71"/>
-      <c r="S2" s="71"/>
-      <c r="T2" s="71"/>
-      <c r="U2" s="71"/>
-      <c r="V2" s="71"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
+      <c r="N2" s="72"/>
+      <c r="O2" s="72"/>
+      <c r="P2" s="72"/>
+      <c r="Q2" s="72"/>
+      <c r="R2" s="72"/>
+      <c r="S2" s="72"/>
+      <c r="T2" s="72"/>
+      <c r="U2" s="72"/>
+      <c r="V2" s="72"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -3447,7 +3441,7 @@
       </c>
       <c r="Q19" s="19">
         <f>'Master Schedule'!C33</f>
-        <v>46091</v>
+        <v>46237</v>
       </c>
       <c r="R19" s="11">
         <v>46295</v>
@@ -4206,20 +4200,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4612,22 +4606,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5799,6 +5793,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5809,15 +5812,6 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5840,6 +5834,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5848,12 +5850,4 @@
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 14:27)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA7C2CBC-69B9-4AA1-9D0F-52034DD4022A}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17342736-9A5A-4BE9-A360-14E602BF2838}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="324" yWindow="108" windowWidth="14988" windowHeight="11484" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -957,30 +957,30 @@
     <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1378,34 +1378,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1443,7 +1443,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="74" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="59" t="s">
@@ -1463,14 +1463,14 @@
       <c r="H5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="74">
-        <v>46213</v>
-      </c>
-      <c r="J5" s="74"/>
+      <c r="I5" s="66">
+        <v>46244</v>
+      </c>
+      <c r="J5" s="66"/>
       <c r="K5" s="48"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="65"/>
+      <c r="A6" s="69"/>
       <c r="B6" s="45" t="s">
         <v>13</v>
       </c>
@@ -1488,12 +1488,12 @@
       <c r="H6" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="65"/>
-      <c r="J6" s="67"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="65"/>
       <c r="K6" s="49"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="68" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="39" t="s">
@@ -1513,14 +1513,14 @@
       <c r="H7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="66" t="s">
+      <c r="I7" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="66"/>
+      <c r="J7" s="64"/>
       <c r="K7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="65"/>
+      <c r="A8" s="69"/>
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1538,12 +1538,12 @@
       <c r="H8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="65"/>
-      <c r="J8" s="67"/>
+      <c r="I8" s="69"/>
+      <c r="J8" s="65"/>
       <c r="K8" s="49"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="68" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="39" t="s">
@@ -1563,14 +1563,14 @@
       <c r="H9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="66">
+      <c r="I9" s="64">
         <v>46218</v>
       </c>
-      <c r="J9" s="66"/>
+      <c r="J9" s="64"/>
       <c r="K9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="65"/>
+      <c r="A10" s="69"/>
       <c r="B10" s="36" t="s">
         <v>13</v>
       </c>
@@ -1588,12 +1588,12 @@
       <c r="H10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="65"/>
-      <c r="J10" s="67"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="65"/>
       <c r="K10" s="49"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="68" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="42" t="s">
@@ -1613,14 +1613,14 @@
       <c r="H11" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="66">
+      <c r="I11" s="64">
         <v>46171</v>
       </c>
-      <c r="J11" s="66"/>
+      <c r="J11" s="64"/>
       <c r="K11" s="50"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="65"/>
+      <c r="A12" s="69"/>
       <c r="B12" s="45" t="s">
         <v>13</v>
       </c>
@@ -1638,12 +1638,12 @@
       <c r="H12" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="65"/>
-      <c r="J12" s="67"/>
+      <c r="I12" s="69"/>
+      <c r="J12" s="65"/>
       <c r="K12" s="49"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="68" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="39" t="s">
@@ -1663,14 +1663,14 @@
       <c r="H13" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="66" t="s">
+      <c r="I13" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="66"/>
+      <c r="J13" s="64"/>
       <c r="K13" s="50"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="65"/>
+      <c r="A14" s="69"/>
       <c r="B14" s="36" t="s">
         <v>13</v>
       </c>
@@ -1688,12 +1688,12 @@
       <c r="H14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="65"/>
-      <c r="J14" s="67"/>
+      <c r="I14" s="69"/>
+      <c r="J14" s="65"/>
       <c r="K14" s="49"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="64" t="s">
+      <c r="A15" s="68" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="42" t="s">
@@ -1713,14 +1713,14 @@
       <c r="H15" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="66">
+      <c r="I15" s="64">
         <v>46199</v>
       </c>
-      <c r="J15" s="66"/>
+      <c r="J15" s="64"/>
       <c r="K15" s="50"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="65"/>
+      <c r="A16" s="69"/>
       <c r="B16" s="45" t="s">
         <v>13</v>
       </c>
@@ -1738,12 +1738,12 @@
       <c r="H16" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="65"/>
-      <c r="J16" s="67"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="65"/>
       <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="71" t="s">
+      <c r="A17" s="70" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="33" t="s">
@@ -1763,14 +1763,14 @@
       <c r="H17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="70">
+      <c r="I17" s="67">
         <v>46305</v>
       </c>
-      <c r="J17" s="70"/>
+      <c r="J17" s="67"/>
       <c r="K17" s="51"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="65"/>
+      <c r="A18" s="69"/>
       <c r="B18" s="36" t="s">
         <v>13</v>
       </c>
@@ -1788,12 +1788,12 @@
       <c r="H18" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="65"/>
-      <c r="J18" s="67"/>
+      <c r="I18" s="69"/>
+      <c r="J18" s="65"/>
       <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="71" t="s">
+      <c r="A19" s="70" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="33" t="s">
@@ -1813,14 +1813,14 @@
       <c r="H19" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="70">
+      <c r="I19" s="67">
         <v>46336</v>
       </c>
-      <c r="J19" s="70"/>
+      <c r="J19" s="67"/>
       <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="65"/>
+      <c r="A20" s="69"/>
       <c r="B20" s="36" t="s">
         <v>13</v>
       </c>
@@ -1838,12 +1838,12 @@
       <c r="H20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="65"/>
-      <c r="J20" s="67"/>
+      <c r="I20" s="69"/>
+      <c r="J20" s="65"/>
       <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="64" t="s">
+      <c r="A21" s="68" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="39" t="s">
@@ -1863,14 +1863,14 @@
       <c r="H21" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="66">
+      <c r="I21" s="64">
         <v>46336</v>
       </c>
-      <c r="J21" s="66"/>
+      <c r="J21" s="64"/>
       <c r="K21" s="52"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="65"/>
+      <c r="A22" s="69"/>
       <c r="B22" s="36" t="s">
         <v>13</v>
       </c>
@@ -1888,12 +1888,12 @@
       <c r="H22" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="65"/>
-      <c r="J22" s="67"/>
+      <c r="I22" s="69"/>
+      <c r="J22" s="65"/>
       <c r="K22" s="53"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="64" t="s">
+      <c r="A23" s="68" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="42" t="s">
@@ -1913,14 +1913,14 @@
       <c r="H23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="66">
+      <c r="I23" s="64">
         <v>46237</v>
       </c>
-      <c r="J23" s="66"/>
+      <c r="J23" s="64"/>
       <c r="K23" s="52"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="65"/>
+      <c r="A24" s="69"/>
       <c r="B24" s="45" t="s">
         <v>13</v>
       </c>
@@ -1938,12 +1938,12 @@
       <c r="H24" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="65"/>
-      <c r="J24" s="67"/>
+      <c r="I24" s="69"/>
+      <c r="J24" s="65"/>
       <c r="K24" s="53"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="64" t="s">
+      <c r="A25" s="68" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="42" t="s">
@@ -1963,14 +1963,14 @@
       <c r="H25" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="66">
+      <c r="I25" s="64">
         <v>46188</v>
       </c>
-      <c r="J25" s="66"/>
+      <c r="J25" s="64"/>
       <c r="K25" s="52"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="65"/>
+      <c r="A26" s="69"/>
       <c r="B26" s="45" t="s">
         <v>13</v>
       </c>
@@ -1988,12 +1988,12 @@
       <c r="H26" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="65"/>
-      <c r="J26" s="67"/>
+      <c r="I26" s="69"/>
+      <c r="J26" s="65"/>
       <c r="K26" s="53"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="64" t="s">
+      <c r="A27" s="68" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="39" t="s">
@@ -2013,14 +2013,14 @@
       <c r="H27" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="66">
+      <c r="I27" s="64">
         <v>46321</v>
       </c>
-      <c r="J27" s="66"/>
+      <c r="J27" s="64"/>
       <c r="K27" s="52"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="65"/>
+      <c r="A28" s="69"/>
       <c r="B28" s="36" t="s">
         <v>13</v>
       </c>
@@ -2038,12 +2038,12 @@
       <c r="H28" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="65"/>
-      <c r="J28" s="67"/>
+      <c r="I28" s="69"/>
+      <c r="J28" s="65"/>
       <c r="K28" s="53"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="64" t="s">
+      <c r="A29" s="68" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="42" t="s">
@@ -2063,14 +2063,14 @@
       <c r="H29" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="66">
+      <c r="I29" s="64">
         <v>46139</v>
       </c>
-      <c r="J29" s="66"/>
+      <c r="J29" s="64"/>
       <c r="K29" s="52"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="65"/>
+      <c r="A30" s="69"/>
       <c r="B30" s="45" t="s">
         <v>13</v>
       </c>
@@ -2088,12 +2088,12 @@
       <c r="H30" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="65"/>
-      <c r="J30" s="67"/>
+      <c r="I30" s="69"/>
+      <c r="J30" s="65"/>
       <c r="K30" s="53"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="64" t="s">
+      <c r="A31" s="68" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="42" t="s">
@@ -2113,14 +2113,14 @@
       <c r="H31" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="66">
+      <c r="I31" s="64">
         <v>46133</v>
       </c>
-      <c r="J31" s="66"/>
+      <c r="J31" s="64"/>
       <c r="K31" s="52"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="65"/>
+      <c r="A32" s="69"/>
       <c r="B32" s="45" t="s">
         <v>13</v>
       </c>
@@ -2138,12 +2138,12 @@
       <c r="H32" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="65"/>
-      <c r="J32" s="67"/>
+      <c r="I32" s="69"/>
+      <c r="J32" s="65"/>
       <c r="K32" s="53"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="64" t="s">
+      <c r="A33" s="68" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="39" t="s">
@@ -2163,14 +2163,14 @@
       <c r="H33" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="66">
+      <c r="I33" s="64">
         <v>46295</v>
       </c>
-      <c r="J33" s="66"/>
+      <c r="J33" s="64"/>
       <c r="K33" s="52"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="65"/>
+      <c r="A34" s="69"/>
       <c r="B34" s="36" t="s">
         <v>13</v>
       </c>
@@ -2188,12 +2188,12 @@
       <c r="H34" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="65"/>
-      <c r="J34" s="67"/>
+      <c r="I34" s="69"/>
+      <c r="J34" s="65"/>
       <c r="K34" s="53"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="64" t="s">
+      <c r="A35" s="68" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="39" t="s">
@@ -2213,14 +2213,14 @@
       <c r="H35" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="66">
+      <c r="I35" s="64">
         <v>45884</v>
       </c>
-      <c r="J35" s="66"/>
+      <c r="J35" s="64"/>
       <c r="K35" s="52"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="65"/>
+      <c r="A36" s="69"/>
       <c r="B36" s="36" t="s">
         <v>13</v>
       </c>
@@ -2238,12 +2238,12 @@
       <c r="H36" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="65"/>
-      <c r="J36" s="67"/>
+      <c r="I36" s="69"/>
+      <c r="J36" s="65"/>
       <c r="K36" s="53"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="64" t="s">
+      <c r="A37" s="68" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="39" t="s">
@@ -2263,14 +2263,14 @@
       <c r="H37" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="66">
+      <c r="I37" s="64">
         <v>45915</v>
       </c>
-      <c r="J37" s="66"/>
+      <c r="J37" s="64"/>
       <c r="K37" s="52"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="65"/>
+      <c r="A38" s="69"/>
       <c r="B38" s="36" t="s">
         <v>13</v>
       </c>
@@ -2288,12 +2288,12 @@
       <c r="H38" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="65"/>
-      <c r="J38" s="67"/>
+      <c r="I38" s="69"/>
+      <c r="J38" s="65"/>
       <c r="K38" s="53"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="64" t="s">
+      <c r="A39" s="68" t="s">
         <v>131</v>
       </c>
       <c r="B39" s="39" t="s">
@@ -2309,12 +2309,12 @@
       <c r="H39" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I39" s="66"/>
-      <c r="J39" s="66"/>
+      <c r="I39" s="64"/>
+      <c r="J39" s="64"/>
       <c r="K39" s="52"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="65"/>
+      <c r="A40" s="69"/>
       <c r="B40" s="56" t="s">
         <v>13</v>
       </c>
@@ -2328,12 +2328,12 @@
       <c r="H40" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="65"/>
-      <c r="J40" s="67"/>
+      <c r="I40" s="69"/>
+      <c r="J40" s="65"/>
       <c r="K40" s="53"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="64" t="s">
+      <c r="A41" s="68" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="39" t="s">
@@ -2353,14 +2353,14 @@
       <c r="H41" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="66">
+      <c r="I41" s="64">
         <v>46230</v>
       </c>
-      <c r="J41" s="66"/>
+      <c r="J41" s="64"/>
       <c r="K41" s="52"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="65"/>
+      <c r="A42" s="69"/>
       <c r="B42" s="56" t="s">
         <v>13</v>
       </c>
@@ -2370,26 +2370,41 @@
       <c r="F42" s="57"/>
       <c r="G42" s="58"/>
       <c r="H42" s="56"/>
-      <c r="I42" s="65"/>
-      <c r="J42" s="67"/>
+      <c r="I42" s="69"/>
+      <c r="J42" s="65"/>
       <c r="K42" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2406,37 +2421,22 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -2471,56 +2471,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="72"/>
-      <c r="P2" s="72"/>
-      <c r="Q2" s="72"/>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="73"/>
+      <c r="Q2" s="73"/>
+      <c r="R2" s="73"/>
+      <c r="S2" s="73"/>
+      <c r="T2" s="73"/>
+      <c r="U2" s="73"/>
+      <c r="V2" s="73"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -4200,20 +4200,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4606,22 +4606,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5540,6 +5540,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5792,15 +5801,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5815,6 +5815,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5833,14 +5841,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 15:28)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17342736-9A5A-4BE9-A360-14E602BF2838}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CBFAFF0-4937-4D65-B797-338A352C1D17}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="324" yWindow="108" windowWidth="14988" windowHeight="11484" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -3127,7 +3127,7 @@
         <v>67</v>
       </c>
       <c r="D14" s="21">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E14" s="16">
         <v>1707089</v>
@@ -3612,7 +3612,7 @@
         <v>67</v>
       </c>
       <c r="D24" s="15">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="E24" s="16">
         <v>203880</v>
@@ -4160,7 +4160,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 17:02)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CBFAFF0-4937-4D65-B797-338A352C1D17}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{937C9C92-53BB-40B4-B11F-C97B1CC6D74C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="141">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -447,6 +447,24 @@
   </si>
   <si>
     <t>Data Actual  Plan</t>
+  </si>
+  <si>
+    <t>ประชุมไซต์ก่อนเริ่มงาน</t>
+  </si>
+  <si>
+    <t>ประชุม,คุยงานแก้ไขหลัง Corring</t>
+  </si>
+  <si>
+    <t>เข้าเคลียร์ติดตั้งหน้างานวันแรก</t>
+  </si>
+  <si>
+    <t>Achalaboon Residence</t>
+  </si>
+  <si>
+    <t>รอข้อมูลจาก Main con</t>
+  </si>
+  <si>
+    <t>Planning</t>
   </si>
 </sst>
 </file>
@@ -459,7 +477,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -559,6 +577,10 @@
       <family val="2"/>
       <charset val="222"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="7">
@@ -778,7 +800,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -981,6 +1003,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1076,6 +1110,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1363,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="41.33203125" bestFit="1" customWidth="1"/>
@@ -2374,8 +2412,51 @@
       <c r="J42" s="65"/>
       <c r="K42" s="53"/>
     </row>
+    <row r="43" spans="1:11">
+      <c r="A43" s="68" t="s">
+        <v>138</v>
+      </c>
+      <c r="B43" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="C43" s="40"/>
+      <c r="D43" s="40"/>
+      <c r="E43" s="40"/>
+      <c r="F43" s="40"/>
+      <c r="G43" s="41">
+        <v>0</v>
+      </c>
+      <c r="H43" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="I43" s="64"/>
+      <c r="J43" s="64"/>
+      <c r="K43" s="52"/>
+    </row>
+    <row r="44" spans="1:11" ht="15" thickBot="1">
+      <c r="A44" s="69"/>
+      <c r="B44" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="57"/>
+      <c r="D44" s="57"/>
+      <c r="E44" s="57"/>
+      <c r="F44" s="57"/>
+      <c r="G44" s="58">
+        <v>0</v>
+      </c>
+      <c r="H44" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="I44" s="69"/>
+      <c r="J44" s="65"/>
+      <c r="K44" s="53"/>
+    </row>
   </sheetData>
-  <mergeCells count="59">
+  <mergeCells count="62">
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="I39:I40"/>
     <mergeCell ref="J39:J40"/>
@@ -2436,7 +2517,7 @@
     <mergeCell ref="J33:J34"/>
     <mergeCell ref="J35:J36"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -3661,6 +3742,43 @@
       </c>
     </row>
     <row r="25" spans="1:22" s="13" customFormat="1" ht="18.600000000000001">
+      <c r="A25" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" s="78">
+        <v>0</v>
+      </c>
+      <c r="E25" s="13">
+        <v>799875</v>
+      </c>
+      <c r="F25" s="13">
+        <v>0</v>
+      </c>
+      <c r="G25" s="13">
+        <v>0</v>
+      </c>
+      <c r="H25" s="13">
+        <f>E25*0.4</f>
+        <v>319950</v>
+      </c>
+      <c r="L25" s="13">
+        <v>0</v>
+      </c>
+      <c r="N25" s="13">
+        <v>0</v>
+      </c>
+      <c r="P25" s="13">
+        <v>384843</v>
+      </c>
+      <c r="T25" s="13" t="s">
+        <v>139</v>
+      </c>
       <c r="V25" s="19"/>
     </row>
     <row r="26" spans="1:22" s="13" customFormat="1" ht="18.600000000000001">
@@ -4160,7 +4278,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4568,22 +4686,55 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="4"/>
+      <c r="A26" s="77">
+        <v>46219</v>
+      </c>
+      <c r="B26" s="76" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="76" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="75">
+        <v>3</v>
+      </c>
+      <c r="E26" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="4"/>
+      <c r="A27" s="3">
+        <v>46224</v>
+      </c>
+      <c r="B27" s="76" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="76" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="4">
+        <v>2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="4"/>
+      <c r="A28" s="3">
+        <v>46226</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="77" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="4">
+        <v>4</v>
+      </c>
+      <c r="E28" t="s">
+        <v>137</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 17:21)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{D6F423AA-70F0-48D1-99A3-0E79A49440FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{937C9C92-53BB-40B4-B11F-C97B1CC6D74C}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{F9904DBD-7032-4B5C-8FB6-1CDB90EC0AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E5C768D-E1C7-46E4-B8C8-9A8A6DDB9C8B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="141">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -979,6 +979,20 @@
     <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -998,23 +1012,9 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1110,10 +1110,6 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1416,34 +1412,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1481,7 +1477,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="78" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="59" t="s">
@@ -1501,14 +1497,14 @@
       <c r="H5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="66">
+      <c r="I5" s="72">
         <v>46244</v>
       </c>
-      <c r="J5" s="66"/>
+      <c r="J5" s="72"/>
       <c r="K5" s="48"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="69"/>
+      <c r="A6" s="75"/>
       <c r="B6" s="45" t="s">
         <v>13</v>
       </c>
@@ -1526,12 +1522,12 @@
       <c r="H6" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="69"/>
-      <c r="J6" s="65"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="71"/>
       <c r="K6" s="49"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="68" t="s">
+      <c r="A7" s="74" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="39" t="s">
@@ -1551,14 +1547,14 @@
       <c r="H7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="64"/>
+      <c r="J7" s="70"/>
       <c r="K7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="69"/>
+      <c r="A8" s="75"/>
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1576,12 +1572,12 @@
       <c r="H8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="69"/>
-      <c r="J8" s="65"/>
+      <c r="I8" s="75"/>
+      <c r="J8" s="71"/>
       <c r="K8" s="49"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="74" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="39" t="s">
@@ -1601,14 +1597,14 @@
       <c r="H9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="64">
+      <c r="I9" s="70">
         <v>46218</v>
       </c>
-      <c r="J9" s="64"/>
+      <c r="J9" s="70"/>
       <c r="K9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="69"/>
+      <c r="A10" s="75"/>
       <c r="B10" s="36" t="s">
         <v>13</v>
       </c>
@@ -1626,12 +1622,12 @@
       <c r="H10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="69"/>
-      <c r="J10" s="65"/>
+      <c r="I10" s="75"/>
+      <c r="J10" s="71"/>
       <c r="K10" s="49"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="68" t="s">
+      <c r="A11" s="74" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="42" t="s">
@@ -1651,14 +1647,14 @@
       <c r="H11" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="64">
+      <c r="I11" s="70">
         <v>46171</v>
       </c>
-      <c r="J11" s="64"/>
+      <c r="J11" s="70"/>
       <c r="K11" s="50"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="69"/>
+      <c r="A12" s="75"/>
       <c r="B12" s="45" t="s">
         <v>13</v>
       </c>
@@ -1676,12 +1672,12 @@
       <c r="H12" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="69"/>
-      <c r="J12" s="65"/>
+      <c r="I12" s="75"/>
+      <c r="J12" s="71"/>
       <c r="K12" s="49"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="68" t="s">
+      <c r="A13" s="74" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="39" t="s">
@@ -1701,14 +1697,14 @@
       <c r="H13" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="64"/>
+      <c r="J13" s="70"/>
       <c r="K13" s="50"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="69"/>
+      <c r="A14" s="75"/>
       <c r="B14" s="36" t="s">
         <v>13</v>
       </c>
@@ -1726,12 +1722,12 @@
       <c r="H14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="69"/>
-      <c r="J14" s="65"/>
+      <c r="I14" s="75"/>
+      <c r="J14" s="71"/>
       <c r="K14" s="49"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="68" t="s">
+      <c r="A15" s="74" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="42" t="s">
@@ -1751,14 +1747,14 @@
       <c r="H15" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="64">
+      <c r="I15" s="70">
         <v>46199</v>
       </c>
-      <c r="J15" s="64"/>
+      <c r="J15" s="70"/>
       <c r="K15" s="50"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="69"/>
+      <c r="A16" s="75"/>
       <c r="B16" s="45" t="s">
         <v>13</v>
       </c>
@@ -1776,12 +1772,12 @@
       <c r="H16" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="69"/>
-      <c r="J16" s="65"/>
+      <c r="I16" s="75"/>
+      <c r="J16" s="71"/>
       <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="70" t="s">
+      <c r="A17" s="76" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="33" t="s">
@@ -1801,14 +1797,14 @@
       <c r="H17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="67">
+      <c r="I17" s="73">
         <v>46305</v>
       </c>
-      <c r="J17" s="67"/>
+      <c r="J17" s="73"/>
       <c r="K17" s="51"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="69"/>
+      <c r="A18" s="75"/>
       <c r="B18" s="36" t="s">
         <v>13</v>
       </c>
@@ -1826,12 +1822,12 @@
       <c r="H18" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="69"/>
-      <c r="J18" s="65"/>
+      <c r="I18" s="75"/>
+      <c r="J18" s="71"/>
       <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="70" t="s">
+      <c r="A19" s="76" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="33" t="s">
@@ -1851,14 +1847,14 @@
       <c r="H19" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="67">
+      <c r="I19" s="73">
         <v>46336</v>
       </c>
-      <c r="J19" s="67"/>
+      <c r="J19" s="73"/>
       <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="69"/>
+      <c r="A20" s="75"/>
       <c r="B20" s="36" t="s">
         <v>13</v>
       </c>
@@ -1876,12 +1872,12 @@
       <c r="H20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="69"/>
-      <c r="J20" s="65"/>
+      <c r="I20" s="75"/>
+      <c r="J20" s="71"/>
       <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="68" t="s">
+      <c r="A21" s="74" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="39" t="s">
@@ -1901,14 +1897,14 @@
       <c r="H21" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="64">
+      <c r="I21" s="70">
         <v>46336</v>
       </c>
-      <c r="J21" s="64"/>
+      <c r="J21" s="70"/>
       <c r="K21" s="52"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="69"/>
+      <c r="A22" s="75"/>
       <c r="B22" s="36" t="s">
         <v>13</v>
       </c>
@@ -1926,12 +1922,12 @@
       <c r="H22" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="69"/>
-      <c r="J22" s="65"/>
+      <c r="I22" s="75"/>
+      <c r="J22" s="71"/>
       <c r="K22" s="53"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="68" t="s">
+      <c r="A23" s="74" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="42" t="s">
@@ -1951,14 +1947,14 @@
       <c r="H23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="64">
+      <c r="I23" s="70">
         <v>46237</v>
       </c>
-      <c r="J23" s="64"/>
+      <c r="J23" s="70"/>
       <c r="K23" s="52"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="69"/>
+      <c r="A24" s="75"/>
       <c r="B24" s="45" t="s">
         <v>13</v>
       </c>
@@ -1976,12 +1972,12 @@
       <c r="H24" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="69"/>
-      <c r="J24" s="65"/>
+      <c r="I24" s="75"/>
+      <c r="J24" s="71"/>
       <c r="K24" s="53"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="68" t="s">
+      <c r="A25" s="74" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="42" t="s">
@@ -2001,14 +1997,14 @@
       <c r="H25" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="64">
+      <c r="I25" s="70">
         <v>46188</v>
       </c>
-      <c r="J25" s="64"/>
+      <c r="J25" s="70"/>
       <c r="K25" s="52"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="69"/>
+      <c r="A26" s="75"/>
       <c r="B26" s="45" t="s">
         <v>13</v>
       </c>
@@ -2026,12 +2022,12 @@
       <c r="H26" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="69"/>
-      <c r="J26" s="65"/>
+      <c r="I26" s="75"/>
+      <c r="J26" s="71"/>
       <c r="K26" s="53"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="68" t="s">
+      <c r="A27" s="74" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="39" t="s">
@@ -2051,14 +2047,14 @@
       <c r="H27" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="64">
+      <c r="I27" s="70">
         <v>46321</v>
       </c>
-      <c r="J27" s="64"/>
+      <c r="J27" s="70"/>
       <c r="K27" s="52"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="69"/>
+      <c r="A28" s="75"/>
       <c r="B28" s="36" t="s">
         <v>13</v>
       </c>
@@ -2076,12 +2072,12 @@
       <c r="H28" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="69"/>
-      <c r="J28" s="65"/>
+      <c r="I28" s="75"/>
+      <c r="J28" s="71"/>
       <c r="K28" s="53"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="68" t="s">
+      <c r="A29" s="74" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="42" t="s">
@@ -2101,14 +2097,14 @@
       <c r="H29" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="64">
+      <c r="I29" s="70">
         <v>46139</v>
       </c>
-      <c r="J29" s="64"/>
+      <c r="J29" s="70"/>
       <c r="K29" s="52"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="69"/>
+      <c r="A30" s="75"/>
       <c r="B30" s="45" t="s">
         <v>13</v>
       </c>
@@ -2126,12 +2122,12 @@
       <c r="H30" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="69"/>
-      <c r="J30" s="65"/>
+      <c r="I30" s="75"/>
+      <c r="J30" s="71"/>
       <c r="K30" s="53"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="68" t="s">
+      <c r="A31" s="74" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="42" t="s">
@@ -2151,14 +2147,14 @@
       <c r="H31" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="64">
+      <c r="I31" s="70">
         <v>46133</v>
       </c>
-      <c r="J31" s="64"/>
+      <c r="J31" s="70"/>
       <c r="K31" s="52"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="69"/>
+      <c r="A32" s="75"/>
       <c r="B32" s="45" t="s">
         <v>13</v>
       </c>
@@ -2176,12 +2172,12 @@
       <c r="H32" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="69"/>
-      <c r="J32" s="65"/>
+      <c r="I32" s="75"/>
+      <c r="J32" s="71"/>
       <c r="K32" s="53"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="68" t="s">
+      <c r="A33" s="74" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="39" t="s">
@@ -2201,14 +2197,14 @@
       <c r="H33" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="64">
+      <c r="I33" s="70">
         <v>46295</v>
       </c>
-      <c r="J33" s="64"/>
+      <c r="J33" s="70"/>
       <c r="K33" s="52"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="69"/>
+      <c r="A34" s="75"/>
       <c r="B34" s="36" t="s">
         <v>13</v>
       </c>
@@ -2226,12 +2222,12 @@
       <c r="H34" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="69"/>
-      <c r="J34" s="65"/>
+      <c r="I34" s="75"/>
+      <c r="J34" s="71"/>
       <c r="K34" s="53"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="68" t="s">
+      <c r="A35" s="74" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="39" t="s">
@@ -2251,14 +2247,14 @@
       <c r="H35" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="64">
+      <c r="I35" s="70">
         <v>45884</v>
       </c>
-      <c r="J35" s="64"/>
+      <c r="J35" s="70"/>
       <c r="K35" s="52"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="69"/>
+      <c r="A36" s="75"/>
       <c r="B36" s="36" t="s">
         <v>13</v>
       </c>
@@ -2276,12 +2272,12 @@
       <c r="H36" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="69"/>
-      <c r="J36" s="65"/>
+      <c r="I36" s="75"/>
+      <c r="J36" s="71"/>
       <c r="K36" s="53"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="68" t="s">
+      <c r="A37" s="74" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="39" t="s">
@@ -2301,14 +2297,14 @@
       <c r="H37" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="64">
+      <c r="I37" s="70">
         <v>45915</v>
       </c>
-      <c r="J37" s="64"/>
+      <c r="J37" s="70"/>
       <c r="K37" s="52"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="69"/>
+      <c r="A38" s="75"/>
       <c r="B38" s="36" t="s">
         <v>13</v>
       </c>
@@ -2326,12 +2322,12 @@
       <c r="H38" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="69"/>
-      <c r="J38" s="65"/>
+      <c r="I38" s="75"/>
+      <c r="J38" s="71"/>
       <c r="K38" s="53"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="68" t="s">
+      <c r="A39" s="74" t="s">
         <v>131</v>
       </c>
       <c r="B39" s="39" t="s">
@@ -2345,14 +2341,14 @@
         <v>0</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I39" s="64"/>
-      <c r="J39" s="64"/>
+        <v>140</v>
+      </c>
+      <c r="I39" s="70"/>
+      <c r="J39" s="70"/>
       <c r="K39" s="52"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="69"/>
+      <c r="A40" s="75"/>
       <c r="B40" s="56" t="s">
         <v>13</v>
       </c>
@@ -2364,14 +2360,14 @@
         <v>0</v>
       </c>
       <c r="H40" s="56" t="s">
-        <v>15</v>
-      </c>
-      <c r="I40" s="69"/>
-      <c r="J40" s="65"/>
+        <v>140</v>
+      </c>
+      <c r="I40" s="75"/>
+      <c r="J40" s="71"/>
       <c r="K40" s="53"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="68" t="s">
+      <c r="A41" s="74" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="39" t="s">
@@ -2391,14 +2387,14 @@
       <c r="H41" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="64">
+      <c r="I41" s="70">
         <v>46230</v>
       </c>
-      <c r="J41" s="64"/>
+      <c r="J41" s="70"/>
       <c r="K41" s="52"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="69"/>
+      <c r="A42" s="75"/>
       <c r="B42" s="56" t="s">
         <v>13</v>
       </c>
@@ -2408,12 +2404,12 @@
       <c r="F42" s="57"/>
       <c r="G42" s="58"/>
       <c r="H42" s="56"/>
-      <c r="I42" s="69"/>
-      <c r="J42" s="65"/>
+      <c r="I42" s="75"/>
+      <c r="J42" s="71"/>
       <c r="K42" s="53"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="68" t="s">
+      <c r="A43" s="74" t="s">
         <v>138</v>
       </c>
       <c r="B43" s="39" t="s">
@@ -2427,14 +2423,14 @@
         <v>0</v>
       </c>
       <c r="H43" s="39" t="s">
-        <v>22</v>
-      </c>
-      <c r="I43" s="64"/>
-      <c r="J43" s="64"/>
+        <v>140</v>
+      </c>
+      <c r="I43" s="70"/>
+      <c r="J43" s="70"/>
       <c r="K43" s="52"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="69"/>
+      <c r="A44" s="75"/>
       <c r="B44" s="56" t="s">
         <v>13</v>
       </c>
@@ -2446,10 +2442,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="56" t="s">
-        <v>22</v>
-      </c>
-      <c r="I44" s="69"/>
-      <c r="J44" s="65"/>
+        <v>140</v>
+      </c>
+      <c r="I44" s="75"/>
+      <c r="J44" s="71"/>
       <c r="K44" s="53"/>
     </row>
   </sheetData>
@@ -2552,56 +2548,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="68"/>
+      <c r="U1" s="68"/>
+      <c r="V1" s="68"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
-      <c r="T2" s="73"/>
-      <c r="U2" s="73"/>
-      <c r="V2" s="73"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="69"/>
+      <c r="V2" s="69"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -3644,7 +3640,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>67</v>
@@ -3741,42 +3737,45 @@
         <v>46213</v>
       </c>
     </row>
-    <row r="25" spans="1:22" s="13" customFormat="1" ht="18.600000000000001">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+      <c r="A25" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="78">
+      <c r="D25" s="67">
         <v>0</v>
       </c>
-      <c r="E25" s="13">
+      <c r="E25" s="12">
         <v>799875</v>
       </c>
-      <c r="F25" s="13">
+      <c r="F25" s="9">
         <v>0</v>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="9">
         <v>0</v>
       </c>
-      <c r="H25" s="13">
+      <c r="H25" s="9">
         <f>E25*0.4</f>
         <v>319950</v>
       </c>
-      <c r="L25" s="13">
+      <c r="L25" s="9">
+        <v>22399</v>
+      </c>
+      <c r="N25" s="9">
         <v>0</v>
       </c>
-      <c r="N25" s="13">
-        <v>0</v>
-      </c>
-      <c r="P25" s="13">
+      <c r="O25" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="P25" s="12">
         <v>384843</v>
       </c>
-      <c r="T25" s="13" t="s">
+      <c r="T25" s="9" t="s">
         <v>139</v>
       </c>
       <c r="V25" s="19"/>
@@ -4278,7 +4277,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4302,6 +4301,7 @@
     <hyperlink ref="U24" r:id="rId10" xr:uid="{DFFF659B-3A50-4FD0-AA9F-289AE4EB0963}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId11"/>
 </worksheet>
 </file>
 
@@ -4318,20 +4318,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4686,16 +4686,16 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="77">
+      <c r="A26" s="66">
         <v>46219</v>
       </c>
-      <c r="B26" s="76" t="s">
+      <c r="B26" s="65" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="76" t="s">
+      <c r="C26" s="65" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="75">
+      <c r="D26" s="64">
         <v>3</v>
       </c>
       <c r="E26" t="s">
@@ -4706,10 +4706,10 @@
       <c r="A27" s="3">
         <v>46224</v>
       </c>
-      <c r="B27" s="76" t="s">
+      <c r="B27" s="65" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="76" t="s">
+      <c r="C27" s="65" t="s">
         <v>61</v>
       </c>
       <c r="D27" s="4">
@@ -4726,7 +4726,7 @@
       <c r="B28" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="77" t="s">
+      <c r="C28" s="66" t="s">
         <v>61</v>
       </c>
       <c r="D28" s="4">
@@ -4757,22 +4757,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5691,15 +5691,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5952,7 +5943,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5965,15 +5956,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5992,7 +5984,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -6001,4 +5993,12 @@
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 17:55)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{F9904DBD-7032-4B5C-8FB6-1CDB90EC0AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E5C768D-E1C7-46E4-B8C8-9A8A6DDB9C8B}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{F9904DBD-7032-4B5C-8FB6-1CDB90EC0AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{787C0A91-B15D-439A-A808-661A8A7411B0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="143">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -465,6 +465,12 @@
   </si>
   <si>
     <t>Planning</t>
+  </si>
+  <si>
+    <t>Huaykwang residence</t>
+  </si>
+  <si>
+    <t>ส่งมอบงานงวดสุดท้าย</t>
   </si>
 </sst>
 </file>
@@ -581,6 +587,7 @@
     <font>
       <sz val="10.5"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1018,10 +1025,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="4">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Comma 2 2 3 2" xfId="3" xr:uid="{10CA6883-C0B4-442D-A7D0-FF27A9ED468E}"/>
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="จุลภาค" xfId="1" builtinId="3"/>
-    <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1110,6 +1117,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4277,7 +4288,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4307,7 +4318,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -4734,6 +4745,40 @@
       </c>
       <c r="E28" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="3">
+        <v>46227</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="66" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="4">
+        <v>4</v>
+      </c>
+      <c r="E29" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="3">
+        <v>46230</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" s="66" t="s">
+        <v>61</v>
+      </c>
+      <c r="D30" s="4">
+        <v>4</v>
+      </c>
+      <c r="E30" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-24 14:50)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{F9904DBD-7032-4B5C-8FB6-1CDB90EC0AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{787C0A91-B15D-439A-A808-661A8A7411B0}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{996805BD-2E1C-4C06-8112-A048AB4BF4BE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="142">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -435,9 +435,6 @@
   </si>
   <si>
     <t>ส่งงาน 100% วันที่ 07/24/2026</t>
-  </si>
-  <si>
-    <t>บ้านคุณทวีชัย สมุทปราการ</t>
   </si>
   <si>
     <t>ราคา Minimum ของผู้รับเหมา</t>
@@ -999,6 +996,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1019,16 +1017,15 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Comma 2 2 3 2" xfId="3" xr:uid="{10CA6883-C0B4-442D-A7D0-FF27A9ED468E}"/>
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="จุลภาค" xfId="1" builtinId="3"/>
+    <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1066,16 +1063,6 @@
             <v>46189</v>
           </cell>
         </row>
-        <row r="7">
-          <cell r="C7">
-            <v>46219</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="C8">
-            <v>46244</v>
-          </cell>
-        </row>
         <row r="10">
           <cell r="C10">
             <v>46168</v>
@@ -1101,26 +1088,12 @@
             <v>46198</v>
           </cell>
         </row>
-        <row r="17">
-          <cell r="C17">
-            <v>46188</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="C18">
-            <v>46200</v>
-          </cell>
-        </row>
       </sheetData>
       <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1426,31 +1399,31 @@
       <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="77"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-      <c r="K2" s="77"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1508,14 +1481,14 @@
       <c r="H5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="72">
+      <c r="I5" s="73">
         <v>46244</v>
       </c>
-      <c r="J5" s="72"/>
+      <c r="J5" s="73"/>
       <c r="K5" s="48"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="75"/>
+      <c r="A6" s="76"/>
       <c r="B6" s="45" t="s">
         <v>13</v>
       </c>
@@ -1533,12 +1506,12 @@
       <c r="H6" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="75"/>
-      <c r="J6" s="71"/>
+      <c r="I6" s="76"/>
+      <c r="J6" s="72"/>
       <c r="K6" s="49"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="74" t="s">
+      <c r="A7" s="75" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="39" t="s">
@@ -1558,14 +1531,14 @@
       <c r="H7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="70" t="s">
+      <c r="I7" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="70"/>
+      <c r="J7" s="71"/>
       <c r="K7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="75"/>
+      <c r="A8" s="76"/>
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1583,12 +1556,12 @@
       <c r="H8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="75"/>
-      <c r="J8" s="71"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="72"/>
       <c r="K8" s="49"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="74" t="s">
+      <c r="A9" s="75" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="39" t="s">
@@ -1608,14 +1581,14 @@
       <c r="H9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="70">
+      <c r="I9" s="71">
         <v>46218</v>
       </c>
-      <c r="J9" s="70"/>
+      <c r="J9" s="71"/>
       <c r="K9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="75"/>
+      <c r="A10" s="76"/>
       <c r="B10" s="36" t="s">
         <v>13</v>
       </c>
@@ -1633,12 +1606,12 @@
       <c r="H10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="75"/>
-      <c r="J10" s="71"/>
+      <c r="I10" s="76"/>
+      <c r="J10" s="72"/>
       <c r="K10" s="49"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="74" t="s">
+      <c r="A11" s="75" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="42" t="s">
@@ -1658,14 +1631,14 @@
       <c r="H11" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="70">
+      <c r="I11" s="71">
         <v>46171</v>
       </c>
-      <c r="J11" s="70"/>
+      <c r="J11" s="71"/>
       <c r="K11" s="50"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="75"/>
+      <c r="A12" s="76"/>
       <c r="B12" s="45" t="s">
         <v>13</v>
       </c>
@@ -1683,12 +1656,12 @@
       <c r="H12" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="75"/>
-      <c r="J12" s="71"/>
+      <c r="I12" s="76"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="49"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="75" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="39" t="s">
@@ -1708,14 +1681,14 @@
       <c r="H13" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="70" t="s">
+      <c r="I13" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="70"/>
+      <c r="J13" s="71"/>
       <c r="K13" s="50"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="75"/>
+      <c r="A14" s="76"/>
       <c r="B14" s="36" t="s">
         <v>13</v>
       </c>
@@ -1733,12 +1706,12 @@
       <c r="H14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="75"/>
-      <c r="J14" s="71"/>
+      <c r="I14" s="76"/>
+      <c r="J14" s="72"/>
       <c r="K14" s="49"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="74" t="s">
+      <c r="A15" s="75" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="42" t="s">
@@ -1758,14 +1731,14 @@
       <c r="H15" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="70">
+      <c r="I15" s="71">
         <v>46199</v>
       </c>
-      <c r="J15" s="70"/>
+      <c r="J15" s="71"/>
       <c r="K15" s="50"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="75"/>
+      <c r="A16" s="76"/>
       <c r="B16" s="45" t="s">
         <v>13</v>
       </c>
@@ -1783,12 +1756,12 @@
       <c r="H16" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="75"/>
-      <c r="J16" s="71"/>
+      <c r="I16" s="76"/>
+      <c r="J16" s="72"/>
       <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="76" t="s">
+      <c r="A17" s="77" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="33" t="s">
@@ -1808,14 +1781,14 @@
       <c r="H17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="73">
+      <c r="I17" s="74">
         <v>46305</v>
       </c>
-      <c r="J17" s="73"/>
+      <c r="J17" s="74"/>
       <c r="K17" s="51"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="75"/>
+      <c r="A18" s="76"/>
       <c r="B18" s="36" t="s">
         <v>13</v>
       </c>
@@ -1833,12 +1806,12 @@
       <c r="H18" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="75"/>
-      <c r="J18" s="71"/>
+      <c r="I18" s="76"/>
+      <c r="J18" s="72"/>
       <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="76" t="s">
+      <c r="A19" s="77" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="33" t="s">
@@ -1858,14 +1831,14 @@
       <c r="H19" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="73">
+      <c r="I19" s="74">
         <v>46336</v>
       </c>
-      <c r="J19" s="73"/>
+      <c r="J19" s="74"/>
       <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="75"/>
+      <c r="A20" s="76"/>
       <c r="B20" s="36" t="s">
         <v>13</v>
       </c>
@@ -1883,12 +1856,12 @@
       <c r="H20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="75"/>
-      <c r="J20" s="71"/>
+      <c r="I20" s="76"/>
+      <c r="J20" s="72"/>
       <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="74" t="s">
+      <c r="A21" s="75" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="39" t="s">
@@ -1908,14 +1881,14 @@
       <c r="H21" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="70">
+      <c r="I21" s="71">
         <v>46336</v>
       </c>
-      <c r="J21" s="70"/>
+      <c r="J21" s="71"/>
       <c r="K21" s="52"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="75"/>
+      <c r="A22" s="76"/>
       <c r="B22" s="36" t="s">
         <v>13</v>
       </c>
@@ -1933,12 +1906,12 @@
       <c r="H22" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="75"/>
-      <c r="J22" s="71"/>
+      <c r="I22" s="76"/>
+      <c r="J22" s="72"/>
       <c r="K22" s="53"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="74" t="s">
+      <c r="A23" s="75" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="42" t="s">
@@ -1958,14 +1931,14 @@
       <c r="H23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="70">
+      <c r="I23" s="71">
         <v>46237</v>
       </c>
-      <c r="J23" s="70"/>
+      <c r="J23" s="71"/>
       <c r="K23" s="52"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="75"/>
+      <c r="A24" s="76"/>
       <c r="B24" s="45" t="s">
         <v>13</v>
       </c>
@@ -1983,12 +1956,12 @@
       <c r="H24" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="75"/>
-      <c r="J24" s="71"/>
+      <c r="I24" s="76"/>
+      <c r="J24" s="72"/>
       <c r="K24" s="53"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="74" t="s">
+      <c r="A25" s="75" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="42" t="s">
@@ -2008,14 +1981,14 @@
       <c r="H25" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="70">
+      <c r="I25" s="71">
         <v>46188</v>
       </c>
-      <c r="J25" s="70"/>
+      <c r="J25" s="71"/>
       <c r="K25" s="52"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="75"/>
+      <c r="A26" s="76"/>
       <c r="B26" s="45" t="s">
         <v>13</v>
       </c>
@@ -2033,12 +2006,12 @@
       <c r="H26" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="75"/>
-      <c r="J26" s="71"/>
+      <c r="I26" s="76"/>
+      <c r="J26" s="72"/>
       <c r="K26" s="53"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="74" t="s">
+      <c r="A27" s="75" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="39" t="s">
@@ -2058,14 +2031,14 @@
       <c r="H27" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="70">
+      <c r="I27" s="71">
         <v>46321</v>
       </c>
-      <c r="J27" s="70"/>
+      <c r="J27" s="71"/>
       <c r="K27" s="52"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="75"/>
+      <c r="A28" s="76"/>
       <c r="B28" s="36" t="s">
         <v>13</v>
       </c>
@@ -2083,12 +2056,12 @@
       <c r="H28" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="75"/>
-      <c r="J28" s="71"/>
+      <c r="I28" s="76"/>
+      <c r="J28" s="72"/>
       <c r="K28" s="53"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="74" t="s">
+      <c r="A29" s="75" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="42" t="s">
@@ -2108,14 +2081,14 @@
       <c r="H29" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="70">
+      <c r="I29" s="71">
         <v>46139</v>
       </c>
-      <c r="J29" s="70"/>
+      <c r="J29" s="71"/>
       <c r="K29" s="52"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="75"/>
+      <c r="A30" s="76"/>
       <c r="B30" s="45" t="s">
         <v>13</v>
       </c>
@@ -2133,12 +2106,12 @@
       <c r="H30" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="75"/>
-      <c r="J30" s="71"/>
+      <c r="I30" s="76"/>
+      <c r="J30" s="72"/>
       <c r="K30" s="53"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="74" t="s">
+      <c r="A31" s="75" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="42" t="s">
@@ -2158,14 +2131,14 @@
       <c r="H31" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="70">
+      <c r="I31" s="71">
         <v>46133</v>
       </c>
-      <c r="J31" s="70"/>
+      <c r="J31" s="71"/>
       <c r="K31" s="52"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="75"/>
+      <c r="A32" s="76"/>
       <c r="B32" s="45" t="s">
         <v>13</v>
       </c>
@@ -2183,12 +2156,12 @@
       <c r="H32" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="75"/>
-      <c r="J32" s="71"/>
+      <c r="I32" s="76"/>
+      <c r="J32" s="72"/>
       <c r="K32" s="53"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="74" t="s">
+      <c r="A33" s="75" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="39" t="s">
@@ -2208,14 +2181,14 @@
       <c r="H33" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="70">
+      <c r="I33" s="71">
         <v>46295</v>
       </c>
-      <c r="J33" s="70"/>
+      <c r="J33" s="71"/>
       <c r="K33" s="52"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="75"/>
+      <c r="A34" s="76"/>
       <c r="B34" s="36" t="s">
         <v>13</v>
       </c>
@@ -2233,12 +2206,12 @@
       <c r="H34" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="75"/>
-      <c r="J34" s="71"/>
+      <c r="I34" s="76"/>
+      <c r="J34" s="72"/>
       <c r="K34" s="53"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="74" t="s">
+      <c r="A35" s="75" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="39" t="s">
@@ -2258,14 +2231,14 @@
       <c r="H35" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="70">
+      <c r="I35" s="71">
         <v>45884</v>
       </c>
-      <c r="J35" s="70"/>
+      <c r="J35" s="71"/>
       <c r="K35" s="52"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="75"/>
+      <c r="A36" s="76"/>
       <c r="B36" s="36" t="s">
         <v>13</v>
       </c>
@@ -2283,12 +2256,12 @@
       <c r="H36" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="75"/>
-      <c r="J36" s="71"/>
+      <c r="I36" s="76"/>
+      <c r="J36" s="72"/>
       <c r="K36" s="53"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="74" t="s">
+      <c r="A37" s="75" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="39" t="s">
@@ -2308,14 +2281,14 @@
       <c r="H37" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="70">
+      <c r="I37" s="71">
         <v>45915</v>
       </c>
-      <c r="J37" s="70"/>
+      <c r="J37" s="71"/>
       <c r="K37" s="52"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="75"/>
+      <c r="A38" s="76"/>
       <c r="B38" s="36" t="s">
         <v>13</v>
       </c>
@@ -2333,13 +2306,13 @@
       <c r="H38" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="75"/>
-      <c r="J38" s="71"/>
+      <c r="I38" s="76"/>
+      <c r="J38" s="72"/>
       <c r="K38" s="53"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="74" t="s">
-        <v>131</v>
+      <c r="A39" s="75" t="s">
+        <v>91</v>
       </c>
       <c r="B39" s="39" t="s">
         <v>11</v>
@@ -2352,14 +2325,14 @@
         <v>0</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>140</v>
-      </c>
-      <c r="I39" s="70"/>
-      <c r="J39" s="70"/>
+        <v>139</v>
+      </c>
+      <c r="I39" s="71"/>
+      <c r="J39" s="71"/>
       <c r="K39" s="52"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="75"/>
+      <c r="A40" s="76"/>
       <c r="B40" s="56" t="s">
         <v>13</v>
       </c>
@@ -2371,14 +2344,14 @@
         <v>0</v>
       </c>
       <c r="H40" s="56" t="s">
-        <v>140</v>
-      </c>
-      <c r="I40" s="75"/>
-      <c r="J40" s="71"/>
+        <v>139</v>
+      </c>
+      <c r="I40" s="76"/>
+      <c r="J40" s="72"/>
       <c r="K40" s="53"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="74" t="s">
+      <c r="A41" s="75" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="39" t="s">
@@ -2398,14 +2371,14 @@
       <c r="H41" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="70">
+      <c r="I41" s="71">
         <v>46230</v>
       </c>
-      <c r="J41" s="70"/>
+      <c r="J41" s="71"/>
       <c r="K41" s="52"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="75"/>
+      <c r="A42" s="76"/>
       <c r="B42" s="56" t="s">
         <v>13</v>
       </c>
@@ -2415,13 +2388,13 @@
       <c r="F42" s="57"/>
       <c r="G42" s="58"/>
       <c r="H42" s="56"/>
-      <c r="I42" s="75"/>
-      <c r="J42" s="71"/>
+      <c r="I42" s="76"/>
+      <c r="J42" s="72"/>
       <c r="K42" s="53"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="74" t="s">
-        <v>138</v>
+      <c r="A43" s="75" t="s">
+        <v>137</v>
       </c>
       <c r="B43" s="39" t="s">
         <v>11</v>
@@ -2434,14 +2407,14 @@
         <v>0</v>
       </c>
       <c r="H43" s="39" t="s">
-        <v>140</v>
-      </c>
-      <c r="I43" s="70"/>
-      <c r="J43" s="70"/>
+        <v>139</v>
+      </c>
+      <c r="I43" s="71"/>
+      <c r="J43" s="71"/>
       <c r="K43" s="52"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="75"/>
+      <c r="A44" s="76"/>
       <c r="B44" s="56" t="s">
         <v>13</v>
       </c>
@@ -2453,10 +2426,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="56" t="s">
-        <v>140</v>
-      </c>
-      <c r="I44" s="75"/>
-      <c r="J44" s="71"/>
+        <v>139</v>
+      </c>
+      <c r="I44" s="76"/>
+      <c r="J44" s="72"/>
       <c r="K44" s="53"/>
     </row>
   </sheetData>
@@ -2585,30 +2558,30 @@
       <c r="V1" s="68"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="70" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
-      <c r="V2" s="69"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="70"/>
+      <c r="N2" s="70"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="70"/>
+      <c r="S2" s="70"/>
+      <c r="T2" s="70"/>
+      <c r="U2" s="70"/>
+      <c r="V2" s="70"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -2840,11 +2813,10 @@
         <v>280000</v>
       </c>
       <c r="Q7" s="19">
-        <f>'[1]Master Schedule'!C7</f>
+        <v>46102</v>
+      </c>
+      <c r="R7" s="19">
         <v>46219</v>
-      </c>
-      <c r="R7" s="19">
-        <v>46102</v>
       </c>
       <c r="S7" s="14"/>
       <c r="T7" s="26" t="s">
@@ -2901,11 +2873,10 @@
         <v>89000</v>
       </c>
       <c r="Q8" s="19">
-        <f>'[1]Master Schedule'!C8</f>
+        <v>46171</v>
+      </c>
+      <c r="R8" s="19">
         <v>46244</v>
-      </c>
-      <c r="R8" s="19">
-        <v>46171</v>
       </c>
       <c r="S8" s="14"/>
       <c r="T8" s="26"/>
@@ -3420,11 +3391,10 @@
         <v>234861</v>
       </c>
       <c r="Q17" s="19">
-        <f>'[1]Master Schedule'!C17</f>
+        <v>46139</v>
+      </c>
+      <c r="R17" s="11">
         <v>46188</v>
-      </c>
-      <c r="R17" s="11">
-        <v>46139</v>
       </c>
       <c r="T17" s="28"/>
       <c r="U17" s="26"/>
@@ -3474,11 +3444,10 @@
         <v>119980</v>
       </c>
       <c r="Q18" s="19">
-        <f>'[1]Master Schedule'!C18</f>
+        <v>46133</v>
+      </c>
+      <c r="R18" s="11">
         <v>46200</v>
-      </c>
-      <c r="R18" s="11">
-        <v>46133</v>
       </c>
       <c r="T18" s="28"/>
       <c r="U18" s="26"/>
@@ -3651,7 +3620,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>67</v>
@@ -3750,10 +3719,10 @@
     </row>
     <row r="25" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
       <c r="A25" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>67</v>
@@ -3787,7 +3756,7 @@
         <v>384843</v>
       </c>
       <c r="T25" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="V25" s="19"/>
     </row>
@@ -4333,16 +4302,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="68"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="70" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4710,7 +4679,7 @@
         <v>3</v>
       </c>
       <c r="E26" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4727,7 +4696,7 @@
         <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -4744,7 +4713,7 @@
         <v>4</v>
       </c>
       <c r="E28" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -4752,7 +4721,7 @@
         <v>46227</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C29" s="66" t="s">
         <v>61</v>
@@ -4778,7 +4747,7 @@
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -4811,13 +4780,13 @@
       <c r="E1" s="68"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="70" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4889,10 +4858,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="C8" s="6">
         <v>46226</v>
@@ -4906,7 +4875,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="6">
@@ -5736,6 +5705,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5988,29 +5979,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6027,23 +6015,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-27 10:28)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{996805BD-2E1C-4C06-8112-A048AB4BF4BE}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5E2E3CC-A260-4216-891E-591C22F5C5DB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -434,9 +434,6 @@
     <t>https://corallife806.sharepoint.com/:b:/s/CoralLife2/IQB85P7JtoSZT6532Il6VakbAcqfI6xy5EwPf0pgbRJpT3Y?e=Qwe5V0</t>
   </si>
   <si>
-    <t>ส่งงาน 100% วันที่ 07/24/2026</t>
-  </si>
-  <si>
     <t>ราคา Minimum ของผู้รับเหมา</t>
   </si>
   <si>
@@ -468,6 +465,9 @@
   </si>
   <si>
     <t>ส่งมอบงานงวดสุดท้าย</t>
+  </si>
+  <si>
+    <t>คิดงานเพิ่ม 3000 บาท ค่ากล่องพรีนัม ส่งงานวันที่ 07/31/2026</t>
   </si>
 </sst>
 </file>
@@ -804,7 +804,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -862,9 +862,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -998,27 +995,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1396,34 +1393,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1461,988 +1458,1016 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="78" t="s">
+      <c r="A5" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="60">
+      <c r="C5" s="59">
         <v>46084</v>
       </c>
-      <c r="D5" s="60">
+      <c r="D5" s="59">
         <v>46127</v>
       </c>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="61">
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="60">
         <v>1</v>
       </c>
-      <c r="H5" s="59" t="s">
+      <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="73">
+      <c r="I5" s="77">
         <v>46244</v>
       </c>
-      <c r="J5" s="73"/>
-      <c r="K5" s="48"/>
+      <c r="J5" s="77"/>
+      <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="76"/>
-      <c r="B6" s="45" t="s">
+      <c r="A6" s="71"/>
+      <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="45">
         <v>46189</v>
       </c>
-      <c r="D6" s="46">
+      <c r="D6" s="45">
         <v>46189</v>
       </c>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="47">
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="46">
         <v>1</v>
       </c>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="76"/>
-      <c r="J6" s="72"/>
-      <c r="K6" s="49"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="70" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="40">
+      <c r="C7" s="39">
         <v>46219</v>
       </c>
-      <c r="D7" s="40">
+      <c r="D7" s="39">
         <v>46233</v>
       </c>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41">
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="40">
         <v>0</v>
       </c>
-      <c r="H7" s="39" t="s">
+      <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="71" t="s">
+      <c r="I7" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="71"/>
-      <c r="K7" s="50"/>
+      <c r="J7" s="72"/>
+      <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="76"/>
-      <c r="B8" s="36" t="s">
+      <c r="A8" s="71"/>
+      <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="37">
+      <c r="C8" s="36">
         <v>46244</v>
       </c>
-      <c r="D8" s="37">
+      <c r="D8" s="36">
         <v>46247</v>
       </c>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="38">
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="37">
         <v>0</v>
       </c>
-      <c r="H8" s="36" t="s">
+      <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="76"/>
-      <c r="J8" s="72"/>
-      <c r="K8" s="49"/>
+      <c r="I8" s="71"/>
+      <c r="J8" s="73"/>
+      <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="75" t="s">
+      <c r="A9" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="40">
+      <c r="C9" s="39">
         <v>46082</v>
       </c>
-      <c r="D9" s="40">
+      <c r="D9" s="39">
         <v>46096</v>
       </c>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="41">
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="40">
         <v>1</v>
       </c>
-      <c r="H9" s="39" t="s">
+      <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="71">
+      <c r="I9" s="72">
         <v>46218</v>
       </c>
-      <c r="J9" s="71"/>
-      <c r="K9" s="50"/>
+      <c r="J9" s="72"/>
+      <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="76"/>
-      <c r="B10" s="36" t="s">
+      <c r="A10" s="71"/>
+      <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="36">
         <v>46168</v>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="36">
         <v>46213</v>
       </c>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="38">
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="37">
         <v>1</v>
       </c>
-      <c r="H10" s="36" t="s">
+      <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="76"/>
-      <c r="J10" s="72"/>
-      <c r="K10" s="49"/>
+      <c r="I10" s="71"/>
+      <c r="J10" s="73"/>
+      <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="75" t="s">
+      <c r="A11" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="42" t="s">
+      <c r="B11" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="43">
+      <c r="C11" s="42">
         <v>46184</v>
       </c>
-      <c r="D11" s="43">
+      <c r="D11" s="42">
         <v>46191</v>
       </c>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="44">
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="43">
         <v>1</v>
       </c>
-      <c r="H11" s="42" t="s">
+      <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="71">
+      <c r="I11" s="72">
         <v>46171</v>
       </c>
-      <c r="J11" s="71"/>
-      <c r="K11" s="50"/>
+      <c r="J11" s="72"/>
+      <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="76"/>
-      <c r="B12" s="45" t="s">
+      <c r="A12" s="71"/>
+      <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="45">
         <v>46200</v>
       </c>
-      <c r="D12" s="46">
+      <c r="D12" s="45">
         <v>46202</v>
       </c>
-      <c r="E12" s="46"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="47">
+      <c r="E12" s="45"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="46">
         <v>1</v>
       </c>
-      <c r="H12" s="45" t="s">
+      <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="76"/>
-      <c r="J12" s="72"/>
-      <c r="K12" s="49"/>
+      <c r="I12" s="71"/>
+      <c r="J12" s="73"/>
+      <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="75" t="s">
+      <c r="A13" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="40">
+      <c r="C13" s="39">
         <v>46392</v>
       </c>
-      <c r="D13" s="40">
+      <c r="D13" s="39">
         <v>46402</v>
       </c>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="41">
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40">
         <v>0</v>
       </c>
-      <c r="H13" s="39" t="s">
+      <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="71" t="s">
+      <c r="I13" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="71"/>
-      <c r="K13" s="50"/>
+      <c r="J13" s="72"/>
+      <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="76"/>
-      <c r="B14" s="36" t="s">
+      <c r="A14" s="71"/>
+      <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="37">
+      <c r="C14" s="36">
         <v>46042</v>
       </c>
-      <c r="D14" s="37">
+      <c r="D14" s="36">
         <v>46042</v>
       </c>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="38">
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="37">
         <v>0</v>
       </c>
-      <c r="H14" s="36" t="s">
+      <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="76"/>
-      <c r="J14" s="72"/>
-      <c r="K14" s="49"/>
+      <c r="I14" s="71"/>
+      <c r="J14" s="73"/>
+      <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="75" t="s">
+      <c r="A15" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="42">
         <v>46168</v>
       </c>
-      <c r="D15" s="43">
+      <c r="D15" s="42">
         <v>46188</v>
       </c>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="44">
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="43">
         <v>1</v>
       </c>
-      <c r="H15" s="42" t="s">
+      <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="71">
+      <c r="I15" s="72">
         <v>46199</v>
       </c>
-      <c r="J15" s="71"/>
-      <c r="K15" s="50"/>
+      <c r="J15" s="72"/>
+      <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="76"/>
-      <c r="B16" s="45" t="s">
+      <c r="A16" s="71"/>
+      <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="45">
         <v>46198</v>
       </c>
-      <c r="D16" s="46">
+      <c r="D16" s="45">
         <v>46199</v>
       </c>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="47">
+      <c r="E16" s="45"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="46">
         <v>1</v>
       </c>
-      <c r="H16" s="45" t="s">
+      <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="76"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="49"/>
+      <c r="I16" s="71"/>
+      <c r="J16" s="73"/>
+      <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="77" t="s">
+      <c r="A17" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="34">
+      <c r="C17" s="33">
         <v>46188</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="33">
         <v>46198</v>
       </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35">
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="34">
         <v>0.8</v>
       </c>
-      <c r="H17" s="33" t="s">
+      <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
       <c r="I17" s="74">
         <v>46305</v>
       </c>
       <c r="J17" s="74"/>
-      <c r="K17" s="51"/>
+      <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="76"/>
-      <c r="B18" s="36" t="s">
+      <c r="A18" s="71"/>
+      <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="37">
+      <c r="C18" s="36">
         <v>46296</v>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="36">
         <v>46298</v>
       </c>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="38">
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="37">
         <v>0.4</v>
       </c>
-      <c r="H18" s="36" t="s">
+      <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="76"/>
-      <c r="J18" s="72"/>
-      <c r="K18" s="49"/>
+      <c r="I18" s="71"/>
+      <c r="J18" s="73"/>
+      <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="77" t="s">
+      <c r="A19" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="34">
+      <c r="C19" s="33">
         <v>46275</v>
       </c>
-      <c r="D19" s="34">
+      <c r="D19" s="33">
         <v>46290</v>
       </c>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="35">
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="34">
         <v>0</v>
       </c>
-      <c r="H19" s="33" t="s">
+      <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
       <c r="I19" s="74">
         <v>46336</v>
       </c>
       <c r="J19" s="74"/>
-      <c r="K19" s="51"/>
+      <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="76"/>
-      <c r="B20" s="36" t="s">
+      <c r="A20" s="71"/>
+      <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="37">
+      <c r="C20" s="36">
         <v>46327</v>
       </c>
-      <c r="D20" s="37">
+      <c r="D20" s="36">
         <v>46329</v>
       </c>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="38">
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="37">
         <v>0</v>
       </c>
-      <c r="H20" s="36" t="s">
+      <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="76"/>
-      <c r="J20" s="72"/>
-      <c r="K20" s="49"/>
+      <c r="I20" s="71"/>
+      <c r="J20" s="73"/>
+      <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="75" t="s">
+      <c r="A21" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="39">
         <v>46240</v>
       </c>
-      <c r="D21" s="40">
+      <c r="D21" s="39">
         <v>46249</v>
       </c>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="41">
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="40">
         <v>0</v>
       </c>
-      <c r="H21" s="39" t="s">
+      <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="71">
+      <c r="I21" s="72">
         <v>46336</v>
       </c>
-      <c r="J21" s="71"/>
-      <c r="K21" s="52"/>
+      <c r="J21" s="72"/>
+      <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="76"/>
-      <c r="B22" s="36" t="s">
+      <c r="A22" s="71"/>
+      <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="36">
         <v>46327</v>
       </c>
-      <c r="D22" s="37">
+      <c r="D22" s="36">
         <v>46329</v>
       </c>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="38">
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="37">
         <v>0</v>
       </c>
-      <c r="H22" s="36" t="s">
+      <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="76"/>
-      <c r="J22" s="72"/>
-      <c r="K22" s="53"/>
+      <c r="I22" s="71"/>
+      <c r="J22" s="73"/>
+      <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B23" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="43">
+      <c r="C23" s="42">
         <v>46190</v>
       </c>
-      <c r="D23" s="43">
+      <c r="D23" s="42">
         <v>46206</v>
       </c>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="44">
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="43">
         <v>1</v>
       </c>
-      <c r="H23" s="42" t="s">
+      <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="72">
         <v>46237</v>
       </c>
-      <c r="J23" s="71"/>
-      <c r="K23" s="52"/>
+      <c r="J23" s="72"/>
+      <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="76"/>
-      <c r="B24" s="45" t="s">
+      <c r="A24" s="71"/>
+      <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="46">
+      <c r="C24" s="45">
         <v>46216</v>
       </c>
-      <c r="D24" s="46">
+      <c r="D24" s="45">
         <v>46220</v>
       </c>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="47">
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="46">
         <v>1</v>
       </c>
-      <c r="H24" s="45" t="s">
+      <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="76"/>
-      <c r="J24" s="72"/>
-      <c r="K24" s="53"/>
+      <c r="I24" s="71"/>
+      <c r="J24" s="73"/>
+      <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="75" t="s">
+      <c r="A25" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="43">
+      <c r="C25" s="42">
         <v>46185</v>
       </c>
-      <c r="D25" s="43">
+      <c r="D25" s="42">
         <v>46188</v>
       </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="44">
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="43">
         <v>1</v>
       </c>
-      <c r="H25" s="42" t="s">
+      <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="71">
+      <c r="I25" s="72">
         <v>46188</v>
       </c>
-      <c r="J25" s="71"/>
-      <c r="K25" s="52"/>
+      <c r="J25" s="72"/>
+      <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="76"/>
-      <c r="B26" s="45" t="s">
+      <c r="A26" s="71"/>
+      <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="45">
         <v>46185</v>
       </c>
-      <c r="D26" s="46">
+      <c r="D26" s="45">
         <v>46188</v>
       </c>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="47">
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="46">
         <v>1</v>
       </c>
-      <c r="H26" s="45" t="s">
+      <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="76"/>
-      <c r="J26" s="72"/>
-      <c r="K26" s="53"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="73"/>
+      <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="75" t="s">
+      <c r="A27" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="39" t="s">
+      <c r="B27" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C27" s="40">
+      <c r="C27" s="39">
         <v>46234</v>
       </c>
-      <c r="D27" s="40">
+      <c r="D27" s="39">
         <v>46247</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="41">
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="40">
         <v>0</v>
       </c>
-      <c r="H27" s="39" t="s">
+      <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="71">
+      <c r="I27" s="72">
         <v>46321</v>
       </c>
-      <c r="J27" s="71"/>
-      <c r="K27" s="52"/>
+      <c r="J27" s="72"/>
+      <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="76"/>
-      <c r="B28" s="36" t="s">
+      <c r="A28" s="71"/>
+      <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="37">
+      <c r="C28" s="36">
         <v>46314</v>
       </c>
-      <c r="D28" s="37">
+      <c r="D28" s="36">
         <v>46316</v>
       </c>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="38">
+      <c r="E28" s="36"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="37">
         <v>0</v>
       </c>
-      <c r="H28" s="36" t="s">
+      <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="76"/>
-      <c r="J28" s="72"/>
-      <c r="K28" s="53"/>
+      <c r="I28" s="71"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="75" t="s">
+      <c r="A29" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="43">
+      <c r="C29" s="42">
         <v>46091</v>
       </c>
-      <c r="D29" s="43">
+      <c r="D29" s="42">
         <v>46100</v>
       </c>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="44">
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="43">
         <v>1</v>
       </c>
-      <c r="H29" s="42" t="s">
+      <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="71">
+      <c r="I29" s="72">
         <v>46139</v>
       </c>
-      <c r="J29" s="71"/>
-      <c r="K29" s="52"/>
+      <c r="J29" s="72"/>
+      <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="76"/>
-      <c r="B30" s="45" t="s">
+      <c r="A30" s="71"/>
+      <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="46">
+      <c r="C30" s="45">
         <v>46120</v>
       </c>
-      <c r="D30" s="46">
+      <c r="D30" s="45">
         <v>46124</v>
       </c>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="47">
+      <c r="E30" s="45"/>
+      <c r="F30" s="45"/>
+      <c r="G30" s="46">
         <v>1</v>
       </c>
-      <c r="H30" s="45" t="s">
+      <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="76"/>
-      <c r="J30" s="72"/>
-      <c r="K30" s="53"/>
+      <c r="I30" s="71"/>
+      <c r="J30" s="73"/>
+      <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="75" t="s">
+      <c r="A31" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="42" t="s">
+      <c r="B31" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C31" s="43">
+      <c r="C31" s="42">
         <v>46091</v>
       </c>
-      <c r="D31" s="43">
+      <c r="D31" s="42">
         <v>46094</v>
       </c>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="44">
+      <c r="E31" s="42"/>
+      <c r="F31" s="42"/>
+      <c r="G31" s="43">
         <v>1</v>
       </c>
-      <c r="H31" s="42" t="s">
+      <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="71">
+      <c r="I31" s="72">
         <v>46133</v>
       </c>
-      <c r="J31" s="71"/>
-      <c r="K31" s="52"/>
+      <c r="J31" s="72"/>
+      <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="76"/>
-      <c r="B32" s="45" t="s">
+      <c r="A32" s="71"/>
+      <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C32" s="46">
+      <c r="C32" s="45">
         <v>46091</v>
       </c>
-      <c r="D32" s="46">
+      <c r="D32" s="45">
         <v>46094</v>
       </c>
-      <c r="E32" s="46"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="47">
+      <c r="E32" s="45"/>
+      <c r="F32" s="45"/>
+      <c r="G32" s="46">
         <v>1</v>
       </c>
-      <c r="H32" s="45" t="s">
+      <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="76"/>
-      <c r="J32" s="72"/>
-      <c r="K32" s="53"/>
+      <c r="I32" s="71"/>
+      <c r="J32" s="73"/>
+      <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="75" t="s">
+      <c r="A33" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="39" t="s">
+      <c r="B33" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="62">
+      <c r="C33" s="61">
         <v>46237</v>
       </c>
-      <c r="D33" s="62">
+      <c r="D33" s="61">
         <v>46248</v>
       </c>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="41">
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="40">
         <v>0</v>
       </c>
-      <c r="H33" s="39" t="s">
+      <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="71">
+      <c r="I33" s="72">
         <v>46295</v>
       </c>
-      <c r="J33" s="71"/>
-      <c r="K33" s="52"/>
+      <c r="J33" s="72"/>
+      <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="76"/>
-      <c r="B34" s="36" t="s">
+      <c r="A34" s="71"/>
+      <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="63">
+      <c r="C34" s="62">
         <v>46296</v>
       </c>
-      <c r="D34" s="63">
+      <c r="D34" s="62">
         <v>46303</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="38">
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="37">
         <v>0</v>
       </c>
-      <c r="H34" s="36" t="s">
+      <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="76"/>
-      <c r="J34" s="72"/>
-      <c r="K34" s="53"/>
+      <c r="I34" s="71"/>
+      <c r="J34" s="73"/>
+      <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="75" t="s">
+      <c r="A35" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="39" t="s">
+      <c r="B35" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C35" s="40">
+      <c r="C35" s="39">
         <v>45723</v>
       </c>
-      <c r="D35" s="40">
+      <c r="D35" s="39">
         <v>45729</v>
       </c>
-      <c r="E35" s="40"/>
-      <c r="F35" s="40"/>
-      <c r="G35" s="41">
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="40">
         <v>1</v>
       </c>
-      <c r="H35" s="39" t="s">
+      <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="71">
+      <c r="I35" s="72">
         <v>45884</v>
       </c>
-      <c r="J35" s="71"/>
-      <c r="K35" s="52"/>
+      <c r="J35" s="72"/>
+      <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="76"/>
-      <c r="B36" s="36" t="s">
+      <c r="A36" s="71"/>
+      <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="37">
+      <c r="C36" s="36">
         <v>45729</v>
       </c>
-      <c r="D36" s="37">
+      <c r="D36" s="36">
         <v>45732</v>
       </c>
-      <c r="E36" s="37"/>
-      <c r="F36" s="37"/>
-      <c r="G36" s="38">
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="37">
         <v>0.9</v>
       </c>
-      <c r="H36" s="36" t="s">
+      <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="76"/>
-      <c r="J36" s="72"/>
-      <c r="K36" s="53"/>
+      <c r="I36" s="71"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="75" t="s">
+      <c r="A37" s="70" t="s">
         <v>32</v>
       </c>
-      <c r="B37" s="39" t="s">
+      <c r="B37" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="40">
+      <c r="C37" s="39">
         <v>45723</v>
       </c>
-      <c r="D37" s="40">
+      <c r="D37" s="39">
         <v>45729</v>
       </c>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="41">
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="40">
         <v>1</v>
       </c>
-      <c r="H37" s="39" t="s">
+      <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="71">
+      <c r="I37" s="72">
         <v>45915</v>
       </c>
-      <c r="J37" s="71"/>
-      <c r="K37" s="52"/>
+      <c r="J37" s="72"/>
+      <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="76"/>
-      <c r="B38" s="36" t="s">
+      <c r="A38" s="71"/>
+      <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="37">
+      <c r="C38" s="36">
         <v>45729</v>
       </c>
-      <c r="D38" s="37">
+      <c r="D38" s="36">
         <v>45862</v>
       </c>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="38">
+      <c r="E38" s="36"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="37">
         <v>0.9</v>
       </c>
-      <c r="H38" s="36" t="s">
+      <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="76"/>
-      <c r="J38" s="72"/>
-      <c r="K38" s="53"/>
+      <c r="I38" s="71"/>
+      <c r="J38" s="73"/>
+      <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="75" t="s">
+      <c r="A39" s="70" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="39" t="s">
+      <c r="B39" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="40"/>
-      <c r="D39" s="40"/>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="41">
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="40">
         <v>0</v>
       </c>
-      <c r="H39" s="39" t="s">
-        <v>139</v>
-      </c>
-      <c r="I39" s="71"/>
-      <c r="J39" s="71"/>
-      <c r="K39" s="52"/>
+      <c r="H39" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="I39" s="72"/>
+      <c r="J39" s="72"/>
+      <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="76"/>
-      <c r="B40" s="56" t="s">
+      <c r="A40" s="71"/>
+      <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C40" s="57"/>
-      <c r="D40" s="57"/>
-      <c r="E40" s="57"/>
-      <c r="F40" s="57"/>
-      <c r="G40" s="58">
+      <c r="C40" s="56"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="57">
         <v>0</v>
       </c>
-      <c r="H40" s="56" t="s">
-        <v>139</v>
-      </c>
-      <c r="I40" s="76"/>
-      <c r="J40" s="72"/>
-      <c r="K40" s="53"/>
+      <c r="H40" s="55" t="s">
+        <v>138</v>
+      </c>
+      <c r="I40" s="71"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="75" t="s">
+      <c r="A41" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="39" t="s">
+      <c r="B41" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="40">
+      <c r="C41" s="39">
         <v>46226</v>
       </c>
-      <c r="D41" s="40">
+      <c r="D41" s="39">
         <v>46228</v>
       </c>
-      <c r="E41" s="40"/>
-      <c r="F41" s="40"/>
-      <c r="G41" s="41">
-        <v>0.35</v>
-      </c>
-      <c r="H41" s="39" t="s">
+      <c r="E41" s="39"/>
+      <c r="F41" s="39"/>
+      <c r="G41" s="40">
+        <v>1</v>
+      </c>
+      <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="71">
-        <v>46230</v>
-      </c>
-      <c r="J41" s="71"/>
-      <c r="K41" s="52"/>
+      <c r="I41" s="72">
+        <v>46234</v>
+      </c>
+      <c r="J41" s="72"/>
+      <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="76"/>
-      <c r="B42" s="56" t="s">
+      <c r="A42" s="71"/>
+      <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C42" s="57"/>
-      <c r="D42" s="57"/>
-      <c r="E42" s="57"/>
-      <c r="F42" s="57"/>
-      <c r="G42" s="58"/>
-      <c r="H42" s="56"/>
-      <c r="I42" s="76"/>
-      <c r="J42" s="72"/>
-      <c r="K42" s="53"/>
+      <c r="C42" s="56"/>
+      <c r="D42" s="56"/>
+      <c r="E42" s="56"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="57"/>
+      <c r="H42" s="55"/>
+      <c r="I42" s="71"/>
+      <c r="J42" s="73"/>
+      <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="75" t="s">
-        <v>137</v>
-      </c>
-      <c r="B43" s="39" t="s">
+      <c r="A43" s="70" t="s">
+        <v>136</v>
+      </c>
+      <c r="B43" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C43" s="40"/>
-      <c r="D43" s="40"/>
-      <c r="E43" s="40"/>
-      <c r="F43" s="40"/>
-      <c r="G43" s="41">
+      <c r="C43" s="39"/>
+      <c r="D43" s="39"/>
+      <c r="E43" s="39"/>
+      <c r="F43" s="39"/>
+      <c r="G43" s="40">
         <v>0</v>
       </c>
-      <c r="H43" s="39" t="s">
-        <v>139</v>
-      </c>
-      <c r="I43" s="71"/>
-      <c r="J43" s="71"/>
-      <c r="K43" s="52"/>
+      <c r="H43" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="I43" s="72"/>
+      <c r="J43" s="72"/>
+      <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="76"/>
-      <c r="B44" s="56" t="s">
+      <c r="A44" s="71"/>
+      <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="57"/>
-      <c r="D44" s="57"/>
-      <c r="E44" s="57"/>
-      <c r="F44" s="57"/>
-      <c r="G44" s="58">
+      <c r="C44" s="56"/>
+      <c r="D44" s="56"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="56"/>
+      <c r="G44" s="57">
         <v>0</v>
       </c>
-      <c r="H44" s="56" t="s">
-        <v>139</v>
-      </c>
-      <c r="I44" s="76"/>
-      <c r="J44" s="72"/>
-      <c r="K44" s="53"/>
+      <c r="H44" s="55" t="s">
+        <v>138</v>
+      </c>
+      <c r="I44" s="71"/>
+      <c r="J44" s="73"/>
+      <c r="K44" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2459,43 +2484,15 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2532,56 +2529,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="T2" s="70"/>
-      <c r="U2" s="70"/>
-      <c r="V2" s="70"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="69"/>
+      <c r="V2" s="69"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -2702,10 +2699,10 @@
         <v>46106</v>
       </c>
       <c r="S5" s="14"/>
-      <c r="T5" s="26" t="s">
+      <c r="T5" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="U5" s="29" t="s">
+      <c r="U5" s="28" t="s">
         <v>80</v>
       </c>
       <c r="V5" s="19"/>
@@ -2761,10 +2758,10 @@
         <v>46264</v>
       </c>
       <c r="S6" s="14"/>
-      <c r="T6" s="26" t="s">
+      <c r="T6" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="U6" s="26"/>
+      <c r="U6" s="25"/>
       <c r="V6" s="19"/>
     </row>
     <row r="7" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
@@ -2819,10 +2816,10 @@
         <v>46219</v>
       </c>
       <c r="S7" s="14"/>
-      <c r="T7" s="26" t="s">
+      <c r="T7" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="U7" s="29" t="s">
+      <c r="U7" s="28" t="s">
         <v>81</v>
       </c>
       <c r="V7" s="19"/>
@@ -2879,8 +2876,8 @@
         <v>46244</v>
       </c>
       <c r="S8" s="14"/>
-      <c r="T8" s="26"/>
-      <c r="U8" s="31" t="s">
+      <c r="T8" s="25"/>
+      <c r="U8" s="30" t="s">
         <v>82</v>
       </c>
       <c r="V8" s="19">
@@ -2933,8 +2930,8 @@
         <v>46447</v>
       </c>
       <c r="S9" s="14"/>
-      <c r="T9" s="26"/>
-      <c r="U9" s="26"/>
+      <c r="T9" s="25"/>
+      <c r="U9" s="25"/>
       <c r="V9" s="19"/>
     </row>
     <row r="10" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
@@ -2990,8 +2987,8 @@
         <v>46199</v>
       </c>
       <c r="S10" s="14"/>
-      <c r="T10" s="27"/>
-      <c r="U10" s="31" t="s">
+      <c r="T10" s="26"/>
+      <c r="U10" s="30" t="s">
         <v>82</v>
       </c>
       <c r="V10" s="19">
@@ -3050,10 +3047,10 @@
         <v>46305</v>
       </c>
       <c r="S11" s="14"/>
-      <c r="T11" s="27" t="s">
+      <c r="T11" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="U11" s="31" t="s">
+      <c r="U11" s="30" t="s">
         <v>83</v>
       </c>
       <c r="V11" s="19">
@@ -3111,10 +3108,10 @@
         <v>46336</v>
       </c>
       <c r="S12" s="14"/>
-      <c r="T12" s="27" t="s">
+      <c r="T12" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="U12" s="26"/>
+      <c r="U12" s="25"/>
       <c r="V12" s="19">
         <v>46331</v>
       </c>
@@ -3165,10 +3162,10 @@
       <c r="R13" s="11">
         <v>46336</v>
       </c>
-      <c r="T13" s="26" t="s">
+      <c r="T13" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="U13" s="31" t="s">
+      <c r="U13" s="30" t="s">
         <v>84</v>
       </c>
       <c r="V13" s="19">
@@ -3185,7 +3182,7 @@
       <c r="C14" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="15">
         <v>1</v>
       </c>
       <c r="E14" s="16">
@@ -3224,10 +3221,10 @@
       <c r="R14" s="11">
         <v>46237</v>
       </c>
-      <c r="T14" s="27" t="s">
+      <c r="T14" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="U14" s="29" t="s">
+      <c r="U14" s="28" t="s">
         <v>70</v>
       </c>
       <c r="V14" s="19">
@@ -3284,8 +3281,8 @@
       <c r="R15" s="11">
         <v>46188</v>
       </c>
-      <c r="T15" s="28"/>
-      <c r="U15" s="26"/>
+      <c r="T15" s="27"/>
+      <c r="U15" s="25"/>
       <c r="V15" s="19">
         <v>46169</v>
       </c>
@@ -3337,10 +3334,10 @@
       <c r="R16" s="11">
         <v>46321</v>
       </c>
-      <c r="T16" s="26" t="s">
+      <c r="T16" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="U16" s="29" t="s">
+      <c r="U16" s="28" t="s">
         <v>85</v>
       </c>
       <c r="V16" s="19">
@@ -3374,7 +3371,7 @@
         <f>E17*1</f>
         <v>600000</v>
       </c>
-      <c r="I17" s="22">
+      <c r="I17" s="21">
         <v>10</v>
       </c>
       <c r="K17" s="14"/>
@@ -3396,8 +3393,8 @@
       <c r="R17" s="11">
         <v>46188</v>
       </c>
-      <c r="T17" s="28"/>
-      <c r="U17" s="26"/>
+      <c r="T17" s="27"/>
+      <c r="U17" s="25"/>
       <c r="V17" s="19">
         <v>46079</v>
       </c>
@@ -3427,7 +3424,7 @@
         <f>E18*1</f>
         <v>317648</v>
       </c>
-      <c r="I18" s="22">
+      <c r="I18" s="21">
         <v>10</v>
       </c>
       <c r="K18" s="14"/>
@@ -3449,8 +3446,8 @@
       <c r="R18" s="11">
         <v>46200</v>
       </c>
-      <c r="T18" s="28"/>
-      <c r="U18" s="26"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="25"/>
       <c r="V18" s="19"/>
     </row>
     <row r="19" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
@@ -3480,7 +3477,7 @@
         <f>455555</f>
         <v>455555</v>
       </c>
-      <c r="I19" s="22">
+      <c r="I19" s="21">
         <v>3</v>
       </c>
       <c r="K19" s="14"/>
@@ -3503,10 +3500,10 @@
       <c r="R19" s="11">
         <v>46295</v>
       </c>
-      <c r="T19" s="27" t="s">
+      <c r="T19" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="U19" s="32" t="s">
+      <c r="U19" s="31" t="s">
         <v>86</v>
       </c>
       <c r="V19" s="19">
@@ -3517,7 +3514,7 @@
       <c r="A20" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="22" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="14" t="s">
@@ -3526,8 +3523,8 @@
       <c r="D20" s="15">
         <v>0.9</v>
       </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="25"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="24"/>
       <c r="G20" s="9">
         <v>255</v>
       </c>
@@ -3548,17 +3545,17 @@
       <c r="R20" s="19">
         <v>45737</v>
       </c>
-      <c r="T20" s="27" t="s">
+      <c r="T20" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="U20" s="26"/>
+      <c r="U20" s="25"/>
       <c r="V20" s="19"/>
     </row>
     <row r="21" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
       <c r="A21" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="22" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="14" t="s">
@@ -3567,7 +3564,7 @@
       <c r="D21" s="15">
         <v>0.9</v>
       </c>
-      <c r="F21" s="25"/>
+      <c r="F21" s="24"/>
       <c r="I21" s="9">
         <v>6</v>
       </c>
@@ -3584,7 +3581,7 @@
       <c r="R21" s="19">
         <v>45737</v>
       </c>
-      <c r="T21" s="27" t="s">
+      <c r="T21" s="26" t="s">
         <v>126</v>
       </c>
       <c r="V21" s="19"/>
@@ -3593,14 +3590,14 @@
       <c r="A22" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="14" t="s">
         <v>89</v>
       </c>
       <c r="D22" s="15"/>
-      <c r="F22" s="25"/>
+      <c r="F22" s="24"/>
       <c r="G22" s="9">
         <v>2484</v>
       </c>
@@ -3610,7 +3607,7 @@
       <c r="P22" s="10"/>
       <c r="Q22" s="19"/>
       <c r="R22" s="19"/>
-      <c r="T22" s="27" t="s">
+      <c r="T22" s="26" t="s">
         <v>88</v>
       </c>
       <c r="V22" s="19"/>
@@ -3620,7 +3617,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>67</v>
@@ -3639,7 +3636,7 @@
         <f>E23*0.5</f>
         <v>230000</v>
       </c>
-      <c r="I23" s="22"/>
+      <c r="I23" s="21"/>
       <c r="K23" s="14"/>
       <c r="L23" s="16">
         <v>15000</v>
@@ -3652,8 +3649,8 @@
       </c>
       <c r="Q23" s="19"/>
       <c r="R23" s="11"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="32"/>
+      <c r="T23" s="26"/>
+      <c r="U23" s="31"/>
       <c r="V23" s="19">
         <v>46209</v>
       </c>
@@ -3669,7 +3666,7 @@
         <v>67</v>
       </c>
       <c r="D24" s="15">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="E24" s="16">
         <v>203880</v>
@@ -3685,14 +3682,14 @@
         <f>E24*0.4</f>
         <v>81552</v>
       </c>
-      <c r="I24" s="22">
+      <c r="I24" s="21">
         <v>6</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="16">
         <v>13500</v>
       </c>
-      <c r="N24" s="55">
+      <c r="N24" s="54">
         <v>497</v>
       </c>
       <c r="O24" s="9" t="s">
@@ -3705,12 +3702,12 @@
         <v>46225</v>
       </c>
       <c r="R24" s="11">
-        <v>46227</v>
-      </c>
-      <c r="T24" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="U24" s="32" t="s">
+        <v>46234</v>
+      </c>
+      <c r="T24" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="U24" s="31" t="s">
         <v>129</v>
       </c>
       <c r="V24" s="19">
@@ -3719,15 +3716,15 @@
     </row>
     <row r="25" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
       <c r="A25" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="67">
+      <c r="D25" s="66">
         <v>0</v>
       </c>
       <c r="E25" s="12">
@@ -3756,7 +3753,7 @@
         <v>384843</v>
       </c>
       <c r="T25" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="V25" s="19"/>
     </row>
@@ -4257,7 +4254,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4298,20 +4295,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4326,7 +4323,7 @@
       <c r="D4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="54" t="s">
+      <c r="E4" s="53" t="s">
         <v>90</v>
       </c>
     </row>
@@ -4666,37 +4663,37 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="66">
+      <c r="A26" s="65">
         <v>46219</v>
       </c>
-      <c r="B26" s="65" t="s">
+      <c r="B26" s="64" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="65" t="s">
+      <c r="C26" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="64">
+      <c r="D26" s="63">
         <v>3</v>
       </c>
       <c r="E26" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="3">
         <v>46224</v>
       </c>
-      <c r="B27" s="65" t="s">
+      <c r="B27" s="64" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="65" t="s">
+      <c r="C27" s="64" t="s">
         <v>61</v>
       </c>
       <c r="D27" s="4">
         <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -4706,14 +4703,14 @@
       <c r="B28" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="66" t="s">
+      <c r="C28" s="65" t="s">
         <v>61</v>
       </c>
       <c r="D28" s="4">
         <v>4</v>
       </c>
       <c r="E28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -4721,9 +4718,9 @@
         <v>46227</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C29" s="66" t="s">
+        <v>139</v>
+      </c>
+      <c r="C29" s="65" t="s">
         <v>61</v>
       </c>
       <c r="D29" s="4">
@@ -4740,14 +4737,14 @@
       <c r="B30" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="66" t="s">
+      <c r="C30" s="65" t="s">
         <v>61</v>
       </c>
       <c r="D30" s="4">
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -4771,22 +4768,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4858,10 +4855,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="C8" s="6">
         <v>46226</v>
@@ -4875,7 +4872,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="6">
@@ -5003,692 +5000,692 @@
       <c r="D28" s="3"/>
     </row>
     <row r="29" spans="1:4">
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
     </row>
     <row r="30" spans="1:4">
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
     </row>
     <row r="32" spans="1:4">
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
     </row>
     <row r="33" spans="3:4">
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
     </row>
     <row r="34" spans="3:4">
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
     </row>
     <row r="35" spans="3:4">
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
     </row>
     <row r="36" spans="3:4">
-      <c r="C36" s="30"/>
-      <c r="D36" s="30"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
     </row>
     <row r="37" spans="3:4">
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
     </row>
     <row r="38" spans="3:4">
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
     </row>
     <row r="39" spans="3:4">
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
     </row>
     <row r="40" spans="3:4">
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
     </row>
     <row r="41" spans="3:4">
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
     </row>
     <row r="42" spans="3:4">
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
     </row>
     <row r="43" spans="3:4">
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
     </row>
     <row r="44" spans="3:4">
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
     </row>
     <row r="45" spans="3:4">
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
     </row>
     <row r="46" spans="3:4">
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
     </row>
     <row r="47" spans="3:4">
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
     </row>
     <row r="48" spans="3:4">
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
     </row>
     <row r="49" spans="3:4">
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
     </row>
     <row r="50" spans="3:4">
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
     </row>
     <row r="51" spans="3:4">
-      <c r="C51" s="30"/>
-      <c r="D51" s="30"/>
+      <c r="C51" s="29"/>
+      <c r="D51" s="29"/>
     </row>
     <row r="52" spans="3:4">
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
+      <c r="C52" s="29"/>
+      <c r="D52" s="29"/>
     </row>
     <row r="53" spans="3:4">
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
     </row>
     <row r="54" spans="3:4">
-      <c r="C54" s="30"/>
-      <c r="D54" s="30"/>
+      <c r="C54" s="29"/>
+      <c r="D54" s="29"/>
     </row>
     <row r="55" spans="3:4">
-      <c r="C55" s="30"/>
-      <c r="D55" s="30"/>
+      <c r="C55" s="29"/>
+      <c r="D55" s="29"/>
     </row>
     <row r="56" spans="3:4">
-      <c r="C56" s="30"/>
-      <c r="D56" s="30"/>
+      <c r="C56" s="29"/>
+      <c r="D56" s="29"/>
     </row>
     <row r="57" spans="3:4">
-      <c r="C57" s="30"/>
-      <c r="D57" s="30"/>
+      <c r="C57" s="29"/>
+      <c r="D57" s="29"/>
     </row>
     <row r="58" spans="3:4">
-      <c r="C58" s="30"/>
-      <c r="D58" s="30"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
     </row>
     <row r="59" spans="3:4">
-      <c r="C59" s="30"/>
-      <c r="D59" s="30"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="29"/>
     </row>
     <row r="60" spans="3:4">
-      <c r="C60" s="30"/>
-      <c r="D60" s="30"/>
+      <c r="C60" s="29"/>
+      <c r="D60" s="29"/>
     </row>
     <row r="61" spans="3:4">
-      <c r="C61" s="30"/>
-      <c r="D61" s="30"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
     </row>
     <row r="62" spans="3:4">
-      <c r="C62" s="30"/>
-      <c r="D62" s="30"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="29"/>
     </row>
     <row r="63" spans="3:4">
-      <c r="C63" s="30"/>
-      <c r="D63" s="30"/>
+      <c r="C63" s="29"/>
+      <c r="D63" s="29"/>
     </row>
     <row r="64" spans="3:4">
-      <c r="C64" s="30"/>
-      <c r="D64" s="30"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
     </row>
     <row r="65" spans="3:4">
-      <c r="C65" s="30"/>
-      <c r="D65" s="30"/>
+      <c r="C65" s="29"/>
+      <c r="D65" s="29"/>
     </row>
     <row r="66" spans="3:4">
-      <c r="C66" s="30"/>
-      <c r="D66" s="30"/>
+      <c r="C66" s="29"/>
+      <c r="D66" s="29"/>
     </row>
     <row r="67" spans="3:4">
-      <c r="C67" s="30"/>
-      <c r="D67" s="30"/>
+      <c r="C67" s="29"/>
+      <c r="D67" s="29"/>
     </row>
     <row r="68" spans="3:4">
-      <c r="C68" s="30"/>
-      <c r="D68" s="30"/>
+      <c r="C68" s="29"/>
+      <c r="D68" s="29"/>
     </row>
     <row r="69" spans="3:4">
-      <c r="C69" s="30"/>
-      <c r="D69" s="30"/>
+      <c r="C69" s="29"/>
+      <c r="D69" s="29"/>
     </row>
     <row r="70" spans="3:4">
-      <c r="C70" s="30"/>
-      <c r="D70" s="30"/>
+      <c r="C70" s="29"/>
+      <c r="D70" s="29"/>
     </row>
     <row r="71" spans="3:4">
-      <c r="C71" s="30"/>
-      <c r="D71" s="30"/>
+      <c r="C71" s="29"/>
+      <c r="D71" s="29"/>
     </row>
     <row r="72" spans="3:4">
-      <c r="C72" s="30"/>
-      <c r="D72" s="30"/>
+      <c r="C72" s="29"/>
+      <c r="D72" s="29"/>
     </row>
     <row r="73" spans="3:4">
-      <c r="C73" s="30"/>
-      <c r="D73" s="30"/>
+      <c r="C73" s="29"/>
+      <c r="D73" s="29"/>
     </row>
     <row r="74" spans="3:4">
-      <c r="C74" s="30"/>
-      <c r="D74" s="30"/>
+      <c r="C74" s="29"/>
+      <c r="D74" s="29"/>
     </row>
     <row r="75" spans="3:4">
-      <c r="C75" s="30"/>
-      <c r="D75" s="30"/>
+      <c r="C75" s="29"/>
+      <c r="D75" s="29"/>
     </row>
     <row r="76" spans="3:4">
-      <c r="C76" s="30"/>
-      <c r="D76" s="30"/>
+      <c r="C76" s="29"/>
+      <c r="D76" s="29"/>
     </row>
     <row r="77" spans="3:4">
-      <c r="C77" s="30"/>
-      <c r="D77" s="30"/>
+      <c r="C77" s="29"/>
+      <c r="D77" s="29"/>
     </row>
     <row r="78" spans="3:4">
-      <c r="C78" s="30"/>
-      <c r="D78" s="30"/>
+      <c r="C78" s="29"/>
+      <c r="D78" s="29"/>
     </row>
     <row r="79" spans="3:4">
-      <c r="C79" s="30"/>
-      <c r="D79" s="30"/>
+      <c r="C79" s="29"/>
+      <c r="D79" s="29"/>
     </row>
     <row r="80" spans="3:4">
-      <c r="C80" s="30"/>
-      <c r="D80" s="30"/>
+      <c r="C80" s="29"/>
+      <c r="D80" s="29"/>
     </row>
     <row r="81" spans="3:4">
-      <c r="C81" s="30"/>
-      <c r="D81" s="30"/>
+      <c r="C81" s="29"/>
+      <c r="D81" s="29"/>
     </row>
     <row r="82" spans="3:4">
-      <c r="C82" s="30"/>
-      <c r="D82" s="30"/>
+      <c r="C82" s="29"/>
+      <c r="D82" s="29"/>
     </row>
     <row r="83" spans="3:4">
-      <c r="C83" s="30"/>
-      <c r="D83" s="30"/>
+      <c r="C83" s="29"/>
+      <c r="D83" s="29"/>
     </row>
     <row r="84" spans="3:4">
-      <c r="C84" s="30"/>
-      <c r="D84" s="30"/>
+      <c r="C84" s="29"/>
+      <c r="D84" s="29"/>
     </row>
     <row r="85" spans="3:4">
-      <c r="C85" s="30"/>
-      <c r="D85" s="30"/>
+      <c r="C85" s="29"/>
+      <c r="D85" s="29"/>
     </row>
     <row r="86" spans="3:4">
-      <c r="C86" s="30"/>
-      <c r="D86" s="30"/>
+      <c r="C86" s="29"/>
+      <c r="D86" s="29"/>
     </row>
     <row r="87" spans="3:4">
-      <c r="C87" s="30"/>
-      <c r="D87" s="30"/>
+      <c r="C87" s="29"/>
+      <c r="D87" s="29"/>
     </row>
     <row r="88" spans="3:4">
-      <c r="C88" s="30"/>
-      <c r="D88" s="30"/>
+      <c r="C88" s="29"/>
+      <c r="D88" s="29"/>
     </row>
     <row r="89" spans="3:4">
-      <c r="C89" s="30"/>
-      <c r="D89" s="30"/>
+      <c r="C89" s="29"/>
+      <c r="D89" s="29"/>
     </row>
     <row r="90" spans="3:4">
-      <c r="C90" s="30"/>
-      <c r="D90" s="30"/>
+      <c r="C90" s="29"/>
+      <c r="D90" s="29"/>
     </row>
     <row r="91" spans="3:4">
-      <c r="C91" s="30"/>
-      <c r="D91" s="30"/>
+      <c r="C91" s="29"/>
+      <c r="D91" s="29"/>
     </row>
     <row r="92" spans="3:4">
-      <c r="C92" s="30"/>
-      <c r="D92" s="30"/>
+      <c r="C92" s="29"/>
+      <c r="D92" s="29"/>
     </row>
     <row r="93" spans="3:4">
-      <c r="C93" s="30"/>
-      <c r="D93" s="30"/>
+      <c r="C93" s="29"/>
+      <c r="D93" s="29"/>
     </row>
     <row r="94" spans="3:4">
-      <c r="C94" s="30"/>
-      <c r="D94" s="30"/>
+      <c r="C94" s="29"/>
+      <c r="D94" s="29"/>
     </row>
     <row r="95" spans="3:4">
-      <c r="C95" s="30"/>
-      <c r="D95" s="30"/>
+      <c r="C95" s="29"/>
+      <c r="D95" s="29"/>
     </row>
     <row r="96" spans="3:4">
-      <c r="C96" s="30"/>
-      <c r="D96" s="30"/>
+      <c r="C96" s="29"/>
+      <c r="D96" s="29"/>
     </row>
     <row r="97" spans="3:4">
-      <c r="C97" s="30"/>
-      <c r="D97" s="30"/>
+      <c r="C97" s="29"/>
+      <c r="D97" s="29"/>
     </row>
     <row r="98" spans="3:4">
-      <c r="C98" s="30"/>
-      <c r="D98" s="30"/>
+      <c r="C98" s="29"/>
+      <c r="D98" s="29"/>
     </row>
     <row r="99" spans="3:4">
-      <c r="C99" s="30"/>
-      <c r="D99" s="30"/>
+      <c r="C99" s="29"/>
+      <c r="D99" s="29"/>
     </row>
     <row r="100" spans="3:4">
-      <c r="C100" s="30"/>
-      <c r="D100" s="30"/>
+      <c r="C100" s="29"/>
+      <c r="D100" s="29"/>
     </row>
     <row r="101" spans="3:4">
-      <c r="C101" s="30"/>
-      <c r="D101" s="30"/>
+      <c r="C101" s="29"/>
+      <c r="D101" s="29"/>
     </row>
     <row r="102" spans="3:4">
-      <c r="C102" s="30"/>
-      <c r="D102" s="30"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="29"/>
     </row>
     <row r="103" spans="3:4">
-      <c r="C103" s="30"/>
-      <c r="D103" s="30"/>
+      <c r="C103" s="29"/>
+      <c r="D103" s="29"/>
     </row>
     <row r="104" spans="3:4">
-      <c r="C104" s="30"/>
-      <c r="D104" s="30"/>
+      <c r="C104" s="29"/>
+      <c r="D104" s="29"/>
     </row>
     <row r="105" spans="3:4">
-      <c r="C105" s="30"/>
-      <c r="D105" s="30"/>
+      <c r="C105" s="29"/>
+      <c r="D105" s="29"/>
     </row>
     <row r="106" spans="3:4">
-      <c r="C106" s="30"/>
-      <c r="D106" s="30"/>
+      <c r="C106" s="29"/>
+      <c r="D106" s="29"/>
     </row>
     <row r="107" spans="3:4">
-      <c r="C107" s="30"/>
-      <c r="D107" s="30"/>
+      <c r="C107" s="29"/>
+      <c r="D107" s="29"/>
     </row>
     <row r="108" spans="3:4">
-      <c r="C108" s="30"/>
-      <c r="D108" s="30"/>
+      <c r="C108" s="29"/>
+      <c r="D108" s="29"/>
     </row>
     <row r="109" spans="3:4">
-      <c r="C109" s="30"/>
-      <c r="D109" s="30"/>
+      <c r="C109" s="29"/>
+      <c r="D109" s="29"/>
     </row>
     <row r="110" spans="3:4">
-      <c r="C110" s="30"/>
-      <c r="D110" s="30"/>
+      <c r="C110" s="29"/>
+      <c r="D110" s="29"/>
     </row>
     <row r="111" spans="3:4">
-      <c r="C111" s="30"/>
-      <c r="D111" s="30"/>
+      <c r="C111" s="29"/>
+      <c r="D111" s="29"/>
     </row>
     <row r="112" spans="3:4">
-      <c r="C112" s="30"/>
-      <c r="D112" s="30"/>
+      <c r="C112" s="29"/>
+      <c r="D112" s="29"/>
     </row>
     <row r="113" spans="3:4">
-      <c r="C113" s="30"/>
-      <c r="D113" s="30"/>
+      <c r="C113" s="29"/>
+      <c r="D113" s="29"/>
     </row>
     <row r="114" spans="3:4">
-      <c r="C114" s="30"/>
-      <c r="D114" s="30"/>
+      <c r="C114" s="29"/>
+      <c r="D114" s="29"/>
     </row>
     <row r="115" spans="3:4">
-      <c r="C115" s="30"/>
-      <c r="D115" s="30"/>
+      <c r="C115" s="29"/>
+      <c r="D115" s="29"/>
     </row>
     <row r="116" spans="3:4">
-      <c r="C116" s="30"/>
-      <c r="D116" s="30"/>
+      <c r="C116" s="29"/>
+      <c r="D116" s="29"/>
     </row>
     <row r="117" spans="3:4">
-      <c r="C117" s="30"/>
-      <c r="D117" s="30"/>
+      <c r="C117" s="29"/>
+      <c r="D117" s="29"/>
     </row>
     <row r="118" spans="3:4">
-      <c r="C118" s="30"/>
-      <c r="D118" s="30"/>
+      <c r="C118" s="29"/>
+      <c r="D118" s="29"/>
     </row>
     <row r="119" spans="3:4">
-      <c r="C119" s="30"/>
-      <c r="D119" s="30"/>
+      <c r="C119" s="29"/>
+      <c r="D119" s="29"/>
     </row>
     <row r="120" spans="3:4">
-      <c r="C120" s="30"/>
-      <c r="D120" s="30"/>
+      <c r="C120" s="29"/>
+      <c r="D120" s="29"/>
     </row>
     <row r="121" spans="3:4">
-      <c r="C121" s="30"/>
-      <c r="D121" s="30"/>
+      <c r="C121" s="29"/>
+      <c r="D121" s="29"/>
     </row>
     <row r="122" spans="3:4">
-      <c r="C122" s="30"/>
-      <c r="D122" s="30"/>
+      <c r="C122" s="29"/>
+      <c r="D122" s="29"/>
     </row>
     <row r="123" spans="3:4">
-      <c r="C123" s="30"/>
-      <c r="D123" s="30"/>
+      <c r="C123" s="29"/>
+      <c r="D123" s="29"/>
     </row>
     <row r="124" spans="3:4">
-      <c r="C124" s="30"/>
-      <c r="D124" s="30"/>
+      <c r="C124" s="29"/>
+      <c r="D124" s="29"/>
     </row>
     <row r="125" spans="3:4">
-      <c r="C125" s="30"/>
-      <c r="D125" s="30"/>
+      <c r="C125" s="29"/>
+      <c r="D125" s="29"/>
     </row>
     <row r="126" spans="3:4">
-      <c r="C126" s="30"/>
-      <c r="D126" s="30"/>
+      <c r="C126" s="29"/>
+      <c r="D126" s="29"/>
     </row>
     <row r="127" spans="3:4">
-      <c r="C127" s="30"/>
-      <c r="D127" s="30"/>
+      <c r="C127" s="29"/>
+      <c r="D127" s="29"/>
     </row>
     <row r="128" spans="3:4">
-      <c r="C128" s="30"/>
-      <c r="D128" s="30"/>
+      <c r="C128" s="29"/>
+      <c r="D128" s="29"/>
     </row>
     <row r="129" spans="3:4">
-      <c r="C129" s="30"/>
-      <c r="D129" s="30"/>
+      <c r="C129" s="29"/>
+      <c r="D129" s="29"/>
     </row>
     <row r="130" spans="3:4">
-      <c r="C130" s="30"/>
-      <c r="D130" s="30"/>
+      <c r="C130" s="29"/>
+      <c r="D130" s="29"/>
     </row>
     <row r="131" spans="3:4">
-      <c r="C131" s="30"/>
-      <c r="D131" s="30"/>
+      <c r="C131" s="29"/>
+      <c r="D131" s="29"/>
     </row>
     <row r="132" spans="3:4">
-      <c r="C132" s="30"/>
-      <c r="D132" s="30"/>
+      <c r="C132" s="29"/>
+      <c r="D132" s="29"/>
     </row>
     <row r="133" spans="3:4">
-      <c r="C133" s="30"/>
-      <c r="D133" s="30"/>
+      <c r="C133" s="29"/>
+      <c r="D133" s="29"/>
     </row>
     <row r="134" spans="3:4">
-      <c r="C134" s="30"/>
-      <c r="D134" s="30"/>
+      <c r="C134" s="29"/>
+      <c r="D134" s="29"/>
     </row>
     <row r="135" spans="3:4">
-      <c r="C135" s="30"/>
-      <c r="D135" s="30"/>
+      <c r="C135" s="29"/>
+      <c r="D135" s="29"/>
     </row>
     <row r="136" spans="3:4">
-      <c r="C136" s="30"/>
-      <c r="D136" s="30"/>
+      <c r="C136" s="29"/>
+      <c r="D136" s="29"/>
     </row>
     <row r="137" spans="3:4">
-      <c r="C137" s="30"/>
-      <c r="D137" s="30"/>
+      <c r="C137" s="29"/>
+      <c r="D137" s="29"/>
     </row>
     <row r="138" spans="3:4">
-      <c r="C138" s="30"/>
-      <c r="D138" s="30"/>
+      <c r="C138" s="29"/>
+      <c r="D138" s="29"/>
     </row>
     <row r="139" spans="3:4">
-      <c r="C139" s="30"/>
-      <c r="D139" s="30"/>
+      <c r="C139" s="29"/>
+      <c r="D139" s="29"/>
     </row>
     <row r="140" spans="3:4">
-      <c r="C140" s="30"/>
-      <c r="D140" s="30"/>
+      <c r="C140" s="29"/>
+      <c r="D140" s="29"/>
     </row>
     <row r="141" spans="3:4">
-      <c r="C141" s="30"/>
-      <c r="D141" s="30"/>
+      <c r="C141" s="29"/>
+      <c r="D141" s="29"/>
     </row>
     <row r="142" spans="3:4">
-      <c r="C142" s="30"/>
-      <c r="D142" s="30"/>
+      <c r="C142" s="29"/>
+      <c r="D142" s="29"/>
     </row>
     <row r="143" spans="3:4">
-      <c r="C143" s="30"/>
-      <c r="D143" s="30"/>
+      <c r="C143" s="29"/>
+      <c r="D143" s="29"/>
     </row>
     <row r="144" spans="3:4">
-      <c r="C144" s="30"/>
-      <c r="D144" s="30"/>
+      <c r="C144" s="29"/>
+      <c r="D144" s="29"/>
     </row>
     <row r="145" spans="3:4">
-      <c r="C145" s="30"/>
-      <c r="D145" s="30"/>
+      <c r="C145" s="29"/>
+      <c r="D145" s="29"/>
     </row>
     <row r="146" spans="3:4">
-      <c r="C146" s="30"/>
-      <c r="D146" s="30"/>
+      <c r="C146" s="29"/>
+      <c r="D146" s="29"/>
     </row>
     <row r="147" spans="3:4">
-      <c r="C147" s="30"/>
-      <c r="D147" s="30"/>
+      <c r="C147" s="29"/>
+      <c r="D147" s="29"/>
     </row>
     <row r="148" spans="3:4">
-      <c r="C148" s="30"/>
-      <c r="D148" s="30"/>
+      <c r="C148" s="29"/>
+      <c r="D148" s="29"/>
     </row>
     <row r="149" spans="3:4">
-      <c r="C149" s="30"/>
-      <c r="D149" s="30"/>
+      <c r="C149" s="29"/>
+      <c r="D149" s="29"/>
     </row>
     <row r="150" spans="3:4">
-      <c r="C150" s="30"/>
-      <c r="D150" s="30"/>
+      <c r="C150" s="29"/>
+      <c r="D150" s="29"/>
     </row>
     <row r="151" spans="3:4">
-      <c r="C151" s="30"/>
-      <c r="D151" s="30"/>
+      <c r="C151" s="29"/>
+      <c r="D151" s="29"/>
     </row>
     <row r="152" spans="3:4">
-      <c r="C152" s="30"/>
-      <c r="D152" s="30"/>
+      <c r="C152" s="29"/>
+      <c r="D152" s="29"/>
     </row>
     <row r="153" spans="3:4">
-      <c r="C153" s="30"/>
-      <c r="D153" s="30"/>
+      <c r="C153" s="29"/>
+      <c r="D153" s="29"/>
     </row>
     <row r="154" spans="3:4">
-      <c r="C154" s="30"/>
-      <c r="D154" s="30"/>
+      <c r="C154" s="29"/>
+      <c r="D154" s="29"/>
     </row>
     <row r="155" spans="3:4">
-      <c r="C155" s="30"/>
-      <c r="D155" s="30"/>
+      <c r="C155" s="29"/>
+      <c r="D155" s="29"/>
     </row>
     <row r="156" spans="3:4">
-      <c r="C156" s="30"/>
-      <c r="D156" s="30"/>
+      <c r="C156" s="29"/>
+      <c r="D156" s="29"/>
     </row>
     <row r="157" spans="3:4">
-      <c r="C157" s="30"/>
-      <c r="D157" s="30"/>
+      <c r="C157" s="29"/>
+      <c r="D157" s="29"/>
     </row>
     <row r="158" spans="3:4">
-      <c r="C158" s="30"/>
-      <c r="D158" s="30"/>
+      <c r="C158" s="29"/>
+      <c r="D158" s="29"/>
     </row>
     <row r="159" spans="3:4">
-      <c r="C159" s="30"/>
-      <c r="D159" s="30"/>
+      <c r="C159" s="29"/>
+      <c r="D159" s="29"/>
     </row>
     <row r="160" spans="3:4">
-      <c r="C160" s="30"/>
-      <c r="D160" s="30"/>
+      <c r="C160" s="29"/>
+      <c r="D160" s="29"/>
     </row>
     <row r="161" spans="3:4">
-      <c r="C161" s="30"/>
-      <c r="D161" s="30"/>
+      <c r="C161" s="29"/>
+      <c r="D161" s="29"/>
     </row>
     <row r="162" spans="3:4">
-      <c r="C162" s="30"/>
-      <c r="D162" s="30"/>
+      <c r="C162" s="29"/>
+      <c r="D162" s="29"/>
     </row>
     <row r="163" spans="3:4">
-      <c r="C163" s="30"/>
-      <c r="D163" s="30"/>
+      <c r="C163" s="29"/>
+      <c r="D163" s="29"/>
     </row>
     <row r="164" spans="3:4">
-      <c r="C164" s="30"/>
-      <c r="D164" s="30"/>
+      <c r="C164" s="29"/>
+      <c r="D164" s="29"/>
     </row>
     <row r="165" spans="3:4">
-      <c r="C165" s="30"/>
-      <c r="D165" s="30"/>
+      <c r="C165" s="29"/>
+      <c r="D165" s="29"/>
     </row>
     <row r="166" spans="3:4">
-      <c r="C166" s="30"/>
-      <c r="D166" s="30"/>
+      <c r="C166" s="29"/>
+      <c r="D166" s="29"/>
     </row>
     <row r="167" spans="3:4">
-      <c r="C167" s="30"/>
-      <c r="D167" s="30"/>
+      <c r="C167" s="29"/>
+      <c r="D167" s="29"/>
     </row>
     <row r="168" spans="3:4">
-      <c r="C168" s="30"/>
-      <c r="D168" s="30"/>
+      <c r="C168" s="29"/>
+      <c r="D168" s="29"/>
     </row>
     <row r="169" spans="3:4">
-      <c r="C169" s="30"/>
-      <c r="D169" s="30"/>
+      <c r="C169" s="29"/>
+      <c r="D169" s="29"/>
     </row>
     <row r="170" spans="3:4">
-      <c r="C170" s="30"/>
-      <c r="D170" s="30"/>
+      <c r="C170" s="29"/>
+      <c r="D170" s="29"/>
     </row>
     <row r="171" spans="3:4">
-      <c r="C171" s="30"/>
-      <c r="D171" s="30"/>
+      <c r="C171" s="29"/>
+      <c r="D171" s="29"/>
     </row>
     <row r="172" spans="3:4">
-      <c r="C172" s="30"/>
-      <c r="D172" s="30"/>
+      <c r="C172" s="29"/>
+      <c r="D172" s="29"/>
     </row>
     <row r="173" spans="3:4">
-      <c r="C173" s="30"/>
-      <c r="D173" s="30"/>
+      <c r="C173" s="29"/>
+      <c r="D173" s="29"/>
     </row>
     <row r="174" spans="3:4">
-      <c r="C174" s="30"/>
-      <c r="D174" s="30"/>
+      <c r="C174" s="29"/>
+      <c r="D174" s="29"/>
     </row>
     <row r="175" spans="3:4">
-      <c r="C175" s="30"/>
-      <c r="D175" s="30"/>
+      <c r="C175" s="29"/>
+      <c r="D175" s="29"/>
     </row>
     <row r="176" spans="3:4">
-      <c r="C176" s="30"/>
-      <c r="D176" s="30"/>
+      <c r="C176" s="29"/>
+      <c r="D176" s="29"/>
     </row>
     <row r="177" spans="3:4">
-      <c r="C177" s="30"/>
-      <c r="D177" s="30"/>
+      <c r="C177" s="29"/>
+      <c r="D177" s="29"/>
     </row>
     <row r="178" spans="3:4">
-      <c r="C178" s="30"/>
-      <c r="D178" s="30"/>
+      <c r="C178" s="29"/>
+      <c r="D178" s="29"/>
     </row>
     <row r="179" spans="3:4">
-      <c r="C179" s="30"/>
-      <c r="D179" s="30"/>
+      <c r="C179" s="29"/>
+      <c r="D179" s="29"/>
     </row>
     <row r="180" spans="3:4">
-      <c r="C180" s="30"/>
-      <c r="D180" s="30"/>
+      <c r="C180" s="29"/>
+      <c r="D180" s="29"/>
     </row>
     <row r="181" spans="3:4">
-      <c r="C181" s="30"/>
-      <c r="D181" s="30"/>
+      <c r="C181" s="29"/>
+      <c r="D181" s="29"/>
     </row>
     <row r="182" spans="3:4">
-      <c r="C182" s="30"/>
-      <c r="D182" s="30"/>
+      <c r="C182" s="29"/>
+      <c r="D182" s="29"/>
     </row>
     <row r="183" spans="3:4">
-      <c r="C183" s="30"/>
-      <c r="D183" s="30"/>
+      <c r="C183" s="29"/>
+      <c r="D183" s="29"/>
     </row>
     <row r="184" spans="3:4">
-      <c r="C184" s="30"/>
-      <c r="D184" s="30"/>
+      <c r="C184" s="29"/>
+      <c r="D184" s="29"/>
     </row>
     <row r="185" spans="3:4">
-      <c r="C185" s="30"/>
-      <c r="D185" s="30"/>
+      <c r="C185" s="29"/>
+      <c r="D185" s="29"/>
     </row>
     <row r="186" spans="3:4">
-      <c r="C186" s="30"/>
-      <c r="D186" s="30"/>
+      <c r="C186" s="29"/>
+      <c r="D186" s="29"/>
     </row>
     <row r="187" spans="3:4">
-      <c r="C187" s="30"/>
-      <c r="D187" s="30"/>
+      <c r="C187" s="29"/>
+      <c r="D187" s="29"/>
     </row>
     <row r="188" spans="3:4">
-      <c r="C188" s="30"/>
-      <c r="D188" s="30"/>
+      <c r="C188" s="29"/>
+      <c r="D188" s="29"/>
     </row>
     <row r="189" spans="3:4">
-      <c r="C189" s="30"/>
-      <c r="D189" s="30"/>
+      <c r="C189" s="29"/>
+      <c r="D189" s="29"/>
     </row>
     <row r="190" spans="3:4">
-      <c r="C190" s="30"/>
-      <c r="D190" s="30"/>
+      <c r="C190" s="29"/>
+      <c r="D190" s="29"/>
     </row>
     <row r="191" spans="3:4">
-      <c r="C191" s="30"/>
-      <c r="D191" s="30"/>
+      <c r="C191" s="29"/>
+      <c r="D191" s="29"/>
     </row>
     <row r="192" spans="3:4">
-      <c r="C192" s="30"/>
-      <c r="D192" s="30"/>
+      <c r="C192" s="29"/>
+      <c r="D192" s="29"/>
     </row>
     <row r="193" spans="3:4">
-      <c r="C193" s="30"/>
-      <c r="D193" s="30"/>
+      <c r="C193" s="29"/>
+      <c r="D193" s="29"/>
     </row>
     <row r="194" spans="3:4">
-      <c r="C194" s="30"/>
-      <c r="D194" s="30"/>
+      <c r="C194" s="29"/>
+      <c r="D194" s="29"/>
     </row>
     <row r="195" spans="3:4">
-      <c r="C195" s="30"/>
-      <c r="D195" s="30"/>
+      <c r="C195" s="29"/>
+      <c r="D195" s="29"/>
     </row>
     <row r="196" spans="3:4">
-      <c r="C196" s="30"/>
-      <c r="D196" s="30"/>
+      <c r="C196" s="29"/>
+      <c r="D196" s="29"/>
     </row>
     <row r="197" spans="3:4">
-      <c r="C197" s="30"/>
-      <c r="D197" s="30"/>
+      <c r="C197" s="29"/>
+      <c r="D197" s="29"/>
     </row>
     <row r="198" spans="3:4">
-      <c r="C198" s="30"/>
-      <c r="D198" s="30"/>
+      <c r="C198" s="29"/>
+      <c r="D198" s="29"/>
     </row>
     <row r="199" spans="3:4">
-      <c r="C199" s="30"/>
-      <c r="D199" s="30"/>
+      <c r="C199" s="29"/>
+      <c r="D199" s="29"/>
     </row>
     <row r="200" spans="3:4">
-      <c r="C200" s="30"/>
-      <c r="D200" s="30"/>
+      <c r="C200" s="29"/>
+      <c r="D200" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5705,6 +5702,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5715,15 +5721,6 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5980,20 +5977,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-27 10:29)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5E2E3CC-A260-4216-891E-591C22F5C5DB}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E6AC9C9-F318-4838-B7C2-7323EB448754}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -993,29 +993,29 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1396,31 +1396,31 @@
       <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="76"/>
+      <c r="J2" s="76"/>
+      <c r="K2" s="76"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1458,7 +1458,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="77" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
@@ -1478,14 +1478,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="77">
+      <c r="I5" s="71">
         <v>46244</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="71"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="71"/>
+      <c r="A6" s="74"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1503,12 +1503,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="71"/>
-      <c r="J6" s="73"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="70"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="73" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1528,14 +1528,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="72" t="s">
+      <c r="I7" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="72"/>
+      <c r="J7" s="69"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="71"/>
+      <c r="A8" s="74"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1553,12 +1553,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="71"/>
-      <c r="J8" s="73"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="70"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="70" t="s">
+      <c r="A9" s="73" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1578,14 +1578,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="72">
+      <c r="I9" s="69">
         <v>46218</v>
       </c>
-      <c r="J9" s="72"/>
+      <c r="J9" s="69"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="71"/>
+      <c r="A10" s="74"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1603,12 +1603,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="71"/>
-      <c r="J10" s="73"/>
+      <c r="I10" s="74"/>
+      <c r="J10" s="70"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="73" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1628,14 +1628,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="72">
+      <c r="I11" s="69">
         <v>46171</v>
       </c>
-      <c r="J11" s="72"/>
+      <c r="J11" s="69"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="71"/>
+      <c r="A12" s="74"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1653,12 +1653,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="71"/>
-      <c r="J12" s="73"/>
+      <c r="I12" s="74"/>
+      <c r="J12" s="70"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="70" t="s">
+      <c r="A13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1678,14 +1678,14 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="72" t="s">
+      <c r="I13" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="72"/>
+      <c r="J13" s="69"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="71"/>
+      <c r="A14" s="74"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1703,12 +1703,12 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="71"/>
-      <c r="J14" s="73"/>
+      <c r="I14" s="74"/>
+      <c r="J14" s="70"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="70" t="s">
+      <c r="A15" s="73" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1728,14 +1728,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="72">
+      <c r="I15" s="69">
         <v>46199</v>
       </c>
-      <c r="J15" s="72"/>
+      <c r="J15" s="69"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="71"/>
+      <c r="A16" s="74"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1753,8 +1753,8 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="71"/>
-      <c r="J16" s="73"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="70"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11">
@@ -1778,14 +1778,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="74">
+      <c r="I17" s="72">
         <v>46305</v>
       </c>
-      <c r="J17" s="74"/>
+      <c r="J17" s="72"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="71"/>
+      <c r="A18" s="74"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1803,8 +1803,8 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="71"/>
-      <c r="J18" s="73"/>
+      <c r="I18" s="74"/>
+      <c r="J18" s="70"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11">
@@ -1828,14 +1828,14 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="74">
+      <c r="I19" s="72">
         <v>46336</v>
       </c>
-      <c r="J19" s="74"/>
+      <c r="J19" s="72"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="71"/>
+      <c r="A20" s="74"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1853,12 +1853,12 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="71"/>
-      <c r="J20" s="73"/>
+      <c r="I20" s="74"/>
+      <c r="J20" s="70"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="70" t="s">
+      <c r="A21" s="73" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1878,14 +1878,14 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="72">
+      <c r="I21" s="69">
         <v>46336</v>
       </c>
-      <c r="J21" s="72"/>
+      <c r="J21" s="69"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="71"/>
+      <c r="A22" s="74"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1903,12 +1903,12 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="71"/>
-      <c r="J22" s="73"/>
+      <c r="I22" s="74"/>
+      <c r="J22" s="70"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="70" t="s">
+      <c r="A23" s="73" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -1928,14 +1928,14 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="72">
+      <c r="I23" s="69">
         <v>46237</v>
       </c>
-      <c r="J23" s="72"/>
+      <c r="J23" s="69"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="71"/>
+      <c r="A24" s="74"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -1953,12 +1953,12 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="71"/>
-      <c r="J24" s="73"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="70"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="70" t="s">
+      <c r="A25" s="73" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -1978,14 +1978,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="72">
+      <c r="I25" s="69">
         <v>46188</v>
       </c>
-      <c r="J25" s="72"/>
+      <c r="J25" s="69"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="71"/>
+      <c r="A26" s="74"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2003,12 +2003,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="71"/>
-      <c r="J26" s="73"/>
+      <c r="I26" s="74"/>
+      <c r="J26" s="70"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="70" t="s">
+      <c r="A27" s="73" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2028,14 +2028,14 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="72">
+      <c r="I27" s="69">
         <v>46321</v>
       </c>
-      <c r="J27" s="72"/>
+      <c r="J27" s="69"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="71"/>
+      <c r="A28" s="74"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2053,12 +2053,12 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="71"/>
-      <c r="J28" s="73"/>
+      <c r="I28" s="74"/>
+      <c r="J28" s="70"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="70" t="s">
+      <c r="A29" s="73" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2078,14 +2078,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="72">
+      <c r="I29" s="69">
         <v>46139</v>
       </c>
-      <c r="J29" s="72"/>
+      <c r="J29" s="69"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="71"/>
+      <c r="A30" s="74"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2103,12 +2103,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="71"/>
-      <c r="J30" s="73"/>
+      <c r="I30" s="74"/>
+      <c r="J30" s="70"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="70" t="s">
+      <c r="A31" s="73" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2128,14 +2128,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="72">
+      <c r="I31" s="69">
         <v>46133</v>
       </c>
-      <c r="J31" s="72"/>
+      <c r="J31" s="69"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="71"/>
+      <c r="A32" s="74"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2153,12 +2153,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="71"/>
-      <c r="J32" s="73"/>
+      <c r="I32" s="74"/>
+      <c r="J32" s="70"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="70" t="s">
+      <c r="A33" s="73" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2178,14 +2178,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="72">
+      <c r="I33" s="69">
         <v>46295</v>
       </c>
-      <c r="J33" s="72"/>
+      <c r="J33" s="69"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="71"/>
+      <c r="A34" s="74"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2203,12 +2203,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="71"/>
-      <c r="J34" s="73"/>
+      <c r="I34" s="74"/>
+      <c r="J34" s="70"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="70" t="s">
+      <c r="A35" s="73" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2228,14 +2228,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="72">
+      <c r="I35" s="69">
         <v>45884</v>
       </c>
-      <c r="J35" s="72"/>
+      <c r="J35" s="69"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="71"/>
+      <c r="A36" s="74"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2253,12 +2253,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="71"/>
-      <c r="J36" s="73"/>
+      <c r="I36" s="74"/>
+      <c r="J36" s="70"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="70" t="s">
+      <c r="A37" s="73" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2278,14 +2278,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="72">
+      <c r="I37" s="69">
         <v>45915</v>
       </c>
-      <c r="J37" s="72"/>
+      <c r="J37" s="69"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="71"/>
+      <c r="A38" s="74"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2303,12 +2303,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="71"/>
-      <c r="J38" s="73"/>
+      <c r="I38" s="74"/>
+      <c r="J38" s="70"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="70" t="s">
+      <c r="A39" s="73" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2324,12 +2324,12 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="72"/>
-      <c r="J39" s="72"/>
+      <c r="I39" s="69"/>
+      <c r="J39" s="69"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="71"/>
+      <c r="A40" s="74"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2343,12 +2343,12 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="71"/>
-      <c r="J40" s="73"/>
+      <c r="I40" s="74"/>
+      <c r="J40" s="70"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="70" t="s">
+      <c r="A41" s="73" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2368,14 +2368,14 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="72">
+      <c r="I41" s="69">
         <v>46234</v>
       </c>
-      <c r="J41" s="72"/>
+      <c r="J41" s="69"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="71"/>
+      <c r="A42" s="74"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2385,12 +2385,12 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="71"/>
-      <c r="J42" s="73"/>
+      <c r="I42" s="74"/>
+      <c r="J42" s="70"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="70" t="s">
+      <c r="A43" s="73" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
@@ -2404,14 +2404,14 @@
         <v>0</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="I43" s="72"/>
-      <c r="J43" s="72"/>
+        <v>22</v>
+      </c>
+      <c r="I43" s="69"/>
+      <c r="J43" s="69"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="71"/>
+      <c r="A44" s="74"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2423,28 +2423,46 @@
         <v>0</v>
       </c>
       <c r="H44" s="55" t="s">
-        <v>138</v>
-      </c>
-      <c r="I44" s="71"/>
-      <c r="J44" s="73"/>
+        <v>22</v>
+      </c>
+      <c r="I44" s="74"/>
+      <c r="J44" s="70"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2461,40 +2479,22 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -2555,30 +2555,30 @@
       <c r="V1" s="67"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
-      <c r="V2" s="69"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="68"/>
+      <c r="P2" s="68"/>
+      <c r="Q2" s="68"/>
+      <c r="R2" s="68"/>
+      <c r="S2" s="68"/>
+      <c r="T2" s="68"/>
+      <c r="U2" s="68"/>
+      <c r="V2" s="68"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -3617,7 +3617,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>138</v>
+        <v>22</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>67</v>
@@ -3719,7 +3719,7 @@
         <v>136</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>138</v>
+        <v>22</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>67</v>
@@ -4299,16 +4299,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="67"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4777,13 +4777,13 @@
       <c r="E1" s="67"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5702,15 +5702,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5721,6 +5712,15 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5977,20 +5977,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-30 15:16)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E6AC9C9-F318-4838-B7C2-7323EB448754}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFD90073-5B89-4B92-979D-15C2FE4D8674}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,12 @@
   <externalReferences>
     <externalReference r:id="rId5"/>
   </externalReferences>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Internal Work'!$A$4:$E$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Schedule'!$A$4:$K$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Site Visit Log'!$A$4:$E$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary Report'!$A$4:$V$189</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="143">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -464,10 +470,13 @@
     <t>Huaykwang residence</t>
   </si>
   <si>
-    <t>ส่งมอบงานงวดสุดท้าย</t>
-  </si>
-  <si>
     <t>คิดงานเพิ่ม 3000 บาท ค่ากล่องพรีนัม ส่งงานวันที่ 07/31/2026</t>
+  </si>
+  <si>
+    <t>ประชุม,คุยงานนัด Owner เข้า Pretest</t>
+  </si>
+  <si>
+    <t>บริษัท อีโค่คูล ไครลเมท เทคโนโลยี จำกัด</t>
   </si>
 </sst>
 </file>
@@ -994,28 +1003,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1396,31 +1405,31 @@
       <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1458,7 +1467,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="76" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
@@ -1478,14 +1487,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="71">
+      <c r="I5" s="77">
         <v>46244</v>
       </c>
-      <c r="J5" s="71"/>
+      <c r="J5" s="77"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="74"/>
+      <c r="A6" s="70"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1503,12 +1512,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="74"/>
-      <c r="J6" s="70"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="72"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="69" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1528,14 +1537,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="69" t="s">
+      <c r="I7" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="69"/>
+      <c r="J7" s="71"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="74"/>
+      <c r="A8" s="70"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1553,12 +1562,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="74"/>
-      <c r="J8" s="70"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="72"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="73" t="s">
+      <c r="A9" s="69" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1578,14 +1587,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="69">
+      <c r="I9" s="71">
         <v>46218</v>
       </c>
-      <c r="J9" s="69"/>
+      <c r="J9" s="71"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="74"/>
+      <c r="A10" s="70"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1603,12 +1612,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="74"/>
-      <c r="J10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="72"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="69" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1628,14 +1637,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="69">
+      <c r="I11" s="71">
         <v>46171</v>
       </c>
-      <c r="J11" s="69"/>
+      <c r="J11" s="71"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="74"/>
+      <c r="A12" s="70"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1653,12 +1662,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="74"/>
-      <c r="J12" s="70"/>
+      <c r="I12" s="70"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="73" t="s">
+      <c r="A13" s="69" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1678,14 +1687,14 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="69" t="s">
+      <c r="I13" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="69"/>
+      <c r="J13" s="71"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="74"/>
+      <c r="A14" s="70"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1703,12 +1712,12 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="74"/>
-      <c r="J14" s="70"/>
+      <c r="I14" s="70"/>
+      <c r="J14" s="72"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="69" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1728,14 +1737,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="69">
+      <c r="I15" s="71">
         <v>46199</v>
       </c>
-      <c r="J15" s="69"/>
+      <c r="J15" s="71"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="74"/>
+      <c r="A16" s="70"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1753,8 +1762,8 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="74"/>
-      <c r="J16" s="70"/>
+      <c r="I16" s="70"/>
+      <c r="J16" s="72"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11">
@@ -1778,14 +1787,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="72">
+      <c r="I17" s="74">
         <v>46305</v>
       </c>
-      <c r="J17" s="72"/>
+      <c r="J17" s="74"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="74"/>
+      <c r="A18" s="70"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1803,8 +1812,8 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="74"/>
-      <c r="J18" s="70"/>
+      <c r="I18" s="70"/>
+      <c r="J18" s="72"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11">
@@ -1828,14 +1837,14 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="72">
+      <c r="I19" s="74">
         <v>46336</v>
       </c>
-      <c r="J19" s="72"/>
+      <c r="J19" s="74"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="74"/>
+      <c r="A20" s="70"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1853,12 +1862,12 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="74"/>
-      <c r="J20" s="70"/>
+      <c r="I20" s="70"/>
+      <c r="J20" s="72"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="73" t="s">
+      <c r="A21" s="69" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1878,14 +1887,14 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="69">
+      <c r="I21" s="71">
         <v>46336</v>
       </c>
-      <c r="J21" s="69"/>
+      <c r="J21" s="71"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="74"/>
+      <c r="A22" s="70"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1903,12 +1912,12 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="74"/>
-      <c r="J22" s="70"/>
+      <c r="I22" s="70"/>
+      <c r="J22" s="72"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="73" t="s">
+      <c r="A23" s="69" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -1928,14 +1937,14 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="69">
+      <c r="I23" s="71">
         <v>46237</v>
       </c>
-      <c r="J23" s="69"/>
+      <c r="J23" s="71"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="74"/>
+      <c r="A24" s="70"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -1953,12 +1962,12 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="74"/>
-      <c r="J24" s="70"/>
+      <c r="I24" s="70"/>
+      <c r="J24" s="72"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="73" t="s">
+      <c r="A25" s="69" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -1978,14 +1987,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="69">
+      <c r="I25" s="71">
         <v>46188</v>
       </c>
-      <c r="J25" s="69"/>
+      <c r="J25" s="71"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="74"/>
+      <c r="A26" s="70"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2003,12 +2012,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="74"/>
-      <c r="J26" s="70"/>
+      <c r="I26" s="70"/>
+      <c r="J26" s="72"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="73" t="s">
+      <c r="A27" s="69" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2028,14 +2037,14 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="69">
+      <c r="I27" s="71">
         <v>46321</v>
       </c>
-      <c r="J27" s="69"/>
+      <c r="J27" s="71"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="74"/>
+      <c r="A28" s="70"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2053,12 +2062,12 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="74"/>
-      <c r="J28" s="70"/>
+      <c r="I28" s="70"/>
+      <c r="J28" s="72"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="73" t="s">
+      <c r="A29" s="69" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2078,14 +2087,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="69">
+      <c r="I29" s="71">
         <v>46139</v>
       </c>
-      <c r="J29" s="69"/>
+      <c r="J29" s="71"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="74"/>
+      <c r="A30" s="70"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2103,12 +2112,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="74"/>
-      <c r="J30" s="70"/>
+      <c r="I30" s="70"/>
+      <c r="J30" s="72"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="73" t="s">
+      <c r="A31" s="69" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2128,14 +2137,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="69">
+      <c r="I31" s="71">
         <v>46133</v>
       </c>
-      <c r="J31" s="69"/>
+      <c r="J31" s="71"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="74"/>
+      <c r="A32" s="70"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2153,12 +2162,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="74"/>
-      <c r="J32" s="70"/>
+      <c r="I32" s="70"/>
+      <c r="J32" s="72"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="73" t="s">
+      <c r="A33" s="69" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2178,14 +2187,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="69">
+      <c r="I33" s="71">
         <v>46295</v>
       </c>
-      <c r="J33" s="69"/>
+      <c r="J33" s="71"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="74"/>
+      <c r="A34" s="70"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2203,12 +2212,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="74"/>
-      <c r="J34" s="70"/>
+      <c r="I34" s="70"/>
+      <c r="J34" s="72"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="73" t="s">
+      <c r="A35" s="69" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2228,14 +2237,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="69">
+      <c r="I35" s="71">
         <v>45884</v>
       </c>
-      <c r="J35" s="69"/>
+      <c r="J35" s="71"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="74"/>
+      <c r="A36" s="70"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2253,12 +2262,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="74"/>
-      <c r="J36" s="70"/>
+      <c r="I36" s="70"/>
+      <c r="J36" s="72"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="73" t="s">
+      <c r="A37" s="69" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2278,14 +2287,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="69">
+      <c r="I37" s="71">
         <v>45915</v>
       </c>
-      <c r="J37" s="69"/>
+      <c r="J37" s="71"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="74"/>
+      <c r="A38" s="70"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2303,12 +2312,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="74"/>
-      <c r="J38" s="70"/>
+      <c r="I38" s="70"/>
+      <c r="J38" s="72"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="69" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2324,12 +2333,12 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="69"/>
-      <c r="J39" s="69"/>
+      <c r="I39" s="71"/>
+      <c r="J39" s="71"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="74"/>
+      <c r="A40" s="70"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2343,12 +2352,12 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="74"/>
-      <c r="J40" s="70"/>
+      <c r="I40" s="70"/>
+      <c r="J40" s="72"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="73" t="s">
+      <c r="A41" s="69" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2368,14 +2377,14 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="69">
+      <c r="I41" s="71">
         <v>46234</v>
       </c>
-      <c r="J41" s="69"/>
+      <c r="J41" s="71"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="74"/>
+      <c r="A42" s="70"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2385,12 +2394,12 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="74"/>
-      <c r="J42" s="70"/>
+      <c r="I42" s="70"/>
+      <c r="J42" s="72"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="73" t="s">
+      <c r="A43" s="69" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
@@ -2406,12 +2415,12 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="69"/>
-      <c r="J43" s="69"/>
+      <c r="I43" s="71"/>
+      <c r="J43" s="71"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="74"/>
+      <c r="A44" s="70"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2425,21 +2434,50 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="74"/>
-      <c r="J44" s="70"/>
+      <c r="I44" s="70"/>
+      <c r="J44" s="72"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
+  <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="62">
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2456,43 +2494,15 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -3523,7 +3533,9 @@
       <c r="D20" s="15">
         <v>0.9</v>
       </c>
-      <c r="E20" s="23"/>
+      <c r="E20" s="23">
+        <v>341236.34</v>
+      </c>
       <c r="F20" s="24"/>
       <c r="G20" s="9">
         <v>255</v>
@@ -3538,7 +3550,12 @@
       <c r="N20" s="9">
         <v>0</v>
       </c>
-      <c r="P20" s="10"/>
+      <c r="O20" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="P20" s="10">
+        <v>228548</v>
+      </c>
       <c r="Q20" s="19">
         <v>45717</v>
       </c>
@@ -3564,6 +3581,9 @@
       <c r="D21" s="15">
         <v>0.9</v>
       </c>
+      <c r="E21" s="16">
+        <v>666700</v>
+      </c>
       <c r="F21" s="24"/>
       <c r="I21" s="9">
         <v>6</v>
@@ -3574,7 +3594,12 @@
       <c r="N21" s="9">
         <v>0</v>
       </c>
-      <c r="P21" s="10"/>
+      <c r="O21" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="P21" s="10">
+        <v>224227</v>
+      </c>
       <c r="Q21" s="19">
         <v>45717</v>
       </c>
@@ -3705,7 +3730,7 @@
         <v>46234</v>
       </c>
       <c r="T24" s="26" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="U24" s="31" t="s">
         <v>129</v>
@@ -4250,11 +4275,12 @@
       <c r="V189" s="19"/>
     </row>
   </sheetData>
+  <autoFilter ref="A4:V189" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4299,16 +4325,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="67"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="68" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="68"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4724,7 +4750,7 @@
         <v>61</v>
       </c>
       <c r="D29" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" t="s">
         <v>124</v>
@@ -4734,20 +4760,21 @@
       <c r="A30" s="3">
         <v>46230</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>100</v>
+      <c r="B30" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="C30" s="65" t="s">
         <v>61</v>
       </c>
       <c r="D30" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:E30" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -5688,6 +5715,7 @@
       <c r="D200" s="29"/>
     </row>
   </sheetData>
+  <autoFilter ref="A4:E200" xr:uid="{0CACF7FE-A4AF-4302-B8F5-800998C4C21C}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -5715,15 +5743,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5976,6 +5995,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
@@ -5988,14 +6016,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6012,4 +6032,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-30 17:54)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFD90073-5B89-4B92-979D-15C2FE4D8674}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA74708-4782-4A89-80A6-2A2930F6DA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3108" yWindow="756" windowWidth="14988" windowHeight="11484" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -1003,28 +1003,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1405,31 +1405,31 @@
       <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="76"/>
+      <c r="J2" s="76"/>
+      <c r="K2" s="76"/>
     </row>
     <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -1467,7 +1467,7 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="77" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
@@ -1487,14 +1487,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="77">
+      <c r="I5" s="71">
         <v>46244</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="71"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="70"/>
+      <c r="A6" s="74"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1512,12 +1512,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="70"/>
-      <c r="J6" s="72"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="70"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="73" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1537,14 +1537,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="71" t="s">
+      <c r="I7" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="71"/>
+      <c r="J7" s="69"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="70"/>
+      <c r="A8" s="74"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1562,12 +1562,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="70"/>
-      <c r="J8" s="72"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="70"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="69" t="s">
+      <c r="A9" s="73" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1587,14 +1587,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="71">
+      <c r="I9" s="69">
         <v>46218</v>
       </c>
-      <c r="J9" s="71"/>
+      <c r="J9" s="69"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="70"/>
+      <c r="A10" s="74"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1612,12 +1612,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="70"/>
-      <c r="J10" s="72"/>
+      <c r="I10" s="74"/>
+      <c r="J10" s="70"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="69" t="s">
+      <c r="A11" s="73" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1637,14 +1637,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="71">
+      <c r="I11" s="69">
         <v>46171</v>
       </c>
-      <c r="J11" s="71"/>
+      <c r="J11" s="69"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="70"/>
+      <c r="A12" s="74"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1662,12 +1662,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="70"/>
-      <c r="J12" s="72"/>
+      <c r="I12" s="74"/>
+      <c r="J12" s="70"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="69" t="s">
+      <c r="A13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1687,14 +1687,14 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="71" t="s">
+      <c r="I13" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="71"/>
+      <c r="J13" s="69"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="70"/>
+      <c r="A14" s="74"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1712,12 +1712,12 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="70"/>
-      <c r="J14" s="72"/>
+      <c r="I14" s="74"/>
+      <c r="J14" s="70"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="69" t="s">
+      <c r="A15" s="73" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1737,14 +1737,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="71">
+      <c r="I15" s="69">
         <v>46199</v>
       </c>
-      <c r="J15" s="71"/>
+      <c r="J15" s="69"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="70"/>
+      <c r="A16" s="74"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1762,8 +1762,8 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="70"/>
-      <c r="J16" s="72"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="70"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11">
@@ -1787,14 +1787,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="74">
+      <c r="I17" s="72">
         <v>46305</v>
       </c>
-      <c r="J17" s="74"/>
+      <c r="J17" s="72"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="70"/>
+      <c r="A18" s="74"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1812,8 +1812,8 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="70"/>
-      <c r="J18" s="72"/>
+      <c r="I18" s="74"/>
+      <c r="J18" s="70"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11">
@@ -1837,14 +1837,14 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="74">
+      <c r="I19" s="72">
         <v>46336</v>
       </c>
-      <c r="J19" s="74"/>
+      <c r="J19" s="72"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="70"/>
+      <c r="A20" s="74"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1862,12 +1862,12 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="70"/>
-      <c r="J20" s="72"/>
+      <c r="I20" s="74"/>
+      <c r="J20" s="70"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="69" t="s">
+      <c r="A21" s="73" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1887,14 +1887,14 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="71">
+      <c r="I21" s="69">
         <v>46336</v>
       </c>
-      <c r="J21" s="71"/>
+      <c r="J21" s="69"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="70"/>
+      <c r="A22" s="74"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1912,12 +1912,12 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="70"/>
-      <c r="J22" s="72"/>
+      <c r="I22" s="74"/>
+      <c r="J22" s="70"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="69" t="s">
+      <c r="A23" s="73" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -1937,14 +1937,14 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="69">
         <v>46237</v>
       </c>
-      <c r="J23" s="71"/>
+      <c r="J23" s="69"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="70"/>
+      <c r="A24" s="74"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -1962,12 +1962,12 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="70"/>
-      <c r="J24" s="72"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="70"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="69" t="s">
+      <c r="A25" s="73" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -1987,14 +1987,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="71">
+      <c r="I25" s="69">
         <v>46188</v>
       </c>
-      <c r="J25" s="71"/>
+      <c r="J25" s="69"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="70"/>
+      <c r="A26" s="74"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2012,12 +2012,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="70"/>
-      <c r="J26" s="72"/>
+      <c r="I26" s="74"/>
+      <c r="J26" s="70"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="69" t="s">
+      <c r="A27" s="73" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2037,14 +2037,14 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="71">
+      <c r="I27" s="69">
         <v>46321</v>
       </c>
-      <c r="J27" s="71"/>
+      <c r="J27" s="69"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="70"/>
+      <c r="A28" s="74"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2062,12 +2062,12 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="70"/>
-      <c r="J28" s="72"/>
+      <c r="I28" s="74"/>
+      <c r="J28" s="70"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="69" t="s">
+      <c r="A29" s="73" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2087,14 +2087,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="71">
+      <c r="I29" s="69">
         <v>46139</v>
       </c>
-      <c r="J29" s="71"/>
+      <c r="J29" s="69"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="70"/>
+      <c r="A30" s="74"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2112,12 +2112,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="70"/>
-      <c r="J30" s="72"/>
+      <c r="I30" s="74"/>
+      <c r="J30" s="70"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="69" t="s">
+      <c r="A31" s="73" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2137,14 +2137,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="71">
+      <c r="I31" s="69">
         <v>46133</v>
       </c>
-      <c r="J31" s="71"/>
+      <c r="J31" s="69"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="70"/>
+      <c r="A32" s="74"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2162,12 +2162,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="70"/>
-      <c r="J32" s="72"/>
+      <c r="I32" s="74"/>
+      <c r="J32" s="70"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="69" t="s">
+      <c r="A33" s="73" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2187,14 +2187,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="71">
+      <c r="I33" s="69">
         <v>46295</v>
       </c>
-      <c r="J33" s="71"/>
+      <c r="J33" s="69"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="70"/>
+      <c r="A34" s="74"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2212,12 +2212,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="70"/>
-      <c r="J34" s="72"/>
+      <c r="I34" s="74"/>
+      <c r="J34" s="70"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="69" t="s">
+      <c r="A35" s="73" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2237,14 +2237,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="71">
+      <c r="I35" s="69">
         <v>45884</v>
       </c>
-      <c r="J35" s="71"/>
+      <c r="J35" s="69"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="70"/>
+      <c r="A36" s="74"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2262,12 +2262,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="70"/>
-      <c r="J36" s="72"/>
+      <c r="I36" s="74"/>
+      <c r="J36" s="70"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="69" t="s">
+      <c r="A37" s="73" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2287,14 +2287,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="71">
+      <c r="I37" s="69">
         <v>45915</v>
       </c>
-      <c r="J37" s="71"/>
+      <c r="J37" s="69"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="70"/>
+      <c r="A38" s="74"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2312,12 +2312,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="70"/>
-      <c r="J38" s="72"/>
+      <c r="I38" s="74"/>
+      <c r="J38" s="70"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="69" t="s">
+      <c r="A39" s="73" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2333,12 +2333,12 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="71"/>
-      <c r="J39" s="71"/>
+      <c r="I39" s="69"/>
+      <c r="J39" s="69"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="70"/>
+      <c r="A40" s="74"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2352,12 +2352,12 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="70"/>
-      <c r="J40" s="72"/>
+      <c r="I40" s="74"/>
+      <c r="J40" s="70"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="69" t="s">
+      <c r="A41" s="73" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2377,14 +2377,14 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="71">
+      <c r="I41" s="69">
         <v>46234</v>
       </c>
-      <c r="J41" s="71"/>
+      <c r="J41" s="69"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="70"/>
+      <c r="A42" s="74"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2394,12 +2394,12 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="70"/>
-      <c r="J42" s="72"/>
+      <c r="I42" s="74"/>
+      <c r="J42" s="70"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="69" t="s">
+      <c r="A43" s="73" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
@@ -2415,12 +2415,12 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="71"/>
-      <c r="J43" s="71"/>
+      <c r="I43" s="69"/>
+      <c r="J43" s="69"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="70"/>
+      <c r="A44" s="74"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2434,27 +2434,45 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="70"/>
-      <c r="J44" s="72"/>
+      <c r="I44" s="74"/>
+      <c r="J44" s="70"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="62">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2471,38 +2489,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -4325,16 +4325,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="67"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="68" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="68"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4843,7 +4843,7 @@
         <v>46224</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4877,7 +4877,7 @@
         <v>46224</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -5730,19 +5730,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5995,6 +5982,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -6005,17 +6005,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6034,6 +6023,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-31 13:42)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA74708-4782-4A89-80A6-2A2930F6DA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1678C19D-7701-4479-84E8-EB3188F027EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -489,7 +489,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -592,6 +592,20 @@
     </font>
     <font>
       <sz val="10.5"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -813,7 +827,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1003,28 +1017,38 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1387,6 +1411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
@@ -1405,33 +1430,33 @@
       <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-    </row>
-    <row r="4" spans="1:11" ht="27.6">
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+    </row>
+    <row r="4" spans="1:11" ht="28.2" thickBot="1">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1466,8 +1491,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="77" t="s">
+    <row r="5" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A5" s="76" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
@@ -1487,14 +1512,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="71">
+      <c r="I5" s="77">
         <v>46244</v>
       </c>
-      <c r="J5" s="71"/>
+      <c r="J5" s="77"/>
       <c r="K5" s="47"/>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="74"/>
+    <row r="6" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A6" s="70"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1512,12 +1537,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="74"/>
-      <c r="J6" s="70"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="72"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="69" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1537,14 +1562,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="69" t="s">
+      <c r="I7" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="69"/>
+      <c r="J7" s="71"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="74"/>
+      <c r="A8" s="70"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1562,12 +1587,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="74"/>
-      <c r="J8" s="70"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="72"/>
       <c r="K8" s="48"/>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="73" t="s">
+    <row r="9" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A9" s="69" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1587,14 +1612,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="69">
+      <c r="I9" s="71">
         <v>46218</v>
       </c>
-      <c r="J9" s="69"/>
+      <c r="J9" s="71"/>
       <c r="K9" s="49"/>
     </row>
-    <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="74"/>
+    <row r="10" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A10" s="70"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1612,12 +1637,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="74"/>
-      <c r="J10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="72"/>
       <c r="K10" s="48"/>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="73" t="s">
+    <row r="11" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A11" s="69" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1637,14 +1662,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="69">
+      <c r="I11" s="71">
         <v>46171</v>
       </c>
-      <c r="J11" s="69"/>
+      <c r="J11" s="71"/>
       <c r="K11" s="49"/>
     </row>
-    <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="74"/>
+    <row r="12" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A12" s="70"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1662,12 +1687,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="74"/>
-      <c r="J12" s="70"/>
+      <c r="I12" s="70"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="73" t="s">
+      <c r="A13" s="69" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1687,14 +1712,14 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="69" t="s">
+      <c r="I13" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="69"/>
+      <c r="J13" s="71"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="74"/>
+      <c r="A14" s="70"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1712,12 +1737,12 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="74"/>
-      <c r="J14" s="70"/>
+      <c r="I14" s="70"/>
+      <c r="J14" s="72"/>
       <c r="K14" s="48"/>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="73" t="s">
+    <row r="15" spans="1:11" hidden="1">
+      <c r="A15" s="69" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1737,14 +1762,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="69">
+      <c r="I15" s="71">
         <v>46199</v>
       </c>
-      <c r="J15" s="69"/>
+      <c r="J15" s="71"/>
       <c r="K15" s="49"/>
     </row>
-    <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="74"/>
+    <row r="16" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A16" s="70"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1762,11 +1787,11 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="74"/>
-      <c r="J16" s="70"/>
+      <c r="I16" s="70"/>
+      <c r="J16" s="72"/>
       <c r="K16" s="48"/>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" hidden="1">
       <c r="A17" s="75" t="s">
         <v>21</v>
       </c>
@@ -1787,14 +1812,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="72">
+      <c r="I17" s="74">
         <v>46305</v>
       </c>
-      <c r="J17" s="72"/>
+      <c r="J17" s="74"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="74"/>
+      <c r="A18" s="70"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1812,8 +1837,8 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="74"/>
-      <c r="J18" s="70"/>
+      <c r="I18" s="70"/>
+      <c r="J18" s="72"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11">
@@ -1837,14 +1862,14 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="72">
-        <v>46336</v>
-      </c>
-      <c r="J19" s="72"/>
+      <c r="I19" s="78">
+        <v>46419</v>
+      </c>
+      <c r="J19" s="74"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="74"/>
+      <c r="A20" s="70"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1862,12 +1887,12 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="74"/>
-      <c r="J20" s="70"/>
+      <c r="I20" s="79"/>
+      <c r="J20" s="72"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="73" t="s">
+      <c r="A21" s="69" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1887,14 +1912,14 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="69">
-        <v>46336</v>
-      </c>
-      <c r="J21" s="69"/>
+      <c r="I21" s="80">
+        <v>46397</v>
+      </c>
+      <c r="J21" s="71"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="74"/>
+      <c r="A22" s="70"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1912,12 +1937,12 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="74"/>
-      <c r="J22" s="70"/>
+      <c r="I22" s="79"/>
+      <c r="J22" s="72"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="73" t="s">
+      <c r="A23" s="69" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -1937,14 +1962,14 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="69">
+      <c r="I23" s="71">
         <v>46237</v>
       </c>
-      <c r="J23" s="69"/>
+      <c r="J23" s="71"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="74"/>
+      <c r="A24" s="70"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -1962,12 +1987,12 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="74"/>
-      <c r="J24" s="70"/>
+      <c r="I24" s="70"/>
+      <c r="J24" s="72"/>
       <c r="K24" s="52"/>
     </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="73" t="s">
+    <row r="25" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A25" s="69" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -1987,14 +2012,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="69">
+      <c r="I25" s="71">
         <v>46188</v>
       </c>
-      <c r="J25" s="69"/>
+      <c r="J25" s="71"/>
       <c r="K25" s="51"/>
     </row>
-    <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="74"/>
+    <row r="26" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A26" s="70"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2012,12 +2037,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="74"/>
-      <c r="J26" s="70"/>
+      <c r="I26" s="70"/>
+      <c r="J26" s="72"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="73" t="s">
+      <c r="A27" s="69" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2037,14 +2062,14 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="69">
+      <c r="I27" s="71">
         <v>46321</v>
       </c>
-      <c r="J27" s="69"/>
+      <c r="J27" s="71"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="74"/>
+      <c r="A28" s="70"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2062,12 +2087,12 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="74"/>
-      <c r="J28" s="70"/>
+      <c r="I28" s="70"/>
+      <c r="J28" s="72"/>
       <c r="K28" s="52"/>
     </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="73" t="s">
+    <row r="29" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A29" s="69" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2087,14 +2112,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="69">
+      <c r="I29" s="71">
         <v>46139</v>
       </c>
-      <c r="J29" s="69"/>
+      <c r="J29" s="71"/>
       <c r="K29" s="51"/>
     </row>
-    <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="74"/>
+    <row r="30" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A30" s="70"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2112,12 +2137,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="74"/>
-      <c r="J30" s="70"/>
+      <c r="I30" s="70"/>
+      <c r="J30" s="72"/>
       <c r="K30" s="52"/>
     </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="73" t="s">
+    <row r="31" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A31" s="69" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2137,14 +2162,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="69">
+      <c r="I31" s="71">
         <v>46133</v>
       </c>
-      <c r="J31" s="69"/>
+      <c r="J31" s="71"/>
       <c r="K31" s="51"/>
     </row>
-    <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="74"/>
+    <row r="32" spans="1:11" ht="15" hidden="1" thickBot="1">
+      <c r="A32" s="70"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2162,12 +2187,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="74"/>
-      <c r="J32" s="70"/>
+      <c r="I32" s="70"/>
+      <c r="J32" s="72"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="73" t="s">
+      <c r="A33" s="69" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2187,14 +2212,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="69">
+      <c r="I33" s="71">
         <v>46295</v>
       </c>
-      <c r="J33" s="69"/>
+      <c r="J33" s="71"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="74"/>
+      <c r="A34" s="70"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2212,12 +2237,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="74"/>
-      <c r="J34" s="70"/>
+      <c r="I34" s="70"/>
+      <c r="J34" s="72"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="73" t="s">
+      <c r="A35" s="69" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2237,14 +2262,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="69">
-        <v>45884</v>
-      </c>
-      <c r="J35" s="69"/>
+      <c r="I35" s="71">
+        <v>45899</v>
+      </c>
+      <c r="J35" s="71"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="74"/>
+      <c r="A36" s="70"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2262,12 +2287,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="74"/>
-      <c r="J36" s="70"/>
+      <c r="I36" s="70"/>
+      <c r="J36" s="72"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="73" t="s">
+      <c r="A37" s="69" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2287,14 +2312,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="69">
-        <v>45915</v>
-      </c>
-      <c r="J37" s="69"/>
+      <c r="I37" s="71">
+        <v>45910</v>
+      </c>
+      <c r="J37" s="71"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="74"/>
+      <c r="A38" s="70"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2312,12 +2337,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="74"/>
-      <c r="J38" s="70"/>
+      <c r="I38" s="70"/>
+      <c r="J38" s="72"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="69" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2333,12 +2358,12 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="69"/>
-      <c r="J39" s="69"/>
+      <c r="I39" s="71"/>
+      <c r="J39" s="71"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="74"/>
+      <c r="A40" s="70"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2352,12 +2377,12 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="74"/>
-      <c r="J40" s="70"/>
+      <c r="I40" s="70"/>
+      <c r="J40" s="72"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="73" t="s">
+      <c r="A41" s="69" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2377,14 +2402,14 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="69">
-        <v>46234</v>
-      </c>
-      <c r="J41" s="69"/>
+      <c r="I41" s="71">
+        <v>46237</v>
+      </c>
+      <c r="J41" s="71"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="74"/>
+      <c r="A42" s="70"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2394,12 +2419,12 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="74"/>
-      <c r="J42" s="70"/>
+      <c r="I42" s="70"/>
+      <c r="J42" s="72"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="73" t="s">
+      <c r="A43" s="69" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
@@ -2415,12 +2440,12 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="69"/>
-      <c r="J43" s="69"/>
+      <c r="I43" s="71"/>
+      <c r="J43" s="71"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="74"/>
+      <c r="A44" s="70"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2434,22 +2459,58 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="74"/>
-      <c r="J44" s="70"/>
+      <c r="I44" s="70"/>
+      <c r="J44" s="72"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters blank="1">
+        <filter val="Construction"/>
+        <filter val="On Hold"/>
+        <filter val="Planning"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="62">
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2466,45 +2527,17 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -2705,8 +2738,8 @@
         <f>'[1]Master Schedule'!C5</f>
         <v>46084</v>
       </c>
-      <c r="R5" s="19">
-        <v>46106</v>
+      <c r="R5" s="81">
+        <v>46248</v>
       </c>
       <c r="S5" s="14"/>
       <c r="T5" s="25" t="s">
@@ -3560,7 +3593,7 @@
         <v>45717</v>
       </c>
       <c r="R20" s="19">
-        <v>45737</v>
+        <v>45899</v>
       </c>
       <c r="T20" s="26" t="s">
         <v>65</v>
@@ -3604,7 +3637,7 @@
         <v>45717</v>
       </c>
       <c r="R21" s="19">
-        <v>45737</v>
+        <v>45910</v>
       </c>
       <c r="T21" s="26" t="s">
         <v>126</v>
@@ -3727,7 +3760,7 @@
         <v>46225</v>
       </c>
       <c r="R24" s="11">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="T24" s="26" t="s">
         <v>140</v>
@@ -4325,16 +4358,16 @@
         <v>57</v>
       </c>
       <c r="B1" s="67"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="68" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="68"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5730,6 +5763,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -5982,29 +6037,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6021,23 +6073,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-08-06 17:35)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1678C19D-7701-4479-84E8-EB3188F027EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6683723C-A3B6-44E3-855E-63C92E5D4C5A}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="144">
   <si>
     <t>MASTER SCHEDULE</t>
   </si>
@@ -477,6 +477,9 @@
   </si>
   <si>
     <t>บริษัท อีโค่คูล ไครลเมท เทคโนโลยี จำกัด</t>
+  </si>
+  <si>
+    <t>เทสและวัดลม</t>
   </si>
 </sst>
 </file>
@@ -489,7 +492,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -603,6 +606,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10.5"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <b/>
       <sz val="10.5"/>
       <color rgb="FFFF0000"/>
@@ -610,7 +623,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -645,8 +658,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -820,6 +845,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -827,7 +867,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -997,12 +1037,6 @@
     <xf numFmtId="9" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1040,16 +1074,32 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma 2 2 3 2" xfId="3" xr:uid="{10CA6883-C0B4-442D-A7D0-FF27A9ED468E}"/>
@@ -1411,7 +1461,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
@@ -1427,34 +1476,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
     </row>
     <row r="4" spans="1:11" ht="28.2" thickBot="1">
       <c r="A4" s="1" t="s">
@@ -1491,17 +1540,17 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A5" s="76" t="s">
+    <row r="5" spans="1:11" ht="15" thickBot="1">
+      <c r="A5" s="74" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="59">
+      <c r="C5" s="76">
         <v>46084</v>
       </c>
-      <c r="D5" s="59">
+      <c r="D5" s="76">
         <v>46127</v>
       </c>
       <c r="E5" s="59"/>
@@ -1512,21 +1561,21 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="77">
+      <c r="I5" s="82">
         <v>46244</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="75"/>
       <c r="K5" s="47"/>
     </row>
-    <row r="6" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A6" s="70"/>
+    <row r="6" spans="1:11" ht="15" thickBot="1">
+      <c r="A6" s="68"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="45">
+      <c r="C6" s="76">
         <v>46189</v>
       </c>
-      <c r="D6" s="45">
+      <c r="D6" s="76">
         <v>46189</v>
       </c>
       <c r="E6" s="45"/>
@@ -1537,22 +1586,22 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="70"/>
-      <c r="J6" s="72"/>
+      <c r="I6" s="83"/>
+      <c r="J6" s="70"/>
       <c r="K6" s="48"/>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="69" t="s">
+    <row r="7" spans="1:11" ht="15" thickBot="1">
+      <c r="A7" s="67" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="39">
-        <v>46219</v>
-      </c>
-      <c r="D7" s="39">
-        <v>46233</v>
+      <c r="C7" s="77">
+        <v>46266</v>
+      </c>
+      <c r="D7" s="77">
+        <v>46275</v>
       </c>
       <c r="E7" s="39"/>
       <c r="F7" s="39"/>
@@ -1562,22 +1611,22 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="71" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="71"/>
+      <c r="I7" s="82">
+        <v>46366</v>
+      </c>
+      <c r="J7" s="69"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="70"/>
+      <c r="A8" s="68"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="36">
-        <v>46244</v>
-      </c>
-      <c r="D8" s="36">
-        <v>46247</v>
+      <c r="C8" s="77">
+        <v>46305</v>
+      </c>
+      <c r="D8" s="77">
+        <v>46308</v>
       </c>
       <c r="E8" s="36"/>
       <c r="F8" s="36"/>
@@ -1587,21 +1636,21 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="70"/>
-      <c r="J8" s="72"/>
+      <c r="I8" s="83"/>
+      <c r="J8" s="70"/>
       <c r="K8" s="48"/>
     </row>
-    <row r="9" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A9" s="69" t="s">
+    <row r="9" spans="1:11" ht="15" thickBot="1">
+      <c r="A9" s="67" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="39">
+      <c r="C9" s="76">
         <v>46082</v>
       </c>
-      <c r="D9" s="39">
+      <c r="D9" s="76">
         <v>46096</v>
       </c>
       <c r="E9" s="39"/>
@@ -1612,21 +1661,21 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="71">
+      <c r="I9" s="82">
         <v>46218</v>
       </c>
-      <c r="J9" s="71"/>
+      <c r="J9" s="69"/>
       <c r="K9" s="49"/>
     </row>
-    <row r="10" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A10" s="70"/>
+    <row r="10" spans="1:11" ht="15" thickBot="1">
+      <c r="A10" s="68"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="76">
         <v>46168</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="76">
         <v>46213</v>
       </c>
       <c r="E10" s="36"/>
@@ -1637,21 +1686,21 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="70"/>
-      <c r="J10" s="72"/>
+      <c r="I10" s="83"/>
+      <c r="J10" s="70"/>
       <c r="K10" s="48"/>
     </row>
-    <row r="11" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A11" s="69" t="s">
+    <row r="11" spans="1:11" ht="15" thickBot="1">
+      <c r="A11" s="67" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="42">
+      <c r="C11" s="76">
         <v>46184</v>
       </c>
-      <c r="D11" s="42">
+      <c r="D11" s="76">
         <v>46191</v>
       </c>
       <c r="E11" s="42"/>
@@ -1662,21 +1711,21 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="71">
+      <c r="I11" s="82">
         <v>46171</v>
       </c>
-      <c r="J11" s="71"/>
+      <c r="J11" s="69"/>
       <c r="K11" s="49"/>
     </row>
-    <row r="12" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A12" s="70"/>
+    <row r="12" spans="1:11" ht="15" thickBot="1">
+      <c r="A12" s="68"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="45">
+      <c r="C12" s="76">
         <v>46200</v>
       </c>
-      <c r="D12" s="45">
+      <c r="D12" s="76">
         <v>46202</v>
       </c>
       <c r="E12" s="45"/>
@@ -1687,21 +1736,21 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="70"/>
-      <c r="J12" s="72"/>
+      <c r="I12" s="83"/>
+      <c r="J12" s="70"/>
       <c r="K12" s="48"/>
     </row>
-    <row r="13" spans="1:11">
-      <c r="A13" s="69" t="s">
+    <row r="13" spans="1:11" ht="15" thickBot="1">
+      <c r="A13" s="67" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="39">
+      <c r="C13" s="77">
         <v>46392</v>
       </c>
-      <c r="D13" s="39">
+      <c r="D13" s="77">
         <v>46402</v>
       </c>
       <c r="E13" s="39"/>
@@ -1712,22 +1761,22 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="71" t="s">
-        <v>16</v>
-      </c>
-      <c r="J13" s="71"/>
+      <c r="I13" s="84">
+        <v>46419</v>
+      </c>
+      <c r="J13" s="69"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="70"/>
+      <c r="A14" s="68"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="36">
-        <v>46042</v>
-      </c>
-      <c r="D14" s="36">
-        <v>46042</v>
+      <c r="C14" s="77">
+        <v>46423</v>
+      </c>
+      <c r="D14" s="77">
+        <v>46428</v>
       </c>
       <c r="E14" s="36"/>
       <c r="F14" s="36"/>
@@ -1737,21 +1786,21 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="70"/>
-      <c r="J14" s="72"/>
+      <c r="I14" s="85"/>
+      <c r="J14" s="70"/>
       <c r="K14" s="48"/>
     </row>
-    <row r="15" spans="1:11" hidden="1">
-      <c r="A15" s="69" t="s">
+    <row r="15" spans="1:11" ht="15" thickBot="1">
+      <c r="A15" s="67" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="42">
+      <c r="C15" s="76">
         <v>46168</v>
       </c>
-      <c r="D15" s="42">
+      <c r="D15" s="76">
         <v>46188</v>
       </c>
       <c r="E15" s="42"/>
@@ -1762,21 +1811,21 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="71">
+      <c r="I15" s="82">
         <v>46199</v>
       </c>
-      <c r="J15" s="71"/>
+      <c r="J15" s="69"/>
       <c r="K15" s="49"/>
     </row>
-    <row r="16" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A16" s="70"/>
+    <row r="16" spans="1:11" ht="15" thickBot="1">
+      <c r="A16" s="68"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="45">
+      <c r="C16" s="76">
         <v>46198</v>
       </c>
-      <c r="D16" s="45">
+      <c r="D16" s="76">
         <v>46199</v>
       </c>
       <c r="E16" s="45"/>
@@ -1787,21 +1836,21 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="70"/>
-      <c r="J16" s="72"/>
+      <c r="I16" s="83"/>
+      <c r="J16" s="70"/>
       <c r="K16" s="48"/>
     </row>
-    <row r="17" spans="1:11" hidden="1">
-      <c r="A17" s="75" t="s">
+    <row r="17" spans="1:11" ht="15" thickBot="1">
+      <c r="A17" s="73" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="33">
+      <c r="C17" s="76">
         <v>46188</v>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="76">
         <v>46198</v>
       </c>
       <c r="E17" s="33"/>
@@ -1812,21 +1861,21 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="74">
+      <c r="I17" s="82">
         <v>46305</v>
       </c>
-      <c r="J17" s="74"/>
+      <c r="J17" s="72"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="70"/>
+      <c r="A18" s="68"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="36">
+      <c r="C18" s="78">
         <v>46296</v>
       </c>
-      <c r="D18" s="36">
+      <c r="D18" s="78">
         <v>46298</v>
       </c>
       <c r="E18" s="36"/>
@@ -1837,22 +1886,22 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="70"/>
-      <c r="J18" s="72"/>
+      <c r="I18" s="83"/>
+      <c r="J18" s="70"/>
       <c r="K18" s="48"/>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="75" t="s">
+    <row r="19" spans="1:11" ht="15" thickBot="1">
+      <c r="A19" s="73" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="33">
-        <v>46275</v>
-      </c>
-      <c r="D19" s="33">
-        <v>46290</v>
+      <c r="C19" s="77">
+        <v>46366</v>
+      </c>
+      <c r="D19" s="77">
+        <v>46381</v>
       </c>
       <c r="E19" s="33"/>
       <c r="F19" s="33"/>
@@ -1862,22 +1911,22 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="78">
+      <c r="I19" s="84">
         <v>46419</v>
       </c>
-      <c r="J19" s="74"/>
+      <c r="J19" s="72"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="70"/>
+      <c r="A20" s="68"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="36">
-        <v>46327</v>
-      </c>
-      <c r="D20" s="36">
-        <v>46329</v>
+      <c r="C20" s="77">
+        <v>46388</v>
+      </c>
+      <c r="D20" s="77">
+        <v>46390</v>
       </c>
       <c r="E20" s="36"/>
       <c r="F20" s="36"/>
@@ -1887,21 +1936,21 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="79"/>
-      <c r="J20" s="72"/>
+      <c r="I20" s="85"/>
+      <c r="J20" s="70"/>
       <c r="K20" s="48"/>
     </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="69" t="s">
+    <row r="21" spans="1:11" ht="15" thickBot="1">
+      <c r="A21" s="67" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="39">
+      <c r="C21" s="77">
         <v>46240</v>
       </c>
-      <c r="D21" s="39">
+      <c r="D21" s="77">
         <v>46249</v>
       </c>
       <c r="E21" s="39"/>
@@ -1912,21 +1961,21 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="80">
+      <c r="I21" s="84">
         <v>46397</v>
       </c>
-      <c r="J21" s="71"/>
+      <c r="J21" s="69"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="70"/>
+      <c r="A22" s="68"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="36">
+      <c r="C22" s="77">
         <v>46327</v>
       </c>
-      <c r="D22" s="36">
+      <c r="D22" s="77">
         <v>46329</v>
       </c>
       <c r="E22" s="36"/>
@@ -1937,22 +1986,22 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="79"/>
-      <c r="J22" s="72"/>
+      <c r="I22" s="85"/>
+      <c r="J22" s="70"/>
       <c r="K22" s="52"/>
     </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="69" t="s">
+    <row r="23" spans="1:11" ht="15" thickBot="1">
+      <c r="A23" s="67" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="42">
-        <v>46190</v>
-      </c>
-      <c r="D23" s="42">
-        <v>46206</v>
+      <c r="C23" s="76">
+        <v>46197</v>
+      </c>
+      <c r="D23" s="76">
+        <v>46209</v>
       </c>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
@@ -1962,22 +2011,22 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="82">
         <v>46237</v>
       </c>
-      <c r="J23" s="71"/>
+      <c r="J23" s="69"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="70"/>
+      <c r="A24" s="68"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="45">
-        <v>46216</v>
-      </c>
-      <c r="D24" s="45">
-        <v>46220</v>
+      <c r="C24" s="76">
+        <v>46209</v>
+      </c>
+      <c r="D24" s="76">
+        <v>46211</v>
       </c>
       <c r="E24" s="45"/>
       <c r="F24" s="45"/>
@@ -1987,21 +2036,21 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="70"/>
-      <c r="J24" s="72"/>
+      <c r="I24" s="83"/>
+      <c r="J24" s="70"/>
       <c r="K24" s="52"/>
     </row>
-    <row r="25" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A25" s="69" t="s">
+    <row r="25" spans="1:11" ht="15" thickBot="1">
+      <c r="A25" s="67" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="42">
+      <c r="C25" s="76">
         <v>46185</v>
       </c>
-      <c r="D25" s="42">
+      <c r="D25" s="76">
         <v>46188</v>
       </c>
       <c r="E25" s="42"/>
@@ -2012,21 +2061,21 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="71">
+      <c r="I25" s="82">
         <v>46188</v>
       </c>
-      <c r="J25" s="71"/>
+      <c r="J25" s="69"/>
       <c r="K25" s="51"/>
     </row>
-    <row r="26" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A26" s="70"/>
+    <row r="26" spans="1:11" ht="15" thickBot="1">
+      <c r="A26" s="68"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="45">
+      <c r="C26" s="76">
         <v>46185</v>
       </c>
-      <c r="D26" s="45">
+      <c r="D26" s="76">
         <v>46188</v>
       </c>
       <c r="E26" s="45"/>
@@ -2037,22 +2086,22 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="70"/>
-      <c r="J26" s="72"/>
+      <c r="I26" s="83"/>
+      <c r="J26" s="70"/>
       <c r="K26" s="52"/>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="69" t="s">
+    <row r="27" spans="1:11" ht="15" thickBot="1">
+      <c r="A27" s="67" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C27" s="39">
-        <v>46234</v>
-      </c>
-      <c r="D27" s="39">
-        <v>46247</v>
+      <c r="C27" s="79">
+        <v>46275</v>
+      </c>
+      <c r="D27" s="79">
+        <v>46295</v>
       </c>
       <c r="E27" s="39"/>
       <c r="F27" s="39"/>
@@ -2062,22 +2111,22 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="71">
-        <v>46321</v>
-      </c>
-      <c r="J27" s="71"/>
+      <c r="I27" s="84">
+        <v>46382</v>
+      </c>
+      <c r="J27" s="69"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="70"/>
+      <c r="A28" s="68"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="36">
-        <v>46314</v>
-      </c>
-      <c r="D28" s="36">
-        <v>46316</v>
+      <c r="C28" s="79">
+        <v>46345</v>
+      </c>
+      <c r="D28" s="79">
+        <v>46347</v>
       </c>
       <c r="E28" s="36"/>
       <c r="F28" s="36"/>
@@ -2087,21 +2136,21 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="70"/>
-      <c r="J28" s="72"/>
+      <c r="I28" s="85"/>
+      <c r="J28" s="70"/>
       <c r="K28" s="52"/>
     </row>
-    <row r="29" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A29" s="69" t="s">
+    <row r="29" spans="1:11" ht="15" thickBot="1">
+      <c r="A29" s="67" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="42">
+      <c r="C29" s="76">
         <v>46091</v>
       </c>
-      <c r="D29" s="42">
+      <c r="D29" s="76">
         <v>46100</v>
       </c>
       <c r="E29" s="42"/>
@@ -2112,21 +2161,21 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="71">
+      <c r="I29" s="82">
         <v>46139</v>
       </c>
-      <c r="J29" s="71"/>
+      <c r="J29" s="69"/>
       <c r="K29" s="51"/>
     </row>
-    <row r="30" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A30" s="70"/>
+    <row r="30" spans="1:11" ht="15" thickBot="1">
+      <c r="A30" s="68"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="45">
+      <c r="C30" s="76">
         <v>46120</v>
       </c>
-      <c r="D30" s="45">
+      <c r="D30" s="76">
         <v>46124</v>
       </c>
       <c r="E30" s="45"/>
@@ -2137,21 +2186,21 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="70"/>
-      <c r="J30" s="72"/>
+      <c r="I30" s="83"/>
+      <c r="J30" s="70"/>
       <c r="K30" s="52"/>
     </row>
-    <row r="31" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A31" s="69" t="s">
+    <row r="31" spans="1:11" ht="15" thickBot="1">
+      <c r="A31" s="67" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C31" s="42">
+      <c r="C31" s="76">
         <v>46091</v>
       </c>
-      <c r="D31" s="42">
+      <c r="D31" s="76">
         <v>46094</v>
       </c>
       <c r="E31" s="42"/>
@@ -2162,21 +2211,21 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="71">
+      <c r="I31" s="82">
         <v>46133</v>
       </c>
-      <c r="J31" s="71"/>
+      <c r="J31" s="69"/>
       <c r="K31" s="51"/>
     </row>
-    <row r="32" spans="1:11" ht="15" hidden="1" thickBot="1">
-      <c r="A32" s="70"/>
+    <row r="32" spans="1:11" ht="15" thickBot="1">
+      <c r="A32" s="68"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C32" s="45">
+      <c r="C32" s="76">
         <v>46091</v>
       </c>
-      <c r="D32" s="45">
+      <c r="D32" s="76">
         <v>46094</v>
       </c>
       <c r="E32" s="45"/>
@@ -2187,21 +2236,21 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="70"/>
-      <c r="J32" s="72"/>
+      <c r="I32" s="83"/>
+      <c r="J32" s="70"/>
       <c r="K32" s="52"/>
     </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="69" t="s">
+    <row r="33" spans="1:11" ht="15" thickBot="1">
+      <c r="A33" s="67" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="61">
+      <c r="C33" s="77">
         <v>46237</v>
       </c>
-      <c r="D33" s="61">
+      <c r="D33" s="77">
         <v>46248</v>
       </c>
       <c r="E33" s="39"/>
@@ -2212,21 +2261,21 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="71">
-        <v>46295</v>
-      </c>
-      <c r="J33" s="71"/>
+      <c r="I33" s="82">
+        <v>46342</v>
+      </c>
+      <c r="J33" s="69"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="70"/>
+      <c r="A34" s="68"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="62">
+      <c r="C34" s="77">
         <v>46296</v>
       </c>
-      <c r="D34" s="62">
+      <c r="D34" s="77">
         <v>46303</v>
       </c>
       <c r="E34" s="36"/>
@@ -2237,21 +2286,21 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="70"/>
-      <c r="J34" s="72"/>
+      <c r="I34" s="83"/>
+      <c r="J34" s="70"/>
       <c r="K34" s="52"/>
     </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="69" t="s">
+    <row r="35" spans="1:11" ht="15" thickBot="1">
+      <c r="A35" s="67" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C35" s="39">
+      <c r="C35" s="76">
         <v>45723</v>
       </c>
-      <c r="D35" s="39">
+      <c r="D35" s="76">
         <v>45729</v>
       </c>
       <c r="E35" s="39"/>
@@ -2262,22 +2311,22 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="71">
-        <v>45899</v>
-      </c>
-      <c r="J35" s="71"/>
+      <c r="I35" s="82">
+        <v>46264</v>
+      </c>
+      <c r="J35" s="69"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="70"/>
+      <c r="A36" s="68"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="36">
-        <v>45729</v>
-      </c>
-      <c r="D36" s="36">
-        <v>45732</v>
+      <c r="C36" s="78">
+        <v>46259</v>
+      </c>
+      <c r="D36" s="78">
+        <v>46264</v>
       </c>
       <c r="E36" s="36"/>
       <c r="F36" s="36"/>
@@ -2287,21 +2336,21 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="70"/>
-      <c r="J36" s="72"/>
+      <c r="I36" s="83"/>
+      <c r="J36" s="70"/>
       <c r="K36" s="52"/>
     </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="69" t="s">
+    <row r="37" spans="1:11" ht="15" thickBot="1">
+      <c r="A37" s="67" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="39">
+      <c r="C37" s="76">
         <v>45723</v>
       </c>
-      <c r="D37" s="39">
+      <c r="D37" s="76">
         <v>45729</v>
       </c>
       <c r="E37" s="39"/>
@@ -2312,22 +2361,22 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="71">
-        <v>45910</v>
-      </c>
-      <c r="J37" s="71"/>
+      <c r="I37" s="82">
+        <v>46295</v>
+      </c>
+      <c r="J37" s="69"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="70"/>
+      <c r="A38" s="68"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="36">
-        <v>45729</v>
-      </c>
-      <c r="D38" s="36">
-        <v>45862</v>
+      <c r="C38" s="77">
+        <v>46264</v>
+      </c>
+      <c r="D38" s="77">
+        <v>46275</v>
       </c>
       <c r="E38" s="36"/>
       <c r="F38" s="36"/>
@@ -2337,19 +2386,23 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="70"/>
-      <c r="J38" s="72"/>
+      <c r="I38" s="83"/>
+      <c r="J38" s="70"/>
       <c r="K38" s="52"/>
     </row>
-    <row r="39" spans="1:11">
-      <c r="A39" s="69" t="s">
+    <row r="39" spans="1:11" ht="15" thickBot="1">
+      <c r="A39" s="67" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
+      <c r="C39" s="80">
+        <v>46280</v>
+      </c>
+      <c r="D39" s="80">
+        <v>46290</v>
+      </c>
       <c r="E39" s="39"/>
       <c r="F39" s="39"/>
       <c r="G39" s="40">
@@ -2358,17 +2411,23 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="71"/>
-      <c r="J39" s="71"/>
+      <c r="I39" s="82">
+        <v>46539</v>
+      </c>
+      <c r="J39" s="69"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="70"/>
+      <c r="A40" s="68"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C40" s="56"/>
-      <c r="D40" s="56"/>
+      <c r="C40" s="80">
+        <v>46510</v>
+      </c>
+      <c r="D40" s="80">
+        <v>46517</v>
+      </c>
       <c r="E40" s="56"/>
       <c r="F40" s="56"/>
       <c r="G40" s="57">
@@ -2377,22 +2436,22 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="70"/>
-      <c r="J40" s="72"/>
+      <c r="I40" s="83"/>
+      <c r="J40" s="70"/>
       <c r="K40" s="52"/>
     </row>
-    <row r="41" spans="1:11">
-      <c r="A41" s="69" t="s">
+    <row r="41" spans="1:11" ht="15" thickBot="1">
+      <c r="A41" s="67" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="39">
-        <v>46226</v>
-      </c>
-      <c r="D41" s="39">
-        <v>46228</v>
+      <c r="C41" s="81">
+        <v>46225</v>
+      </c>
+      <c r="D41" s="81">
+        <v>46237</v>
       </c>
       <c r="E41" s="39"/>
       <c r="F41" s="39"/>
@@ -2402,36 +2461,40 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="71">
+      <c r="I41" s="82">
         <v>46237</v>
       </c>
-      <c r="J41" s="71"/>
+      <c r="J41" s="69"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="70"/>
+      <c r="A42" s="68"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C42" s="56"/>
-      <c r="D42" s="56"/>
+      <c r="C42" s="80"/>
+      <c r="D42" s="80"/>
       <c r="E42" s="56"/>
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="70"/>
-      <c r="J42" s="72"/>
+      <c r="I42" s="83"/>
+      <c r="J42" s="70"/>
       <c r="K42" s="52"/>
     </row>
-    <row r="43" spans="1:11">
-      <c r="A43" s="69" t="s">
+    <row r="43" spans="1:11" ht="15" thickBot="1">
+      <c r="A43" s="67" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C43" s="39"/>
-      <c r="D43" s="39"/>
+      <c r="C43" s="80">
+        <v>46290</v>
+      </c>
+      <c r="D43" s="80">
+        <v>46305</v>
+      </c>
       <c r="E43" s="39"/>
       <c r="F43" s="39"/>
       <c r="G43" s="40">
@@ -2440,17 +2503,23 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="71"/>
-      <c r="J43" s="71"/>
+      <c r="I43" s="82">
+        <v>46447</v>
+      </c>
+      <c r="J43" s="69"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="70"/>
+      <c r="A44" s="68"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="56"/>
-      <c r="D44" s="56"/>
+      <c r="C44" s="80">
+        <v>46419</v>
+      </c>
+      <c r="D44" s="80">
+        <v>46428</v>
+      </c>
       <c r="E44" s="56"/>
       <c r="F44" s="56"/>
       <c r="G44" s="57">
@@ -2459,20 +2528,12 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="70"/>
-      <c r="J44" s="72"/>
+      <c r="I44" s="83"/>
+      <c r="J44" s="70"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="7">
-      <filters blank="1">
-        <filter val="Construction"/>
-        <filter val="On Hold"/>
-        <filter val="Planning"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="62">
     <mergeCell ref="J37:J38"/>
     <mergeCell ref="J21:J22"/>
@@ -2537,7 +2598,7 @@
     <mergeCell ref="I41:I42"/>
     <mergeCell ref="J41:J42"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -2572,56 +2633,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="65"/>
+      <c r="V1" s="65"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="68"/>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
-      <c r="U2" s="68"/>
-      <c r="V2" s="68"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="66"/>
+      <c r="M2" s="66"/>
+      <c r="N2" s="66"/>
+      <c r="O2" s="66"/>
+      <c r="P2" s="66"/>
+      <c r="Q2" s="66"/>
+      <c r="R2" s="66"/>
+      <c r="S2" s="66"/>
+      <c r="T2" s="66"/>
+      <c r="U2" s="66"/>
+      <c r="V2" s="66"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -2738,8 +2799,8 @@
         <f>'[1]Master Schedule'!C5</f>
         <v>46084</v>
       </c>
-      <c r="R5" s="81">
-        <v>46248</v>
+      <c r="R5" s="19">
+        <v>46106</v>
       </c>
       <c r="S5" s="14"/>
       <c r="T5" s="25" t="s">
@@ -2998,7 +3059,7 @@
         <v>138000</v>
       </c>
       <c r="G10" s="16">
-        <v>370</v>
+        <v>470</v>
       </c>
       <c r="H10" s="16">
         <f>E10*1</f>
@@ -3236,7 +3297,8 @@
         <v>525343.22400000005</v>
       </c>
       <c r="G14" s="16">
-        <v>215</v>
+        <f>215+146.7</f>
+        <v>361.7</v>
       </c>
       <c r="H14" s="16">
         <f>E14*0.8</f>
@@ -3593,7 +3655,7 @@
         <v>45717</v>
       </c>
       <c r="R20" s="19">
-        <v>45899</v>
+        <v>45737</v>
       </c>
       <c r="T20" s="26" t="s">
         <v>65</v>
@@ -3637,7 +3699,7 @@
         <v>45717</v>
       </c>
       <c r="R21" s="19">
-        <v>45910</v>
+        <v>45737</v>
       </c>
       <c r="T21" s="26" t="s">
         <v>126</v>
@@ -3657,7 +3719,8 @@
       <c r="D22" s="15"/>
       <c r="F22" s="24"/>
       <c r="G22" s="9">
-        <v>2484</v>
+        <f>2484+107</f>
+        <v>2591</v>
       </c>
       <c r="M22" s="9">
         <v>10000</v>
@@ -3760,7 +3823,7 @@
         <v>46225</v>
       </c>
       <c r="R24" s="11">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="T24" s="26" t="s">
         <v>140</v>
@@ -3782,7 +3845,7 @@
       <c r="C25" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="66">
+      <c r="D25" s="64">
         <v>0</v>
       </c>
       <c r="E25" s="12">
@@ -4343,7 +4406,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -4354,20 +4417,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="66" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4722,16 +4785,16 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="65">
+      <c r="A26" s="63">
         <v>46219</v>
       </c>
-      <c r="B26" s="64" t="s">
+      <c r="B26" s="62" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="64" t="s">
+      <c r="C26" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="63">
+      <c r="D26" s="61">
         <v>3</v>
       </c>
       <c r="E26" t="s">
@@ -4742,10 +4805,10 @@
       <c r="A27" s="3">
         <v>46224</v>
       </c>
-      <c r="B27" s="64" t="s">
+      <c r="B27" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="64" t="s">
+      <c r="C27" s="62" t="s">
         <v>61</v>
       </c>
       <c r="D27" s="4">
@@ -4762,7 +4825,7 @@
       <c r="B28" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="65" t="s">
+      <c r="C28" s="63" t="s">
         <v>61</v>
       </c>
       <c r="D28" s="4">
@@ -4779,7 +4842,7 @@
       <c r="B29" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C29" s="65" t="s">
+      <c r="C29" s="63" t="s">
         <v>61</v>
       </c>
       <c r="D29" s="4">
@@ -4796,7 +4859,7 @@
       <c r="B30" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C30" s="65" t="s">
+      <c r="C30" s="63" t="s">
         <v>61</v>
       </c>
       <c r="D30" s="4">
@@ -4804,6 +4867,23 @@
       </c>
       <c r="E30" t="s">
         <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="3">
+        <v>46234</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="63" t="s">
+        <v>61</v>
+      </c>
+      <c r="D31" s="4">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -4828,22 +4908,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="66" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4876,7 +4956,7 @@
         <v>46224</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4910,7 +4990,7 @@
         <v>46224</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -5763,15 +5843,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5784,7 +5855,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -6037,15 +6108,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -6056,7 +6128,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6073,4 +6145,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-08-07 09:12)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{F600DE45-4501-465C-9806-A81742F36D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6683723C-A3B6-44E3-855E-63C92E5D4C5A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1049,49 +1049,40 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1100,6 +1091,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma 2 2 3 2" xfId="3" xr:uid="{10CA6883-C0B4-442D-A7D0-FF27A9ED468E}"/>
@@ -1476,34 +1476,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="83"/>
+      <c r="J2" s="83"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="4" spans="1:11" ht="28.2" thickBot="1">
       <c r="A4" s="1" t="s">
@@ -1541,16 +1541,16 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" thickBot="1">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="85" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="76">
+      <c r="C5" s="65">
         <v>46084</v>
       </c>
-      <c r="D5" s="76">
+      <c r="D5" s="65">
         <v>46127</v>
       </c>
       <c r="E5" s="59"/>
@@ -1561,21 +1561,21 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="82">
+      <c r="I5" s="77">
         <v>46244</v>
       </c>
-      <c r="J5" s="75"/>
+      <c r="J5" s="73"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="68"/>
+      <c r="A6" s="76"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="76">
+      <c r="C6" s="65">
         <v>46189</v>
       </c>
-      <c r="D6" s="76">
+      <c r="D6" s="65">
         <v>46189</v>
       </c>
       <c r="E6" s="45"/>
@@ -1586,21 +1586,21 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="83"/>
-      <c r="J6" s="70"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="72"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="75" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="77">
+      <c r="C7" s="66">
         <v>46266</v>
       </c>
-      <c r="D7" s="77">
+      <c r="D7" s="66">
         <v>46275</v>
       </c>
       <c r="E7" s="39"/>
@@ -1611,21 +1611,21 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="82">
+      <c r="I7" s="77">
         <v>46366</v>
       </c>
-      <c r="J7" s="69"/>
+      <c r="J7" s="71"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="68"/>
+      <c r="A8" s="76"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="77">
+      <c r="C8" s="66">
         <v>46305</v>
       </c>
-      <c r="D8" s="77">
+      <c r="D8" s="66">
         <v>46308</v>
       </c>
       <c r="E8" s="36"/>
@@ -1636,21 +1636,21 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="83"/>
-      <c r="J8" s="70"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="72"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
-      <c r="A9" s="67" t="s">
+      <c r="A9" s="75" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="65">
         <v>46082</v>
       </c>
-      <c r="D9" s="76">
+      <c r="D9" s="65">
         <v>46096</v>
       </c>
       <c r="E9" s="39"/>
@@ -1661,21 +1661,21 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="82">
+      <c r="I9" s="77">
         <v>46218</v>
       </c>
-      <c r="J9" s="69"/>
+      <c r="J9" s="71"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="68"/>
+      <c r="A10" s="76"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="76">
+      <c r="C10" s="65">
         <v>46168</v>
       </c>
-      <c r="D10" s="76">
+      <c r="D10" s="65">
         <v>46213</v>
       </c>
       <c r="E10" s="36"/>
@@ -1686,21 +1686,21 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="83"/>
-      <c r="J10" s="70"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="72"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11" ht="15" thickBot="1">
-      <c r="A11" s="67" t="s">
+      <c r="A11" s="75" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="76">
+      <c r="C11" s="65">
         <v>46184</v>
       </c>
-      <c r="D11" s="76">
+      <c r="D11" s="65">
         <v>46191</v>
       </c>
       <c r="E11" s="42"/>
@@ -1711,21 +1711,21 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="82">
+      <c r="I11" s="77">
         <v>46171</v>
       </c>
-      <c r="J11" s="69"/>
+      <c r="J11" s="71"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="68"/>
+      <c r="A12" s="76"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="76">
+      <c r="C12" s="65">
         <v>46200</v>
       </c>
-      <c r="D12" s="76">
+      <c r="D12" s="65">
         <v>46202</v>
       </c>
       <c r="E12" s="45"/>
@@ -1736,21 +1736,21 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="83"/>
-      <c r="J12" s="70"/>
+      <c r="I12" s="78"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11" ht="15" thickBot="1">
-      <c r="A13" s="67" t="s">
+      <c r="A13" s="75" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="77">
+      <c r="C13" s="66">
         <v>46392</v>
       </c>
-      <c r="D13" s="77">
+      <c r="D13" s="66">
         <v>46402</v>
       </c>
       <c r="E13" s="39"/>
@@ -1761,21 +1761,21 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="84">
+      <c r="I13" s="79">
         <v>46419</v>
       </c>
-      <c r="J13" s="69"/>
+      <c r="J13" s="71"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="68"/>
+      <c r="A14" s="76"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="77">
+      <c r="C14" s="66">
         <v>46423</v>
       </c>
-      <c r="D14" s="77">
+      <c r="D14" s="66">
         <v>46428</v>
       </c>
       <c r="E14" s="36"/>
@@ -1786,21 +1786,21 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="85"/>
-      <c r="J14" s="70"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="72"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11" ht="15" thickBot="1">
-      <c r="A15" s="67" t="s">
+      <c r="A15" s="75" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="76">
+      <c r="C15" s="65">
         <v>46168</v>
       </c>
-      <c r="D15" s="76">
+      <c r="D15" s="65">
         <v>46188</v>
       </c>
       <c r="E15" s="42"/>
@@ -1811,21 +1811,21 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="82">
+      <c r="I15" s="77">
         <v>46199</v>
       </c>
-      <c r="J15" s="69"/>
+      <c r="J15" s="71"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="68"/>
+      <c r="A16" s="76"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="76">
+      <c r="C16" s="65">
         <v>46198</v>
       </c>
-      <c r="D16" s="76">
+      <c r="D16" s="65">
         <v>46199</v>
       </c>
       <c r="E16" s="45"/>
@@ -1836,21 +1836,21 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="83"/>
-      <c r="J16" s="70"/>
+      <c r="I16" s="78"/>
+      <c r="J16" s="72"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1">
-      <c r="A17" s="73" t="s">
+      <c r="A17" s="81" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="76">
+      <c r="C17" s="65">
         <v>46188</v>
       </c>
-      <c r="D17" s="76">
+      <c r="D17" s="65">
         <v>46198</v>
       </c>
       <c r="E17" s="33"/>
@@ -1861,21 +1861,21 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="82">
+      <c r="I17" s="77">
         <v>46305</v>
       </c>
-      <c r="J17" s="72"/>
+      <c r="J17" s="74"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="68"/>
+      <c r="A18" s="76"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="78">
+      <c r="C18" s="67">
         <v>46296</v>
       </c>
-      <c r="D18" s="78">
+      <c r="D18" s="67">
         <v>46298</v>
       </c>
       <c r="E18" s="36"/>
@@ -1886,21 +1886,21 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="83"/>
-      <c r="J18" s="70"/>
+      <c r="I18" s="78"/>
+      <c r="J18" s="72"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11" ht="15" thickBot="1">
-      <c r="A19" s="73" t="s">
+      <c r="A19" s="81" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="77">
+      <c r="C19" s="66">
         <v>46366</v>
       </c>
-      <c r="D19" s="77">
+      <c r="D19" s="66">
         <v>46381</v>
       </c>
       <c r="E19" s="33"/>
@@ -1911,21 +1911,21 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="84">
+      <c r="I19" s="79">
         <v>46419</v>
       </c>
-      <c r="J19" s="72"/>
+      <c r="J19" s="74"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="68"/>
+      <c r="A20" s="76"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="77">
+      <c r="C20" s="66">
         <v>46388</v>
       </c>
-      <c r="D20" s="77">
+      <c r="D20" s="66">
         <v>46390</v>
       </c>
       <c r="E20" s="36"/>
@@ -1936,21 +1936,21 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="85"/>
-      <c r="J20" s="70"/>
+      <c r="I20" s="80"/>
+      <c r="J20" s="72"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="75" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="77">
+      <c r="C21" s="66">
         <v>46240</v>
       </c>
-      <c r="D21" s="77">
+      <c r="D21" s="66">
         <v>46249</v>
       </c>
       <c r="E21" s="39"/>
@@ -1961,21 +1961,21 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="84">
+      <c r="I21" s="79">
         <v>46397</v>
       </c>
-      <c r="J21" s="69"/>
+      <c r="J21" s="71"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="68"/>
+      <c r="A22" s="76"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="77">
+      <c r="C22" s="66">
         <v>46327</v>
       </c>
-      <c r="D22" s="77">
+      <c r="D22" s="66">
         <v>46329</v>
       </c>
       <c r="E22" s="36"/>
@@ -1986,21 +1986,21 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="85"/>
-      <c r="J22" s="70"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="72"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11" ht="15" thickBot="1">
-      <c r="A23" s="67" t="s">
+      <c r="A23" s="75" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="76">
+      <c r="C23" s="65">
         <v>46197</v>
       </c>
-      <c r="D23" s="76">
+      <c r="D23" s="65">
         <v>46209</v>
       </c>
       <c r="E23" s="42"/>
@@ -2011,21 +2011,21 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="82">
+      <c r="I23" s="77">
         <v>46237</v>
       </c>
-      <c r="J23" s="69"/>
+      <c r="J23" s="71"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="68"/>
+      <c r="A24" s="76"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="76">
+      <c r="C24" s="65">
         <v>46209</v>
       </c>
-      <c r="D24" s="76">
+      <c r="D24" s="65">
         <v>46211</v>
       </c>
       <c r="E24" s="45"/>
@@ -2036,21 +2036,21 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="83"/>
-      <c r="J24" s="70"/>
+      <c r="I24" s="78"/>
+      <c r="J24" s="72"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11" ht="15" thickBot="1">
-      <c r="A25" s="67" t="s">
+      <c r="A25" s="75" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="65">
         <v>46185</v>
       </c>
-      <c r="D25" s="76">
+      <c r="D25" s="65">
         <v>46188</v>
       </c>
       <c r="E25" s="42"/>
@@ -2061,21 +2061,21 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="82">
+      <c r="I25" s="77">
         <v>46188</v>
       </c>
-      <c r="J25" s="69"/>
+      <c r="J25" s="71"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="68"/>
+      <c r="A26" s="76"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="76">
+      <c r="C26" s="65">
         <v>46185</v>
       </c>
-      <c r="D26" s="76">
+      <c r="D26" s="65">
         <v>46188</v>
       </c>
       <c r="E26" s="45"/>
@@ -2086,21 +2086,21 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="83"/>
-      <c r="J26" s="70"/>
+      <c r="I26" s="78"/>
+      <c r="J26" s="72"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11" ht="15" thickBot="1">
-      <c r="A27" s="67" t="s">
+      <c r="A27" s="75" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C27" s="79">
+      <c r="C27" s="68">
         <v>46275</v>
       </c>
-      <c r="D27" s="79">
+      <c r="D27" s="68">
         <v>46295</v>
       </c>
       <c r="E27" s="39"/>
@@ -2111,21 +2111,21 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="84">
+      <c r="I27" s="79">
         <v>46382</v>
       </c>
-      <c r="J27" s="69"/>
+      <c r="J27" s="71"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="68"/>
+      <c r="A28" s="76"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="79">
+      <c r="C28" s="68">
         <v>46345</v>
       </c>
-      <c r="D28" s="79">
+      <c r="D28" s="68">
         <v>46347</v>
       </c>
       <c r="E28" s="36"/>
@@ -2136,21 +2136,21 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="85"/>
-      <c r="J28" s="70"/>
+      <c r="I28" s="80"/>
+      <c r="J28" s="72"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11" ht="15" thickBot="1">
-      <c r="A29" s="67" t="s">
+      <c r="A29" s="75" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="76">
+      <c r="C29" s="65">
         <v>46091</v>
       </c>
-      <c r="D29" s="76">
+      <c r="D29" s="65">
         <v>46100</v>
       </c>
       <c r="E29" s="42"/>
@@ -2161,21 +2161,21 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="82">
+      <c r="I29" s="77">
         <v>46139</v>
       </c>
-      <c r="J29" s="69"/>
+      <c r="J29" s="71"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="68"/>
+      <c r="A30" s="76"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="76">
+      <c r="C30" s="65">
         <v>46120</v>
       </c>
-      <c r="D30" s="76">
+      <c r="D30" s="65">
         <v>46124</v>
       </c>
       <c r="E30" s="45"/>
@@ -2186,21 +2186,21 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="83"/>
-      <c r="J30" s="70"/>
+      <c r="I30" s="78"/>
+      <c r="J30" s="72"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11" ht="15" thickBot="1">
-      <c r="A31" s="67" t="s">
+      <c r="A31" s="75" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C31" s="76">
+      <c r="C31" s="65">
         <v>46091</v>
       </c>
-      <c r="D31" s="76">
+      <c r="D31" s="65">
         <v>46094</v>
       </c>
       <c r="E31" s="42"/>
@@ -2211,21 +2211,21 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="82">
+      <c r="I31" s="77">
         <v>46133</v>
       </c>
-      <c r="J31" s="69"/>
+      <c r="J31" s="71"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="68"/>
+      <c r="A32" s="76"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C32" s="76">
+      <c r="C32" s="65">
         <v>46091</v>
       </c>
-      <c r="D32" s="76">
+      <c r="D32" s="65">
         <v>46094</v>
       </c>
       <c r="E32" s="45"/>
@@ -2236,21 +2236,21 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="83"/>
-      <c r="J32" s="70"/>
+      <c r="I32" s="78"/>
+      <c r="J32" s="72"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11" ht="15" thickBot="1">
-      <c r="A33" s="67" t="s">
+      <c r="A33" s="75" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="77">
+      <c r="C33" s="66">
         <v>46237</v>
       </c>
-      <c r="D33" s="77">
+      <c r="D33" s="66">
         <v>46248</v>
       </c>
       <c r="E33" s="39"/>
@@ -2261,21 +2261,21 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="82">
+      <c r="I33" s="77">
         <v>46342</v>
       </c>
-      <c r="J33" s="69"/>
+      <c r="J33" s="71"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="68"/>
+      <c r="A34" s="76"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="77">
+      <c r="C34" s="66">
         <v>46296</v>
       </c>
-      <c r="D34" s="77">
+      <c r="D34" s="66">
         <v>46303</v>
       </c>
       <c r="E34" s="36"/>
@@ -2286,21 +2286,21 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="83"/>
-      <c r="J34" s="70"/>
+      <c r="I34" s="78"/>
+      <c r="J34" s="72"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11" ht="15" thickBot="1">
-      <c r="A35" s="67" t="s">
+      <c r="A35" s="75" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C35" s="76">
+      <c r="C35" s="65">
         <v>45723</v>
       </c>
-      <c r="D35" s="76">
+      <c r="D35" s="65">
         <v>45729</v>
       </c>
       <c r="E35" s="39"/>
@@ -2311,21 +2311,21 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="82">
+      <c r="I35" s="77">
         <v>46264</v>
       </c>
-      <c r="J35" s="69"/>
+      <c r="J35" s="71"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="68"/>
+      <c r="A36" s="76"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="78">
+      <c r="C36" s="67">
         <v>46259</v>
       </c>
-      <c r="D36" s="78">
+      <c r="D36" s="67">
         <v>46264</v>
       </c>
       <c r="E36" s="36"/>
@@ -2336,21 +2336,21 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="83"/>
-      <c r="J36" s="70"/>
+      <c r="I36" s="78"/>
+      <c r="J36" s="72"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11" ht="15" thickBot="1">
-      <c r="A37" s="67" t="s">
+      <c r="A37" s="75" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="76">
+      <c r="C37" s="65">
         <v>45723</v>
       </c>
-      <c r="D37" s="76">
+      <c r="D37" s="65">
         <v>45729</v>
       </c>
       <c r="E37" s="39"/>
@@ -2361,21 +2361,21 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="82">
+      <c r="I37" s="77">
         <v>46295</v>
       </c>
-      <c r="J37" s="69"/>
+      <c r="J37" s="71"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="68"/>
+      <c r="A38" s="76"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="77">
+      <c r="C38" s="66">
         <v>46264</v>
       </c>
-      <c r="D38" s="77">
+      <c r="D38" s="66">
         <v>46275</v>
       </c>
       <c r="E38" s="36"/>
@@ -2386,21 +2386,21 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="83"/>
-      <c r="J38" s="70"/>
+      <c r="I38" s="78"/>
+      <c r="J38" s="72"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11" ht="15" thickBot="1">
-      <c r="A39" s="67" t="s">
+      <c r="A39" s="75" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="80">
+      <c r="C39" s="69">
         <v>46280</v>
       </c>
-      <c r="D39" s="80">
+      <c r="D39" s="69">
         <v>46290</v>
       </c>
       <c r="E39" s="39"/>
@@ -2411,21 +2411,21 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="82">
+      <c r="I39" s="77">
         <v>46539</v>
       </c>
-      <c r="J39" s="69"/>
+      <c r="J39" s="71"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="68"/>
+      <c r="A40" s="76"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C40" s="80">
+      <c r="C40" s="69">
         <v>46510</v>
       </c>
-      <c r="D40" s="80">
+      <c r="D40" s="69">
         <v>46517</v>
       </c>
       <c r="E40" s="56"/>
@@ -2436,21 +2436,21 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="83"/>
-      <c r="J40" s="70"/>
+      <c r="I40" s="78"/>
+      <c r="J40" s="72"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11" ht="15" thickBot="1">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="75" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="81">
+      <c r="C41" s="70">
         <v>46225</v>
       </c>
-      <c r="D41" s="81">
+      <c r="D41" s="70">
         <v>46237</v>
       </c>
       <c r="E41" s="39"/>
@@ -2461,38 +2461,38 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="82">
+      <c r="I41" s="77">
         <v>46237</v>
       </c>
-      <c r="J41" s="69"/>
+      <c r="J41" s="71"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="68"/>
+      <c r="A42" s="76"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C42" s="80"/>
-      <c r="D42" s="80"/>
+      <c r="C42" s="69"/>
+      <c r="D42" s="69"/>
       <c r="E42" s="56"/>
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="83"/>
-      <c r="J42" s="70"/>
+      <c r="I42" s="78"/>
+      <c r="J42" s="72"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11" ht="15" thickBot="1">
-      <c r="A43" s="67" t="s">
+      <c r="A43" s="75" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C43" s="80">
+      <c r="C43" s="69">
         <v>46290</v>
       </c>
-      <c r="D43" s="80">
+      <c r="D43" s="69">
         <v>46305</v>
       </c>
       <c r="E43" s="39"/>
@@ -2503,21 +2503,21 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="82">
+      <c r="I43" s="77">
         <v>46447</v>
       </c>
-      <c r="J43" s="69"/>
+      <c r="J43" s="71"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="68"/>
+      <c r="A44" s="76"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="80">
+      <c r="C44" s="69">
         <v>46419</v>
       </c>
-      <c r="D44" s="80">
+      <c r="D44" s="69">
         <v>46428</v>
       </c>
       <c r="E44" s="56"/>
@@ -2528,27 +2528,45 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="83"/>
-      <c r="J44" s="70"/>
+      <c r="I44" s="78"/>
+      <c r="J44" s="72"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="62">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2565,38 +2583,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2633,56 +2633,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="82" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
-      <c r="N1" s="65"/>
-      <c r="O1" s="65"/>
-      <c r="P1" s="65"/>
-      <c r="Q1" s="65"/>
-      <c r="R1" s="65"/>
-      <c r="S1" s="65"/>
-      <c r="T1" s="65"/>
-      <c r="U1" s="65"/>
-      <c r="V1" s="65"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="82"/>
+      <c r="S1" s="82"/>
+      <c r="T1" s="82"/>
+      <c r="U1" s="82"/>
+      <c r="V1" s="82"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="66"/>
-      <c r="O2" s="66"/>
-      <c r="P2" s="66"/>
-      <c r="Q2" s="66"/>
-      <c r="R2" s="66"/>
-      <c r="S2" s="66"/>
-      <c r="T2" s="66"/>
-      <c r="U2" s="66"/>
-      <c r="V2" s="66"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="84"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
+      <c r="N2" s="84"/>
+      <c r="O2" s="84"/>
+      <c r="P2" s="84"/>
+      <c r="Q2" s="84"/>
+      <c r="R2" s="84"/>
+      <c r="S2" s="84"/>
+      <c r="T2" s="84"/>
+      <c r="U2" s="84"/>
+      <c r="V2" s="84"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -4417,20 +4417,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="82" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="84" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4908,22 +4908,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="82" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="84" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5843,16 +5843,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6109,21 +6105,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6148,9 +6145,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-08-07 09:31)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76A77EEA-30F4-4EB8-91CD-2D3EA821E969}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -1067,18 +1067,6 @@
     <xf numFmtId="164" fontId="18" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1087,6 +1075,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="19" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1094,11 +1090,15 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1476,34 +1476,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="83"/>
-      <c r="J2" s="83"/>
-      <c r="K2" s="83"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
     </row>
     <row r="4" spans="1:11" ht="28.2" thickBot="1">
       <c r="A4" s="1" t="s">
@@ -1541,7 +1541,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" thickBot="1">
-      <c r="A5" s="85" t="s">
+      <c r="A5" s="83" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
@@ -1561,14 +1561,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="77">
+      <c r="I5" s="73">
         <v>46244</v>
       </c>
-      <c r="J5" s="73"/>
+      <c r="J5" s="85"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="76"/>
+      <c r="A6" s="72"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1586,12 +1586,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="78"/>
-      <c r="J6" s="72"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="76"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="71" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1611,14 +1611,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="77">
+      <c r="I7" s="73">
         <v>46366</v>
       </c>
-      <c r="J7" s="71"/>
+      <c r="J7" s="75"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="76"/>
+      <c r="A8" s="72"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1636,12 +1636,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="78"/>
-      <c r="J8" s="72"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="76"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
-      <c r="A9" s="75" t="s">
+      <c r="A9" s="71" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1661,14 +1661,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="77">
+      <c r="I9" s="73">
         <v>46218</v>
       </c>
-      <c r="J9" s="71"/>
+      <c r="J9" s="75"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="76"/>
+      <c r="A10" s="72"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1686,12 +1686,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="78"/>
-      <c r="J10" s="72"/>
+      <c r="I10" s="74"/>
+      <c r="J10" s="76"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11" ht="15" thickBot="1">
-      <c r="A11" s="75" t="s">
+      <c r="A11" s="71" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1711,14 +1711,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="77">
+      <c r="I11" s="73">
         <v>46171</v>
       </c>
-      <c r="J11" s="71"/>
+      <c r="J11" s="75"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="76"/>
+      <c r="A12" s="72"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1736,12 +1736,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="78"/>
-      <c r="J12" s="72"/>
+      <c r="I12" s="74"/>
+      <c r="J12" s="76"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11" ht="15" thickBot="1">
-      <c r="A13" s="75" t="s">
+      <c r="A13" s="71" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1764,11 +1764,11 @@
       <c r="I13" s="79">
         <v>46419</v>
       </c>
-      <c r="J13" s="71"/>
+      <c r="J13" s="75"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="76"/>
+      <c r="A14" s="72"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1787,11 +1787,11 @@
         <v>15</v>
       </c>
       <c r="I14" s="80"/>
-      <c r="J14" s="72"/>
+      <c r="J14" s="76"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11" ht="15" thickBot="1">
-      <c r="A15" s="75" t="s">
+      <c r="A15" s="71" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1811,14 +1811,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="77">
+      <c r="I15" s="73">
         <v>46199</v>
       </c>
-      <c r="J15" s="71"/>
+      <c r="J15" s="75"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="76"/>
+      <c r="A16" s="72"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1836,8 +1836,8 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="78"/>
-      <c r="J16" s="72"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="76"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1">
@@ -1861,14 +1861,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="77">
+      <c r="I17" s="73">
         <v>46305</v>
       </c>
-      <c r="J17" s="74"/>
+      <c r="J17" s="84"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="76"/>
+      <c r="A18" s="72"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1886,8 +1886,8 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="78"/>
-      <c r="J18" s="72"/>
+      <c r="I18" s="74"/>
+      <c r="J18" s="76"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11" ht="15" thickBot="1">
@@ -1914,11 +1914,11 @@
       <c r="I19" s="79">
         <v>46419</v>
       </c>
-      <c r="J19" s="74"/>
+      <c r="J19" s="84"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="76"/>
+      <c r="A20" s="72"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1937,11 +1937,11 @@
         <v>15</v>
       </c>
       <c r="I20" s="80"/>
-      <c r="J20" s="72"/>
+      <c r="J20" s="76"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1">
-      <c r="A21" s="75" t="s">
+      <c r="A21" s="71" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1964,11 +1964,11 @@
       <c r="I21" s="79">
         <v>46397</v>
       </c>
-      <c r="J21" s="71"/>
+      <c r="J21" s="75"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="76"/>
+      <c r="A22" s="72"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1987,11 +1987,11 @@
         <v>15</v>
       </c>
       <c r="I22" s="80"/>
-      <c r="J22" s="72"/>
+      <c r="J22" s="76"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11" ht="15" thickBot="1">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="71" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -2011,14 +2011,14 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="77">
+      <c r="I23" s="73">
         <v>46237</v>
       </c>
-      <c r="J23" s="71"/>
+      <c r="J23" s="75"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="76"/>
+      <c r="A24" s="72"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -2036,12 +2036,12 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="78"/>
-      <c r="J24" s="72"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="76"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11" ht="15" thickBot="1">
-      <c r="A25" s="75" t="s">
+      <c r="A25" s="71" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -2061,14 +2061,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="77">
+      <c r="I25" s="73">
         <v>46188</v>
       </c>
-      <c r="J25" s="71"/>
+      <c r="J25" s="75"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="76"/>
+      <c r="A26" s="72"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2086,12 +2086,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="78"/>
-      <c r="J26" s="72"/>
+      <c r="I26" s="74"/>
+      <c r="J26" s="76"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11" ht="15" thickBot="1">
-      <c r="A27" s="75" t="s">
+      <c r="A27" s="71" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2114,11 +2114,11 @@
       <c r="I27" s="79">
         <v>46382</v>
       </c>
-      <c r="J27" s="71"/>
+      <c r="J27" s="75"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="76"/>
+      <c r="A28" s="72"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2137,11 +2137,11 @@
         <v>22</v>
       </c>
       <c r="I28" s="80"/>
-      <c r="J28" s="72"/>
+      <c r="J28" s="76"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11" ht="15" thickBot="1">
-      <c r="A29" s="75" t="s">
+      <c r="A29" s="71" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2161,14 +2161,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="77">
+      <c r="I29" s="73">
         <v>46139</v>
       </c>
-      <c r="J29" s="71"/>
+      <c r="J29" s="75"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="76"/>
+      <c r="A30" s="72"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2186,12 +2186,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="78"/>
-      <c r="J30" s="72"/>
+      <c r="I30" s="74"/>
+      <c r="J30" s="76"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11" ht="15" thickBot="1">
-      <c r="A31" s="75" t="s">
+      <c r="A31" s="71" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2211,14 +2211,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="77">
+      <c r="I31" s="73">
         <v>46133</v>
       </c>
-      <c r="J31" s="71"/>
+      <c r="J31" s="75"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="76"/>
+      <c r="A32" s="72"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2236,12 +2236,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="78"/>
-      <c r="J32" s="72"/>
+      <c r="I32" s="74"/>
+      <c r="J32" s="76"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11" ht="15" thickBot="1">
-      <c r="A33" s="75" t="s">
+      <c r="A33" s="71" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2261,14 +2261,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="77">
+      <c r="I33" s="73">
         <v>46342</v>
       </c>
-      <c r="J33" s="71"/>
+      <c r="J33" s="75"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="76"/>
+      <c r="A34" s="72"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2286,12 +2286,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="78"/>
-      <c r="J34" s="72"/>
+      <c r="I34" s="74"/>
+      <c r="J34" s="76"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11" ht="15" thickBot="1">
-      <c r="A35" s="75" t="s">
+      <c r="A35" s="71" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2311,14 +2311,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="77">
+      <c r="I35" s="73">
         <v>46264</v>
       </c>
-      <c r="J35" s="71"/>
+      <c r="J35" s="75"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="76"/>
+      <c r="A36" s="72"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2336,12 +2336,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="78"/>
-      <c r="J36" s="72"/>
+      <c r="I36" s="74"/>
+      <c r="J36" s="76"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11" ht="15" thickBot="1">
-      <c r="A37" s="75" t="s">
+      <c r="A37" s="71" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2361,14 +2361,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="77">
+      <c r="I37" s="73">
         <v>46295</v>
       </c>
-      <c r="J37" s="71"/>
+      <c r="J37" s="75"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="76"/>
+      <c r="A38" s="72"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2386,12 +2386,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="78"/>
-      <c r="J38" s="72"/>
+      <c r="I38" s="74"/>
+      <c r="J38" s="76"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11" ht="15" thickBot="1">
-      <c r="A39" s="75" t="s">
+      <c r="A39" s="71" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2411,14 +2411,14 @@
       <c r="H39" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="77">
+      <c r="I39" s="73">
         <v>46539</v>
       </c>
-      <c r="J39" s="71"/>
+      <c r="J39" s="75"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="76"/>
+      <c r="A40" s="72"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2436,12 +2436,12 @@
       <c r="H40" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="I40" s="78"/>
-      <c r="J40" s="72"/>
+      <c r="I40" s="74"/>
+      <c r="J40" s="76"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11" ht="15" thickBot="1">
-      <c r="A41" s="75" t="s">
+      <c r="A41" s="71" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2461,14 +2461,14 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="77">
+      <c r="I41" s="73">
         <v>46237</v>
       </c>
-      <c r="J41" s="71"/>
+      <c r="J41" s="75"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="76"/>
+      <c r="A42" s="72"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2478,12 +2478,12 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="78"/>
-      <c r="J42" s="72"/>
+      <c r="I42" s="74"/>
+      <c r="J42" s="76"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11" ht="15" thickBot="1">
-      <c r="A43" s="75" t="s">
+      <c r="A43" s="71" t="s">
         <v>136</v>
       </c>
       <c r="B43" s="38" t="s">
@@ -2503,14 +2503,14 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="77">
+      <c r="I43" s="73">
         <v>46447</v>
       </c>
-      <c r="J43" s="71"/>
+      <c r="J43" s="75"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="76"/>
+      <c r="A44" s="72"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2528,22 +2528,50 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="78"/>
-      <c r="J44" s="72"/>
+      <c r="I44" s="74"/>
+      <c r="J44" s="76"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="62">
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="A1:K1"/>
@@ -2560,43 +2588,15 @@
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2633,56 +2633,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="77" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82"/>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
-      <c r="Q1" s="82"/>
-      <c r="R1" s="82"/>
-      <c r="S1" s="82"/>
-      <c r="T1" s="82"/>
-      <c r="U1" s="82"/>
-      <c r="V1" s="82"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="77"/>
+      <c r="V1" s="77"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="82" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="84"/>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
-      <c r="N2" s="84"/>
-      <c r="O2" s="84"/>
-      <c r="P2" s="84"/>
-      <c r="Q2" s="84"/>
-      <c r="R2" s="84"/>
-      <c r="S2" s="84"/>
-      <c r="T2" s="84"/>
-      <c r="U2" s="84"/>
-      <c r="V2" s="84"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="82"/>
+      <c r="M2" s="82"/>
+      <c r="N2" s="82"/>
+      <c r="O2" s="82"/>
+      <c r="P2" s="82"/>
+      <c r="Q2" s="82"/>
+      <c r="R2" s="82"/>
+      <c r="S2" s="82"/>
+      <c r="T2" s="82"/>
+      <c r="U2" s="82"/>
+      <c r="V2" s="82"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -3281,7 +3281,7 @@
         <v>25</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>67</v>
@@ -3781,7 +3781,7 @@
         <v>100</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C24" s="14" t="s">
         <v>67</v>
@@ -4376,7 +4376,7 @@
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B5:B40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Construction,Completed,Planning,On Hold"</formula1>
     </dataValidation>
@@ -4417,20 +4417,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="77" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="82" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4908,22 +4908,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="77" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="82" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5843,15 +5843,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -6104,6 +6095,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6118,14 +6118,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6144,6 +6136,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-08-07 14:21)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76A77EEA-30F4-4EB8-91CD-2D3EA821E969}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7B36C9-D88C-4634-9068-32A66562C287}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -440,9 +440,6 @@
     <t>https://corallife806.sharepoint.com/:b:/s/CoralLife2/IQB85P7JtoSZT6532Il6VakbAcqfI6xy5EwPf0pgbRJpT3Y?e=Qwe5V0</t>
   </si>
   <si>
-    <t>ราคา Minimum ของผู้รับเหมา</t>
-  </si>
-  <si>
     <t>ทำราคาขั้นต่ำ ในกรณีงานเล็กเป็นงานเหมา</t>
   </si>
   <si>
@@ -480,6 +477,9 @@
   </si>
   <si>
     <t>เทสและวัดลม</t>
+  </si>
+  <si>
+    <t>Revise ราคาของผู้รับเหมา</t>
   </si>
 </sst>
 </file>
@@ -1067,6 +1067,8 @@
     <xf numFmtId="164" fontId="18" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1081,7 +1083,6 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="19" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1090,7 +1091,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1124,7 +1124,8 @@
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId3"/>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Schedule"/>
@@ -1476,34 +1477,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
     </row>
     <row r="4" spans="1:11" ht="28.2" thickBot="1">
       <c r="A4" s="1" t="s">
@@ -1561,14 +1562,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="73">
+      <c r="I5" s="75">
         <v>46244</v>
       </c>
       <c r="J5" s="85"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="72"/>
+      <c r="A6" s="74"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1586,12 +1587,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="74"/>
-      <c r="J6" s="76"/>
+      <c r="I6" s="76"/>
+      <c r="J6" s="78"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1">
-      <c r="A7" s="71" t="s">
+      <c r="A7" s="73" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1611,14 +1612,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="73">
+      <c r="I7" s="75">
         <v>46366</v>
       </c>
-      <c r="J7" s="75"/>
+      <c r="J7" s="77"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="72"/>
+      <c r="A8" s="74"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1636,12 +1637,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="74"/>
-      <c r="J8" s="76"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="78"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
-      <c r="A9" s="71" t="s">
+      <c r="A9" s="73" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1661,14 +1662,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="73">
+      <c r="I9" s="75">
         <v>46218</v>
       </c>
-      <c r="J9" s="75"/>
+      <c r="J9" s="77"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="72"/>
+      <c r="A10" s="74"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1686,12 +1687,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="74"/>
-      <c r="J10" s="76"/>
+      <c r="I10" s="76"/>
+      <c r="J10" s="78"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11" ht="15" thickBot="1">
-      <c r="A11" s="71" t="s">
+      <c r="A11" s="73" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1711,14 +1712,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="73">
+      <c r="I11" s="75">
         <v>46171</v>
       </c>
-      <c r="J11" s="75"/>
+      <c r="J11" s="77"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="72"/>
+      <c r="A12" s="74"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1736,12 +1737,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="74"/>
-      <c r="J12" s="76"/>
+      <c r="I12" s="76"/>
+      <c r="J12" s="78"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11" ht="15" thickBot="1">
-      <c r="A13" s="71" t="s">
+      <c r="A13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1761,14 +1762,14 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="79">
+      <c r="I13" s="80">
         <v>46419</v>
       </c>
-      <c r="J13" s="75"/>
+      <c r="J13" s="77"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="72"/>
+      <c r="A14" s="74"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1786,12 +1787,12 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="80"/>
-      <c r="J14" s="76"/>
+      <c r="I14" s="81"/>
+      <c r="J14" s="78"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11" ht="15" thickBot="1">
-      <c r="A15" s="71" t="s">
+      <c r="A15" s="73" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1811,14 +1812,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="73">
+      <c r="I15" s="75">
         <v>46199</v>
       </c>
-      <c r="J15" s="75"/>
+      <c r="J15" s="77"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="72"/>
+      <c r="A16" s="74"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1836,12 +1837,12 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="74"/>
-      <c r="J16" s="76"/>
+      <c r="I16" s="76"/>
+      <c r="J16" s="78"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1">
-      <c r="A17" s="81" t="s">
+      <c r="A17" s="82" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="32" t="s">
@@ -1861,14 +1862,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="73">
+      <c r="I17" s="75">
         <v>46305</v>
       </c>
       <c r="J17" s="84"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="72"/>
+      <c r="A18" s="74"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1886,12 +1887,12 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="74"/>
-      <c r="J18" s="76"/>
+      <c r="I18" s="76"/>
+      <c r="J18" s="78"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11" ht="15" thickBot="1">
-      <c r="A19" s="81" t="s">
+      <c r="A19" s="82" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="32" t="s">
@@ -1911,14 +1912,14 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="79">
+      <c r="I19" s="80">
         <v>46419</v>
       </c>
       <c r="J19" s="84"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="72"/>
+      <c r="A20" s="74"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1936,12 +1937,12 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="80"/>
-      <c r="J20" s="76"/>
+      <c r="I20" s="81"/>
+      <c r="J20" s="78"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1">
-      <c r="A21" s="71" t="s">
+      <c r="A21" s="73" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1961,14 +1962,14 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="79">
+      <c r="I21" s="80">
         <v>46397</v>
       </c>
-      <c r="J21" s="75"/>
+      <c r="J21" s="77"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="72"/>
+      <c r="A22" s="74"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1986,12 +1987,12 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="80"/>
-      <c r="J22" s="76"/>
+      <c r="I22" s="81"/>
+      <c r="J22" s="78"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11" ht="15" thickBot="1">
-      <c r="A23" s="71" t="s">
+      <c r="A23" s="73" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -2011,14 +2012,14 @@
       <c r="H23" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="73">
+      <c r="I23" s="75">
         <v>46237</v>
       </c>
-      <c r="J23" s="75"/>
+      <c r="J23" s="77"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="72"/>
+      <c r="A24" s="74"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -2036,12 +2037,12 @@
       <c r="H24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="74"/>
-      <c r="J24" s="76"/>
+      <c r="I24" s="76"/>
+      <c r="J24" s="78"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11" ht="15" thickBot="1">
-      <c r="A25" s="71" t="s">
+      <c r="A25" s="73" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -2061,14 +2062,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="73">
+      <c r="I25" s="75">
         <v>46188</v>
       </c>
-      <c r="J25" s="75"/>
+      <c r="J25" s="77"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="72"/>
+      <c r="A26" s="74"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2086,12 +2087,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="74"/>
-      <c r="J26" s="76"/>
+      <c r="I26" s="76"/>
+      <c r="J26" s="78"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11" ht="15" thickBot="1">
-      <c r="A27" s="71" t="s">
+      <c r="A27" s="73" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2111,14 +2112,14 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="79">
+      <c r="I27" s="80">
         <v>46382</v>
       </c>
-      <c r="J27" s="75"/>
+      <c r="J27" s="77"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="72"/>
+      <c r="A28" s="74"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2136,12 +2137,12 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="80"/>
-      <c r="J28" s="76"/>
+      <c r="I28" s="81"/>
+      <c r="J28" s="78"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11" ht="15" thickBot="1">
-      <c r="A29" s="71" t="s">
+      <c r="A29" s="73" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2161,14 +2162,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="73">
+      <c r="I29" s="75">
         <v>46139</v>
       </c>
-      <c r="J29" s="75"/>
+      <c r="J29" s="77"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="72"/>
+      <c r="A30" s="74"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2186,12 +2187,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="74"/>
-      <c r="J30" s="76"/>
+      <c r="I30" s="76"/>
+      <c r="J30" s="78"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11" ht="15" thickBot="1">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="73" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2211,14 +2212,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="73">
+      <c r="I31" s="75">
         <v>46133</v>
       </c>
-      <c r="J31" s="75"/>
+      <c r="J31" s="77"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="72"/>
+      <c r="A32" s="74"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2236,12 +2237,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="74"/>
-      <c r="J32" s="76"/>
+      <c r="I32" s="76"/>
+      <c r="J32" s="78"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11" ht="15" thickBot="1">
-      <c r="A33" s="71" t="s">
+      <c r="A33" s="73" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2261,14 +2262,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="73">
+      <c r="I33" s="75">
         <v>46342</v>
       </c>
-      <c r="J33" s="75"/>
+      <c r="J33" s="77"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="72"/>
+      <c r="A34" s="74"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2286,12 +2287,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="74"/>
-      <c r="J34" s="76"/>
+      <c r="I34" s="76"/>
+      <c r="J34" s="78"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11" ht="15" thickBot="1">
-      <c r="A35" s="71" t="s">
+      <c r="A35" s="73" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2311,14 +2312,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="73">
+      <c r="I35" s="75">
         <v>46264</v>
       </c>
-      <c r="J35" s="75"/>
+      <c r="J35" s="77"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="72"/>
+      <c r="A36" s="74"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2336,12 +2337,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="74"/>
-      <c r="J36" s="76"/>
+      <c r="I36" s="76"/>
+      <c r="J36" s="78"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11" ht="15" thickBot="1">
-      <c r="A37" s="71" t="s">
+      <c r="A37" s="73" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2361,14 +2362,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="73">
+      <c r="I37" s="75">
         <v>46295</v>
       </c>
-      <c r="J37" s="75"/>
+      <c r="J37" s="77"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="72"/>
+      <c r="A38" s="74"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2386,12 +2387,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="74"/>
-      <c r="J38" s="76"/>
+      <c r="I38" s="76"/>
+      <c r="J38" s="78"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11" ht="15" thickBot="1">
-      <c r="A39" s="71" t="s">
+      <c r="A39" s="73" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2409,16 +2410,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="I39" s="73">
+        <v>137</v>
+      </c>
+      <c r="I39" s="75">
         <v>46539</v>
       </c>
-      <c r="J39" s="75"/>
+      <c r="J39" s="77"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="72"/>
+      <c r="A40" s="74"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2434,14 +2435,14 @@
         <v>0</v>
       </c>
       <c r="H40" s="55" t="s">
-        <v>138</v>
-      </c>
-      <c r="I40" s="74"/>
-      <c r="J40" s="76"/>
+        <v>137</v>
+      </c>
+      <c r="I40" s="76"/>
+      <c r="J40" s="78"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11" ht="15" thickBot="1">
-      <c r="A41" s="71" t="s">
+      <c r="A41" s="73" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2461,14 +2462,14 @@
       <c r="H41" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="73">
+      <c r="I41" s="75">
         <v>46237</v>
       </c>
-      <c r="J41" s="75"/>
+      <c r="J41" s="77"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="72"/>
+      <c r="A42" s="74"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2478,13 +2479,13 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="74"/>
-      <c r="J42" s="76"/>
+      <c r="I42" s="76"/>
+      <c r="J42" s="78"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11" ht="15" thickBot="1">
-      <c r="A43" s="71" t="s">
-        <v>136</v>
+      <c r="A43" s="73" t="s">
+        <v>135</v>
       </c>
       <c r="B43" s="38" t="s">
         <v>11</v>
@@ -2503,14 +2504,14 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="73">
+      <c r="I43" s="75">
         <v>46447</v>
       </c>
-      <c r="J43" s="75"/>
+      <c r="J43" s="77"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="72"/>
+      <c r="A44" s="74"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2528,8 +2529,8 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="74"/>
-      <c r="J44" s="76"/>
+      <c r="I44" s="76"/>
+      <c r="J44" s="78"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
@@ -2633,56 +2634,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="77"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="82"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="82"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="82"/>
-      <c r="Q2" s="82"/>
-      <c r="R2" s="82"/>
-      <c r="S2" s="82"/>
-      <c r="T2" s="82"/>
-      <c r="U2" s="82"/>
-      <c r="V2" s="82"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
+      <c r="N2" s="72"/>
+      <c r="O2" s="72"/>
+      <c r="P2" s="72"/>
+      <c r="Q2" s="72"/>
+      <c r="R2" s="72"/>
+      <c r="S2" s="72"/>
+      <c r="T2" s="72"/>
+      <c r="U2" s="72"/>
+      <c r="V2" s="72"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -3646,7 +3647,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P20" s="10">
         <v>228548</v>
@@ -3690,7 +3691,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P21" s="10">
         <v>224227</v>
@@ -3826,7 +3827,7 @@
         <v>46234</v>
       </c>
       <c r="T24" s="26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="U24" s="31" t="s">
         <v>129</v>
@@ -3837,7 +3838,7 @@
     </row>
     <row r="25" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
       <c r="A25" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>22</v>
@@ -3874,7 +3875,7 @@
         <v>384843</v>
       </c>
       <c r="T25" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="V25" s="19"/>
     </row>
@@ -4417,20 +4418,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="82"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4798,7 +4799,7 @@
         <v>3</v>
       </c>
       <c r="E26" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4815,7 +4816,7 @@
         <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -4832,7 +4833,7 @@
         <v>4</v>
       </c>
       <c r="E28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -4840,7 +4841,7 @@
         <v>46227</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C29" s="63" t="s">
         <v>61</v>
@@ -4866,7 +4867,7 @@
         <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -4883,7 +4884,7 @@
         <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -4908,22 +4909,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="82"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4956,7 +4957,7 @@
         <v>46224</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4990,15 +4991,15 @@
         <v>46224</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="C8" s="6">
         <v>46226</v>
@@ -5012,7 +5013,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="6">
@@ -5843,6 +5844,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -6095,29 +6118,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CD2A335-1DEC-4C21-977A-9ED57024A196}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6134,23 +6154,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-08-07 15:23)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7B36C9-D88C-4634-9068-32A66562C287}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{0CEBE545-894A-44A9-891E-5BB094C4C614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3495988F-557D-44E5-B304-C6059BF4A29C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2010,7 +2010,7 @@
         <v>1</v>
       </c>
       <c r="H23" s="41" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I23" s="75">
         <v>46237</v>
@@ -2035,7 +2035,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="44" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I24" s="76"/>
       <c r="J24" s="78"/>
@@ -2460,7 +2460,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I41" s="75">
         <v>46237</v>
@@ -2611,6 +2611,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V189"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
@@ -2869,7 +2870,7 @@
       <c r="U6" s="25"/>
       <c r="V6" s="19"/>
     </row>
-    <row r="7" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="7" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A7" s="14" t="s">
         <v>17</v>
       </c>
@@ -2929,7 +2930,7 @@
       </c>
       <c r="V7" s="19"/>
     </row>
-    <row r="8" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="8" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A8" s="14" t="s">
         <v>18</v>
       </c>
@@ -3039,7 +3040,7 @@
       <c r="U9" s="25"/>
       <c r="V9" s="19"/>
     </row>
-    <row r="10" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="10" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A10" s="9" t="s">
         <v>20</v>
       </c>
@@ -3277,7 +3278,7 @@
         <v>46147</v>
       </c>
     </row>
-    <row r="14" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="14" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A14" s="9" t="s">
         <v>25</v>
       </c>
@@ -3337,7 +3338,7 @@
         <v>46169</v>
       </c>
     </row>
-    <row r="15" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="15" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A15" s="9" t="s">
         <v>26</v>
       </c>
@@ -3450,7 +3451,7 @@
         <v>46182</v>
       </c>
     </row>
-    <row r="17" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="17" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A17" s="9" t="s">
         <v>28</v>
       </c>
@@ -3505,7 +3506,7 @@
         <v>46079</v>
       </c>
     </row>
-    <row r="18" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="18" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A18" s="9" t="s">
         <v>29</v>
       </c>
@@ -3567,7 +3568,7 @@
         <v>67</v>
       </c>
       <c r="D19" s="15">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E19" s="16">
         <v>832813</v>
@@ -3707,7 +3708,7 @@
       </c>
       <c r="V21" s="19"/>
     </row>
-    <row r="22" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="22" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A22" s="9" t="s">
         <v>87</v>
       </c>
@@ -3777,7 +3778,7 @@
         <v>46209</v>
       </c>
     </row>
-    <row r="24" spans="1:22" s="9" customFormat="1" ht="18.600000000000001">
+    <row r="24" spans="1:22" s="9" customFormat="1" ht="18.600000000000001" hidden="1">
       <c r="A24" s="9" t="s">
         <v>100</v>
       </c>
@@ -4372,7 +4373,14 @@
       <c r="V189" s="19"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:V189" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A4:V189" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="1">
+      <filters blank="1">
+        <filter val="Construction"/>
+        <filter val="On Hold"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:V2"/>

</xml_diff>

<commit_message>
Update dashboard/data (2026-08-07 17:45)
</commit_message>
<xml_diff>
--- a/Construction_Portfolio_Template.xlsx
+++ b/Construction_Portfolio_Template.xlsx
@@ -1067,8 +1067,18 @@
     <xf numFmtId="164" fontId="18" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1077,13 +1087,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="19" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1091,14 +1094,11 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1477,34 +1477,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="83"/>
+      <c r="J2" s="83"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="4" spans="1:11" ht="28.2" thickBot="1">
       <c r="A4" s="1" t="s">
@@ -1542,7 +1542,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" thickBot="1">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="85" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="58" t="s">
@@ -1562,14 +1562,14 @@
       <c r="H5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="75">
+      <c r="I5" s="77">
         <v>46244</v>
       </c>
-      <c r="J5" s="85"/>
+      <c r="J5" s="73"/>
       <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="74"/>
+      <c r="A6" s="76"/>
       <c r="B6" s="44" t="s">
         <v>13</v>
       </c>
@@ -1587,12 +1587,12 @@
       <c r="H6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="76"/>
-      <c r="J6" s="78"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="72"/>
       <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="75" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="38" t="s">
@@ -1612,14 +1612,14 @@
       <c r="H7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="75">
+      <c r="I7" s="77">
         <v>46366</v>
       </c>
-      <c r="J7" s="77"/>
+      <c r="J7" s="71"/>
       <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="A8" s="74"/>
+      <c r="A8" s="76"/>
       <c r="B8" s="35" t="s">
         <v>13</v>
       </c>
@@ -1637,12 +1637,12 @@
       <c r="H8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="76"/>
-      <c r="J8" s="78"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="72"/>
       <c r="K8" s="48"/>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
-      <c r="A9" s="73" t="s">
+      <c r="A9" s="75" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="38" t="s">
@@ -1662,14 +1662,14 @@
       <c r="H9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="75">
+      <c r="I9" s="77">
         <v>46218</v>
       </c>
-      <c r="J9" s="77"/>
+      <c r="J9" s="71"/>
       <c r="K9" s="49"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
-      <c r="A10" s="74"/>
+      <c r="A10" s="76"/>
       <c r="B10" s="35" t="s">
         <v>13</v>
       </c>
@@ -1687,12 +1687,12 @@
       <c r="H10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="76"/>
-      <c r="J10" s="78"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="72"/>
       <c r="K10" s="48"/>
     </row>
     <row r="11" spans="1:11" ht="15" thickBot="1">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="75" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="41" t="s">
@@ -1712,14 +1712,14 @@
       <c r="H11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="75">
+      <c r="I11" s="77">
         <v>46171</v>
       </c>
-      <c r="J11" s="77"/>
+      <c r="J11" s="71"/>
       <c r="K11" s="49"/>
     </row>
     <row r="12" spans="1:11" ht="15" thickBot="1">
-      <c r="A12" s="74"/>
+      <c r="A12" s="76"/>
       <c r="B12" s="44" t="s">
         <v>13</v>
       </c>
@@ -1737,12 +1737,12 @@
       <c r="H12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="76"/>
-      <c r="J12" s="78"/>
+      <c r="I12" s="78"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="48"/>
     </row>
     <row r="13" spans="1:11" ht="15" thickBot="1">
-      <c r="A13" s="73" t="s">
+      <c r="A13" s="75" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="38" t="s">
@@ -1762,14 +1762,14 @@
       <c r="H13" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="80">
+      <c r="I13" s="79">
         <v>46419</v>
       </c>
-      <c r="J13" s="77"/>
+      <c r="J13" s="71"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1">
-      <c r="A14" s="74"/>
+      <c r="A14" s="76"/>
       <c r="B14" s="35" t="s">
         <v>13</v>
       </c>
@@ -1787,12 +1787,12 @@
       <c r="H14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="81"/>
-      <c r="J14" s="78"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="72"/>
       <c r="K14" s="48"/>
     </row>
     <row r="15" spans="1:11" ht="15" thickBot="1">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="75" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="41" t="s">
@@ -1812,14 +1812,14 @@
       <c r="H15" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="75">
+      <c r="I15" s="77">
         <v>46199</v>
       </c>
-      <c r="J15" s="77"/>
+      <c r="J15" s="71"/>
       <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
-      <c r="A16" s="74"/>
+      <c r="A16" s="76"/>
       <c r="B16" s="44" t="s">
         <v>13</v>
       </c>
@@ -1837,12 +1837,12 @@
       <c r="H16" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="76"/>
-      <c r="J16" s="78"/>
+      <c r="I16" s="78"/>
+      <c r="J16" s="72"/>
       <c r="K16" s="48"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1">
-      <c r="A17" s="82" t="s">
+      <c r="A17" s="81" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="32" t="s">
@@ -1862,14 +1862,14 @@
       <c r="H17" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="75">
+      <c r="I17" s="77">
         <v>46305</v>
       </c>
-      <c r="J17" s="84"/>
+      <c r="J17" s="74"/>
       <c r="K17" s="50"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
-      <c r="A18" s="74"/>
+      <c r="A18" s="76"/>
       <c r="B18" s="35" t="s">
         <v>13</v>
       </c>
@@ -1887,12 +1887,12 @@
       <c r="H18" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="76"/>
-      <c r="J18" s="78"/>
+      <c r="I18" s="78"/>
+      <c r="J18" s="72"/>
       <c r="K18" s="48"/>
     </row>
     <row r="19" spans="1:11" ht="15" thickBot="1">
-      <c r="A19" s="82" t="s">
+      <c r="A19" s="81" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="32" t="s">
@@ -1912,14 +1912,14 @@
       <c r="H19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="80">
+      <c r="I19" s="79">
         <v>46419</v>
       </c>
-      <c r="J19" s="84"/>
+      <c r="J19" s="74"/>
       <c r="K19" s="50"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
-      <c r="A20" s="74"/>
+      <c r="A20" s="76"/>
       <c r="B20" s="35" t="s">
         <v>13</v>
       </c>
@@ -1937,12 +1937,12 @@
       <c r="H20" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="81"/>
-      <c r="J20" s="78"/>
+      <c r="I20" s="80"/>
+      <c r="J20" s="72"/>
       <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1">
-      <c r="A21" s="73" t="s">
+      <c r="A21" s="75" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1962,14 +1962,14 @@
       <c r="H21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="80">
+      <c r="I21" s="79">
         <v>46397</v>
       </c>
-      <c r="J21" s="77"/>
+      <c r="J21" s="71"/>
       <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
-      <c r="A22" s="74"/>
+      <c r="A22" s="76"/>
       <c r="B22" s="35" t="s">
         <v>13</v>
       </c>
@@ -1987,12 +1987,12 @@
       <c r="H22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="81"/>
-      <c r="J22" s="78"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="72"/>
       <c r="K22" s="52"/>
     </row>
     <row r="23" spans="1:11" ht="15" thickBot="1">
-      <c r="A23" s="73" t="s">
+      <c r="A23" s="75" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="41" t="s">
@@ -2012,14 +2012,14 @@
       <c r="H23" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I23" s="75">
+      <c r="I23" s="77">
         <v>46237</v>
       </c>
-      <c r="J23" s="77"/>
+      <c r="J23" s="71"/>
       <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="74"/>
+      <c r="A24" s="76"/>
       <c r="B24" s="44" t="s">
         <v>13</v>
       </c>
@@ -2037,12 +2037,12 @@
       <c r="H24" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I24" s="76"/>
-      <c r="J24" s="78"/>
+      <c r="I24" s="78"/>
+      <c r="J24" s="72"/>
       <c r="K24" s="52"/>
     </row>
     <row r="25" spans="1:11" ht="15" thickBot="1">
-      <c r="A25" s="73" t="s">
+      <c r="A25" s="75" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="41" t="s">
@@ -2062,14 +2062,14 @@
       <c r="H25" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="75">
+      <c r="I25" s="77">
         <v>46188</v>
       </c>
-      <c r="J25" s="77"/>
+      <c r="J25" s="71"/>
       <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
-      <c r="A26" s="74"/>
+      <c r="A26" s="76"/>
       <c r="B26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2087,12 +2087,12 @@
       <c r="H26" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="76"/>
-      <c r="J26" s="78"/>
+      <c r="I26" s="78"/>
+      <c r="J26" s="72"/>
       <c r="K26" s="52"/>
     </row>
     <row r="27" spans="1:11" ht="15" thickBot="1">
-      <c r="A27" s="73" t="s">
+      <c r="A27" s="75" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="38" t="s">
@@ -2112,14 +2112,14 @@
       <c r="H27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="80">
+      <c r="I27" s="79">
         <v>46382</v>
       </c>
-      <c r="J27" s="77"/>
+      <c r="J27" s="71"/>
       <c r="K27" s="51"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1">
-      <c r="A28" s="74"/>
+      <c r="A28" s="76"/>
       <c r="B28" s="35" t="s">
         <v>13</v>
       </c>
@@ -2137,12 +2137,12 @@
       <c r="H28" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="81"/>
-      <c r="J28" s="78"/>
+      <c r="I28" s="80"/>
+      <c r="J28" s="72"/>
       <c r="K28" s="52"/>
     </row>
     <row r="29" spans="1:11" ht="15" thickBot="1">
-      <c r="A29" s="73" t="s">
+      <c r="A29" s="75" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="41" t="s">
@@ -2162,14 +2162,14 @@
       <c r="H29" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="75">
+      <c r="I29" s="77">
         <v>46139</v>
       </c>
-      <c r="J29" s="77"/>
+      <c r="J29" s="71"/>
       <c r="K29" s="51"/>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
-      <c r="A30" s="74"/>
+      <c r="A30" s="76"/>
       <c r="B30" s="44" t="s">
         <v>13</v>
       </c>
@@ -2187,12 +2187,12 @@
       <c r="H30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="76"/>
-      <c r="J30" s="78"/>
+      <c r="I30" s="78"/>
+      <c r="J30" s="72"/>
       <c r="K30" s="52"/>
     </row>
     <row r="31" spans="1:11" ht="15" thickBot="1">
-      <c r="A31" s="73" t="s">
+      <c r="A31" s="75" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="41" t="s">
@@ -2212,14 +2212,14 @@
       <c r="H31" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I31" s="75">
+      <c r="I31" s="77">
         <v>46133</v>
       </c>
-      <c r="J31" s="77"/>
+      <c r="J31" s="71"/>
       <c r="K31" s="51"/>
     </row>
     <row r="32" spans="1:11" ht="15" thickBot="1">
-      <c r="A32" s="74"/>
+      <c r="A32" s="76"/>
       <c r="B32" s="44" t="s">
         <v>13</v>
       </c>
@@ -2237,12 +2237,12 @@
       <c r="H32" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="I32" s="76"/>
-      <c r="J32" s="78"/>
+      <c r="I32" s="78"/>
+      <c r="J32" s="72"/>
       <c r="K32" s="52"/>
     </row>
     <row r="33" spans="1:11" ht="15" thickBot="1">
-      <c r="A33" s="73" t="s">
+      <c r="A33" s="75" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="38" t="s">
@@ -2262,14 +2262,14 @@
       <c r="H33" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="75">
+      <c r="I33" s="77">
         <v>46342</v>
       </c>
-      <c r="J33" s="77"/>
+      <c r="J33" s="71"/>
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
-      <c r="A34" s="74"/>
+      <c r="A34" s="76"/>
       <c r="B34" s="35" t="s">
         <v>13</v>
       </c>
@@ -2287,12 +2287,12 @@
       <c r="H34" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I34" s="76"/>
-      <c r="J34" s="78"/>
+      <c r="I34" s="78"/>
+      <c r="J34" s="72"/>
       <c r="K34" s="52"/>
     </row>
     <row r="35" spans="1:11" ht="15" thickBot="1">
-      <c r="A35" s="73" t="s">
+      <c r="A35" s="75" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="38" t="s">
@@ -2312,14 +2312,14 @@
       <c r="H35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="75">
+      <c r="I35" s="77">
         <v>46264</v>
       </c>
-      <c r="J35" s="77"/>
+      <c r="J35" s="71"/>
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="1:11" ht="15" thickBot="1">
-      <c r="A36" s="74"/>
+      <c r="A36" s="76"/>
       <c r="B36" s="35" t="s">
         <v>13</v>
       </c>
@@ -2337,12 +2337,12 @@
       <c r="H36" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="76"/>
-      <c r="J36" s="78"/>
+      <c r="I36" s="78"/>
+      <c r="J36" s="72"/>
       <c r="K36" s="52"/>
     </row>
     <row r="37" spans="1:11" ht="15" thickBot="1">
-      <c r="A37" s="73" t="s">
+      <c r="A37" s="75" t="s">
         <v>32</v>
       </c>
       <c r="B37" s="38" t="s">
@@ -2362,14 +2362,14 @@
       <c r="H37" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="75">
+      <c r="I37" s="77">
         <v>46295</v>
       </c>
-      <c r="J37" s="77"/>
+      <c r="J37" s="71"/>
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1">
-      <c r="A38" s="74"/>
+      <c r="A38" s="76"/>
       <c r="B38" s="35" t="s">
         <v>13</v>
       </c>
@@ -2387,12 +2387,12 @@
       <c r="H38" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="76"/>
-      <c r="J38" s="78"/>
+      <c r="I38" s="78"/>
+      <c r="J38" s="72"/>
       <c r="K38" s="52"/>
     </row>
     <row r="39" spans="1:11" ht="15" thickBot="1">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="75" t="s">
         <v>91</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -2412,14 +2412,14 @@
       <c r="H39" s="38" t="s">
         <v>137</v>
       </c>
-      <c r="I39" s="75">
+      <c r="I39" s="77">
         <v>46539</v>
       </c>
-      <c r="J39" s="77"/>
+      <c r="J39" s="71"/>
       <c r="K39" s="51"/>
     </row>
     <row r="40" spans="1:11" ht="15" thickBot="1">
-      <c r="A40" s="74"/>
+      <c r="A40" s="76"/>
       <c r="B40" s="55" t="s">
         <v>13</v>
       </c>
@@ -2437,12 +2437,12 @@
       <c r="H40" s="55" t="s">
         <v>137</v>
       </c>
-      <c r="I40" s="76"/>
-      <c r="J40" s="78"/>
+      <c r="I40" s="78"/>
+      <c r="J40" s="72"/>
       <c r="K40" s="52"/>
     </row>
     <row r="41" spans="1:11" ht="15" thickBot="1">
-      <c r="A41" s="73" t="s">
+      <c r="A41" s="75" t="s">
         <v>100</v>
       </c>
       <c r="B41" s="38" t="s">
@@ -2462,14 +2462,14 @@
       <c r="H41" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I41" s="75">
+      <c r="I41" s="77">
         <v>46237</v>
       </c>
-      <c r="J41" s="77"/>
+      <c r="J41" s="71"/>
       <c r="K41" s="51"/>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1">
-      <c r="A42" s="74"/>
+      <c r="A42" s="76"/>
       <c r="B42" s="55" t="s">
         <v>13</v>
       </c>
@@ -2479,12 +2479,12 @@
       <c r="F42" s="56"/>
       <c r="G42" s="57"/>
       <c r="H42" s="55"/>
-      <c r="I42" s="76"/>
-      <c r="J42" s="78"/>
+      <c r="I42" s="78"/>
+      <c r="J42" s="72"/>
       <c r="K42" s="52"/>
     </row>
     <row r="43" spans="1:11" ht="15" thickBot="1">
-      <c r="A43" s="73" t="s">
+      <c r="A43" s="75" t="s">
         <v>135</v>
       </c>
       <c r="B43" s="38" t="s">
@@ -2504,14 +2504,14 @@
       <c r="H43" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="I43" s="75">
+      <c r="I43" s="77">
         <v>46447</v>
       </c>
-      <c r="J43" s="77"/>
+      <c r="J43" s="71"/>
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickBot="1">
-      <c r="A44" s="74"/>
+      <c r="A44" s="76"/>
       <c r="B44" s="55" t="s">
         <v>13</v>
       </c>
@@ -2529,27 +2529,45 @@
       <c r="H44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I44" s="76"/>
-      <c r="J44" s="78"/>
+      <c r="I44" s="78"/>
+      <c r="J44" s="72"/>
       <c r="K44" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:K44" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="62">
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="J19:J20"/>
@@ -2566,38 +2584,20 @@
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="I29:I30"/>
     <mergeCell ref="A33:A34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="J35:J36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H5:H48" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2635,56 +2635,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="82" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="82"/>
+      <c r="S1" s="82"/>
+      <c r="T1" s="82"/>
+      <c r="U1" s="82"/>
+      <c r="V1" s="82"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="72"/>
-      <c r="P2" s="72"/>
-      <c r="Q2" s="72"/>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="84"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
+      <c r="N2" s="84"/>
+      <c r="O2" s="84"/>
+      <c r="P2" s="84"/>
+      <c r="Q2" s="84"/>
+      <c r="R2" s="84"/>
+      <c r="S2" s="84"/>
+      <c r="T2" s="84"/>
+      <c r="U2" s="84"/>
+      <c r="V2" s="84"/>
     </row>
     <row r="4" spans="1:22" ht="41.4">
       <c r="A4" s="1" t="s">
@@ -4426,20 +4426,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="82" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="84" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4917,22 +4917,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="82" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="84" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -5852,15 +5852,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -5871,6 +5862,15 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6127,20 +6127,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B14C1EB-02DF-450B-8928-EA02D20EAB49}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235994A7-6E6B-494E-A465-C3E876960F00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>